<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 1)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -742,8 +742,664 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1174748969</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>HDSelectShop</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>[NEW] [新商品] ドクダミポアディープクレンジングフォーム 150ml (2個)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>4431</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="b">
+        <v>0</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174748969</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1171434085</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>HDSelectShop</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>PDRNヒアルロン酸100モイスチャライジングクリーム 60ml (2個) + PDRN ヒアルロン酸カプセル 100セラム 30ml</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>12801</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="b">
+        <v>0</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171434085</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1180595613</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>HDSelectShop</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>PDRN 100ヒアルロン酸 ブースター トナー 250ml + PDRNヒアルロン酸100モイスチャライジングクリーム 60ml + PDRN ヒアルロン酸カプセル 100セラム 30ml</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>11931</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" t="b">
+        <v>0</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180595613</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1151371296</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>HDSelectShop</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>アトバリア365 ハイドロエッセンス 200ml (2個)</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>8763</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" t="b">
+        <v>0</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1151371296</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>1127146298</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>HDSelectShop</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>5番 マスクパック (10枚) / 白玉グルタチオンＣふりかけマスク</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>4695</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" t="b">
+        <v>0</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1127146298</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1194303928</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>blanc-lapin</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>ジョーマローン JO MALONE ピオニー &amp;amp; ブラッシュ スエード ハンド クリーム 30ml ハンドケア [159109]【メール便可】</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Peony</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>3820</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="b">
+        <v>0</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194303928</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1176803786</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>blanc-lapin</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>ベルバイ BELLE BAI ベルナンバー5 オードパルファン / ヴァーダント ヒア 50ml フレグランス 香水 ユニセックス 男性用 女性用 [530095]</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>BELLE BAI</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>3300</v>
+      </c>
+      <c r="G14" t="n">
+        <v>2</v>
+      </c>
+      <c r="H14" t="b">
+        <v>0</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1176803786</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>1207120487</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ALife07</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>モイスチャー レイヤー サンプロテクション SPF50+ PA++++ 50ml</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>3650</v>
+      </c>
+      <c r="G15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" t="b">
+        <v>0</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207120487</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>1195110594</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ALife07</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>ビタC プラス スポット コレクティング＆ファーミング アンプル 40ml 2個</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>ミシャ</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>3965</v>
+      </c>
+      <c r="G16" t="n">
+        <v>2</v>
+      </c>
+      <c r="H16" t="b">
+        <v>0</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195110594</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>1203232874</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>zozoro0213</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>[洗顔パフプレゼント] ヤマノイモクレンジング吸着パックフォーム 120ml</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>ハンユル</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>2280</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="b">
+        <v>0</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203232874</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>1210182731</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>zozoro0213</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>ナチュラル オールインワン カバー ローション 50g</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>オブジェ</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>4275</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="b">
+        <v>0</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210182731</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>1193372038</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>kpink77</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>【1+1】【韓国コスメ】ショッキングビタミン ミルクトーンアップ デイクリーム, 55g 2個 /(保湿/弾力/輝き/鎮静/トーンアップクリーム)</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>ラベルヤング</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>3604</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="b">
+        <v>0</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193372038</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>1210528997</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>kpink77</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>【1+1セット】クリーンティーツリーリポソーム カーミングマスク 5枚入×2個 ヒアルロン酸 パンテノール 水分 鎮静 保湿 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>3069</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="b">
+        <v>0</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210528997</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>1210272622</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>kpink77</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>【1+1セット】ウォータフルエッセンスサンクリーム SPF50+ PA++++ 50ml×2個 保湿 UVケア エッセンス 日焼け止め 化粧下地 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>6442</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="b">
+        <v>0</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210272622</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>1206508858</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>kpink77</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>【1+1セット】ソフトリセット グリーンクレンジングバーム 100ml 2個 メイク落とし 保湿洗顔 角質ケア 毛穴汚れケア 韓国コスメ しっとりディープクレンジング</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>ヒュッゲ</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>6279</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="b">
+        <v>0</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206508858</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>1206240655</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>kpink77</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>ウォーターtoアンプルトリートメント 200ml 1個 毛髪保湿 ツヤ髪ケア しっとりヘアケア ホームケア 韓国コスメ 上品な香り デイリーケア</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>サミュ</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>6459</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="b">
+        <v>0</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206240655</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J7"/>
+  <autoFilter ref="A1:J23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 3, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$35</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1398,8 +1398,500 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>1205550323</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>dgrm</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>リジュラン ダーマ ヒーラー ポア タイトニング トナー パッド 220mL</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>3960</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="b">
+        <v>0</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205550323</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>1158425809</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>dgrm</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>グリーンディープポアクレンジングバーム 100g</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>ドクタージー</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G25" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" t="b">
+        <v>0</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1158425809</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>1177829431</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>dgrm</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>マイファーストセラム 50ml</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>De:maf</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>2430</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="b">
+        <v>0</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1177829431</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>1109209881</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>korkorshop</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>[NEW]ヒストラップイージーエフコンプレックスアンプル63％80ml / EGF</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>HISTOLAB</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>9737</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="b">
+        <v>0</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1109209881</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>1212903876</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>AVECPUBLIC</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>マデカクリームシーズン7タイムリバース, 50ml, 2個</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>センテリアン24</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>3340</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" t="b">
+        <v>0</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212903876</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>1212902580</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>AVECPUBLIC</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>アドバンスドナイトリペアシンクロナイズドマルチリカバリーコンプレックス, 100ml</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>エスティローダー</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>9000</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" t="b">
+        <v>0</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212902580</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>1193369860</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>korikori</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>新作 ティーツリーオイルロールオン 5ml ニキビ 鎮静</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>ブランネイチャー</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>2642</v>
+      </c>
+      <c r="G30" t="n">
+        <v>1</v>
+      </c>
+      <c r="H30" t="b">
+        <v>0</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193369860</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>1206535075</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>korikori</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>[NEW] 9倍高濃縮 ドクダミトナーパッド 70枚 毛穴ケア 鎮静ケア</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>ブランネイチャー</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>4870</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" t="b">
+        <v>0</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206535075</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>1182701536</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>korikori</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>トリデン BEST マスクパック 30枚セット（水分＋シカ＋ビタミン） 保湿シートマスクマルチケアマスク</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>トリデン</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>6959</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" t="b">
+        <v>0</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1182701536</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>1209977461</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>mijincosme</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>夏美祭 MJケア シートマスク 【60枚】 SALE 選べるセット(6種X各10枚) 組合せ自由 - プラス1枚付き - 保湿 セット 個包装 韓国パック 大容量 シートパック フェイスパック</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>MIJIN COSMETICS</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>2700</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" t="b">
+        <v>0</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209977461</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>1194316158</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>mijin-cosme</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>メール便 無料 - アクロパス ニードルパッチ 目元 ほうれい線 レチアールエヌ スリム パッチ 3box - PDRN × レチノール配合 - 部分集中ケア - 正規品</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>ACROPASS</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>8700</v>
+      </c>
+      <c r="G34" t="n">
+        <v>1</v>
+      </c>
+      <c r="H34" t="b">
+        <v>0</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194316158</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>1212657160</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>kacos</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>レッドトマト ジェリーリップマスク / グリーントマト スムージーリップスクラブ 12g</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>FULLY</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" t="b">
+        <v>0</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212657160</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J23"/>
+  <autoFilter ref="A1:J35"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 6, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$52</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J35"/>
+  <dimension ref="A1:J52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1890,8 +1890,705 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>1193630936</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>KTOPMARKET</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>ガラク ナイアシン 3.0 エッセンス 60ml</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>3150</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" t="b">
+        <v>0</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193630936</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>1175324790</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>transia</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>センシティブ スージング ジェルクリーム 100g ひんやりうるおい 低刺激 水分クリーム ベタつきにくい 敏感肌 朝夜兼用 オイルフリー ノンコメド印象 軽い使用感</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Mary&amp;amp;May</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>2760</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" t="b">
+        <v>0</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1175324790</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>1201200397</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>transia</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>アクネブレミッシュ鎮静ボディウォッシュ 460ml 背中ニキビ・肌トラブルを改善する 背中ニキビ・ボディのざらつきケア さっぱり洗浄 つっぱりにくい デイリー用</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Nodor</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>3970</v>
+      </c>
+      <c r="G38" t="n">
+        <v>3</v>
+      </c>
+      <c r="H38" t="b">
+        <v>0</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201200397</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>1205730042</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>biniyosul</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>ダーマヒーラー ポアタイトニング トナーパッド 220ml</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>3990</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" t="b">
+        <v>0</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205730042</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>1168692108</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>210506</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>【正規品】松の木 鎮静 シカ クレンザー 150ml</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>3290</v>
+      </c>
+      <c r="G40" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" t="b">
+        <v>0</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168692108</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>1164469069</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>210506</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>【正規品】グリーンシカ コラーゲン クリアフォーム 2.0 300ml</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>3690</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" t="b">
+        <v>0</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1164469069</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>1163729695</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>210506</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>【正規品】ディープポア クレンジング ソーダフォーム 150ml</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>3590</v>
+      </c>
+      <c r="G42" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" t="b">
+        <v>0</v>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1163729695</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>1206937740</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>210506</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>【正規品】ティアミドール ブースターセラム 30ml</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>ユーセリン</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>6990</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" t="b">
+        <v>0</v>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206937740</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>1205554253</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>210506</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>【正規品】トラネキサム酸スキンブースタークリーム 100ml</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>メディテラピー</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>4990</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" t="b">
+        <v>0</v>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205554253</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>1205580942</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>nicewind</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>3番 ボドルボドル毛穴結セラム 30ml</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>2561</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" t="b">
+        <v>0</v>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205580942</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>1203332451</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>nicewind</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>ズーム バイ メイクアップ フィクサー 50ml 1+1</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>ZOOM BY JUNG SAEM MOOL</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>1876</v>
+      </c>
+      <c r="G46" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" t="b">
+        <v>0</v>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203332451</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>1205081404</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>nicewind</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>[CU ビタミンU] アンプルトナー 130ml 1+1（皮膚科から始まったメディカルスキンケア）</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>CUSKIN</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>11119</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" t="b">
+        <v>0</v>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205081404</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>1208146662</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>nicewind</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>アクネプロジェル30ml ニキビ肌の緩和機能性鎮静効果</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>東亜製薬</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>4168</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" t="b">
+        <v>0</v>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208146662</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>1211372508</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>nicewind</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>[NEW]c-PDRNブースターショットジェルマスク 5枚 1個</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>4314</v>
+      </c>
+      <c r="G49" t="n">
+        <v>1</v>
+      </c>
+      <c r="H49" t="b">
+        <v>0</v>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211372508</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>1158907027</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Butler_lounge</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>【ハリ＆リフティングケア】ナンバーズイン 9番 NMN BIO リフティング フルフェイスパック 4枚入り＋引き締めシート付き</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>2470</v>
+      </c>
+      <c r="G50" t="n">
+        <v>1</v>
+      </c>
+      <c r="H50" t="b">
+        <v>0</v>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1158907027</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>1178361427</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>furimakei</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>ZARA MAN 香水 TOBACCO COLLECTION RICH WARM ADDICTIVE 100ML オードトワレ</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>ザラ</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>7263</v>
+      </c>
+      <c r="G51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H51" t="b">
+        <v>0</v>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1178361427</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>1178361387</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>furimakei</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>ディスカバリーセット（5MLX2） アナザー13 + サンタル33</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LE LABO</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>9588</v>
+      </c>
+      <c r="G52" t="n">
+        <v>0</v>
+      </c>
+      <c r="H52" t="b">
+        <v>0</v>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1178361387</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J35"/>
+  <autoFilter ref="A1:J52"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 9, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$73</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J52"/>
+  <dimension ref="A1:J73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2587,8 +2587,869 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>1175756083</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>20240208</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>セレブ愛用 オートイン カーミング クリーム 100ml しっとり鎮静ジェル 保湿 敏感肌 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Purito</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>2384</v>
+      </c>
+      <c r="G53" t="n">
+        <v>0</v>
+      </c>
+      <c r="H53" t="b">
+        <v>0</v>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1175756083</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>1172113145</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>20240208</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>ヘリ愛用！ 緑豆 クレンジングオイル 選べる200ml/50ml 黒ずみオフ オリヤン 即日発送</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>ビープレーン</t>
+        </is>
+      </c>
+      <c r="F54" t="n">
+        <v>2809</v>
+      </c>
+      <c r="G54" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" t="b">
+        <v>0</v>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172113145</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>1212617523</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>ITRADE</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>アトバリア365クリーム30mL×3個 + ダーマUV365バリアハイドロミネラル日焼け止め20ml x3個</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>2290</v>
+      </c>
+      <c r="G55" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" t="b">
+        <v>0</v>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212617523</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>1211535086</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>DEARHOUR</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>【選べる2点SET】PDRNゼリーセラムミスト/キャビアPDRNリアルディープマスク(4枚)/PDRNリポソームバブルブースター</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Biodance</t>
+        </is>
+      </c>
+      <c r="F56" t="n">
+        <v>3650</v>
+      </c>
+      <c r="G56" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" t="b">
+        <v>0</v>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211535086</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>1073637416</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>DEARHOUR</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>バイタル ハイドラ ソリューション ハイドロプランプ ウォータークリーム 50ml 1EA</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Dr.Jart+</t>
+        </is>
+      </c>
+      <c r="F57" t="n">
+        <v>3170</v>
+      </c>
+      <c r="G57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H57" t="b">
+        <v>0</v>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1073637416</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>1073637368</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>DEARHOUR</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>シカペア スリーペア インテンシブ S リペア マスク 75ml 1EA</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Dr.Jart+</t>
+        </is>
+      </c>
+      <c r="F58" t="n">
+        <v>3340</v>
+      </c>
+      <c r="G58" t="n">
+        <v>0</v>
+      </c>
+      <c r="H58" t="b">
+        <v>0</v>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1073637368</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>1211103356</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>iS2japan</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>ツバキディープコラーゲン弾力アンプル, 30ml</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F59" t="n">
+        <v>2160</v>
+      </c>
+      <c r="G59" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" t="b">
+        <v>0</v>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211103356</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>1192583562</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>iS2japan</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>ツバキディープコラーゲン弾力クリーム, 50ml</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F60" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G60" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" t="b">
+        <v>0</v>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192583562</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>1192583554</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>iS2japan</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>[正規品] Biodance ハイドロセラノールアンプル, 30ml</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Biodance</t>
+        </is>
+      </c>
+      <c r="F61" t="n">
+        <v>2450</v>
+      </c>
+      <c r="G61" t="n">
+        <v>0</v>
+      </c>
+      <c r="H61" t="b">
+        <v>0</v>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192583554</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>1213549964</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>CHERIBEAU</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>【SEVENTEEN ミンギュ ミニスタンディ2種付き】アノブ 選べるヘアケアセット / ヘアオイル / 洗い流さないトリートメント / シャンプー / ヘアマスク / 韓国ヘアケア</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>UNOVE</t>
+        </is>
+      </c>
+      <c r="F62" t="n">
+        <v>5170</v>
+      </c>
+      <c r="G62" t="n">
+        <v>0</v>
+      </c>
+      <c r="H62" t="b">
+        <v>0</v>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213549964</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>1206876078</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>CHERIBEAU</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>[1+1] 復活草ビフィダセラム ファーミングドロップ 50ml</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>アビブ</t>
+        </is>
+      </c>
+      <c r="F63" t="n">
+        <v>3660</v>
+      </c>
+      <c r="G63" t="n">
+        <v>0</v>
+      </c>
+      <c r="H63" t="b">
+        <v>0</v>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206876078</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>1125754461</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>museshop</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>[1+1]レッドブレミッシュクリアスージングクリーム 50ml 2個+10ml 2個/正規品</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>ドクタージー</t>
+        </is>
+      </c>
+      <c r="F64" t="n">
+        <v>3469</v>
+      </c>
+      <c r="G64" t="n">
+        <v>0</v>
+      </c>
+      <c r="H64" t="b">
+        <v>0</v>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1125754461</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>1212553298</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>museshop</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>【正規品+GIFT付き】リードルショット コラーゲンクリーム 50ml＋スティックパウチ 3個</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F65" t="n">
+        <v>3021</v>
+      </c>
+      <c r="G65" t="n">
+        <v>0</v>
+      </c>
+      <c r="H65" t="b">
+        <v>0</v>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212553298</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>1212350487</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>museshop</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>[1+1]MEDI AHAイボ取りクリーム25ml 2個&amp;nbsp; / メディオルガ稗粒腫スポットクリーム/ポツポツちびイボ</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>mediorga</t>
+        </is>
+      </c>
+      <c r="F66" t="n">
+        <v>3666</v>
+      </c>
+      <c r="G66" t="n">
+        <v>0</v>
+      </c>
+      <c r="H66" t="b">
+        <v>0</v>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212350487</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>1212350471</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>museshop</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>[1+1]メディオルガブライトニングクリーム30ml 2個/しみ取りクリーム お肌のトーンアップ</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>mediorga</t>
+        </is>
+      </c>
+      <c r="F67" t="n">
+        <v>3055</v>
+      </c>
+      <c r="G67" t="n">
+        <v>0</v>
+      </c>
+      <c r="H67" t="b">
+        <v>0</v>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212350471</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>1212350473</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>museshop</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>MEDI AHAイボ取りクリーム25ml/ メディオルガ稗粒腫スポットクリーム/ポツポツちびイボ</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>mediorga</t>
+        </is>
+      </c>
+      <c r="F68" t="n">
+        <v>2331</v>
+      </c>
+      <c r="G68" t="n">
+        <v>1</v>
+      </c>
+      <c r="H68" t="b">
+        <v>0</v>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212350473</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>1146049607</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>K-BOOBOO</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>シカペア インテンシブ スージング リペアクリーム 50ml+15ml+15ml</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Dr.Jart+</t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>2860</v>
+      </c>
+      <c r="G69" t="n">
+        <v>2</v>
+      </c>
+      <c r="H69" t="b">
+        <v>0</v>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1146049607</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>1201944372</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>jp-mong</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>ライスブライトニング酵素洗顔パウダー, 40g / 韓国 人気 乾燥肌 敏感肌 米ぬか酵素洗顔クレンジング</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F70" t="n">
+        <v>3741</v>
+      </c>
+      <c r="G70" t="n">
+        <v>0</v>
+      </c>
+      <c r="H70" t="b">
+        <v>0</v>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201944372</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>1171710365</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>jp-mong</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>[NEW]PDRN 100 ヒアルロン酸 ブースター トナー 250ml, 1個 / 韓国 人気 導入化粧水 ブースター</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F71" t="n">
+        <v>3664</v>
+      </c>
+      <c r="G71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H71" t="b">
+        <v>0</v>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171710365</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>1168040059</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>jp-mong</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>ドクダミ77 スージングトナー 350ml, 1個 / 韓国 人気 どくだみ 敏感肌 ニキビ 跡 赤み 鎮静 保湿 化粧水</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F72" t="n">
+        <v>4313</v>
+      </c>
+      <c r="G72" t="n">
+        <v>2</v>
+      </c>
+      <c r="H72" t="b">
+        <v>0</v>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168040059</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>1145729526</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>jp-mong</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>[大容量] ドクダミ 77 スージングトナー 350ml+詰め替え350ml / 韓国 人気 低刺激 鎮静 化粧水</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F73" t="n">
+        <v>5495</v>
+      </c>
+      <c r="G73" t="n">
+        <v>0</v>
+      </c>
+      <c r="H73" t="b">
+        <v>0</v>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1145729526</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J52"/>
+  <autoFilter ref="A1:J73"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 12, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$90</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J73"/>
+  <dimension ref="A1:J90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3448,8 +3448,705 @@
         </is>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>1191354937</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>kptown</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>【60枚】24Kゴールド レチノール アイパッチ 目元ケア エイジングケア しわ ハリ 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Terez &amp;amp; Honor</t>
+        </is>
+      </c>
+      <c r="F74" t="n">
+        <v>2800</v>
+      </c>
+      <c r="G74" t="n">
+        <v>2</v>
+      </c>
+      <c r="H74" t="b">
+        <v>0</v>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191354937</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>1191354082</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>kptown</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>【60枚】ビタミンC ナイアシンアミド アイパッチ 目元パック 目の下パック トラネキサム酸 ヒアルロン酸 うるおい 保湿 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Terez &amp;amp; Honor</t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>2480</v>
+      </c>
+      <c r="G75" t="n">
+        <v>0</v>
+      </c>
+      <c r="H75" t="b">
+        <v>0</v>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191354082</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>1189557181</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>kptown</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>メラノンX クリーム 30ml×3個セット / 透明感 / くすみケア / 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F76" t="n">
+        <v>3950</v>
+      </c>
+      <c r="G76" t="n">
+        <v>2</v>
+      </c>
+      <c r="H76" t="b">
+        <v>0</v>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189557181</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>1213443102</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>sweetcocoria</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>[正規品]アーバンエコ ハラケケ トナー 150ml, 1個</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ザセム</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>3028</v>
+      </c>
+      <c r="G77" t="n">
+        <v>0</v>
+      </c>
+      <c r="H77" t="b">
+        <v>0</v>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213443102</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>1200735680</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>sweetcocoria</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>[正規品]ALL NEW シグニア リファイニング ウォーターエッセンス 180ml, 1個</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ヘラ</t>
+        </is>
+      </c>
+      <c r="F78" t="n">
+        <v>10543</v>
+      </c>
+      <c r="G78" t="n">
+        <v>0</v>
+      </c>
+      <c r="H78" t="b">
+        <v>0</v>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200735680</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>1196714483</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>sweetcocoria</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>[正規品] レチノール レティジェクション セラム 30ml, 1個</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>アイオペ</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>7345</v>
+      </c>
+      <c r="G79" t="n">
+        <v>0</v>
+      </c>
+      <c r="H79" t="b">
+        <v>0</v>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196714483</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>1165247523</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>sweetcocoria</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>[正規品] オールデイ メイクアップフィクサー 75ml 1個</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ソーナチュラル</t>
+        </is>
+      </c>
+      <c r="F80" t="n">
+        <v>3013</v>
+      </c>
+      <c r="G80" t="n">
+        <v>0</v>
+      </c>
+      <c r="H80" t="b">
+        <v>0</v>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1165247523</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>1213167963</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>sweetcocoria</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>[正規品]インテンスケア ゴールド 24K スネイルフォームクレンザー 150ml, 1個</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>トニーモリー</t>
+        </is>
+      </c>
+      <c r="F81" t="n">
+        <v>2434</v>
+      </c>
+      <c r="G81" t="n">
+        <v>0</v>
+      </c>
+      <c r="H81" t="b">
+        <v>0</v>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213167963</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>1211709109</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>leoshopkorea</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>ミジャンセン サロン10 タンパク質 トリートメント 280ml ハイダメージ 髪質改善 補修 保湿 ヘアケア 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>ミジャンセン</t>
+        </is>
+      </c>
+      <c r="F82" t="n">
+        <v>2541</v>
+      </c>
+      <c r="G82" t="n">
+        <v>0</v>
+      </c>
+      <c r="H82" t="b">
+        <v>0</v>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211709109</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>1195464780</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>leoshopkorea</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>[1+1]大容量 メラトーニング ワンデーアンプル 30ml +30ml 大容量 / 韓国NO.1シミケアアンプル DW-EGF配合 コスパ 肝斑 そばかす 集中ケア 正規品</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>イージーデュー</t>
+        </is>
+      </c>
+      <c r="F83" t="n">
+        <v>11891</v>
+      </c>
+      <c r="G83" t="n">
+        <v>0</v>
+      </c>
+      <c r="H83" t="b">
+        <v>0</v>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195464780</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>1205052684</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>MOMOCHI_SHOP</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>【毛穴洗顔】 ゼロ毛穴 クレンジングフォーム 120g サリチル酸 BHA洗顔 カプセル洗顔 韓国洗顔 毛穴ケア 皮脂ケア フォーム洗顔 韓国スキンケア 角質ケア 毛穴汚れ 韓国コスメ デイリー洗顔</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F84" t="n">
+        <v>2210</v>
+      </c>
+      <c r="G84" t="n">
+        <v>0</v>
+      </c>
+      <c r="H84" t="b">
+        <v>0</v>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205052684</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>1212968157</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>MOMOCHI_SHOP</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>【目元ハリケア】 アイファルト アイバック クリーム 10ml 目元たるみ アイクリーム 保湿 レチノール EGF ナイアシンアミド セラミド 目元ケア 乾燥小じわ 韓国コスメ くまケア</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Dr.Melaxin</t>
+        </is>
+      </c>
+      <c r="F85" t="n">
+        <v>3100</v>
+      </c>
+      <c r="G85" t="n">
+        <v>0</v>
+      </c>
+      <c r="H85" t="b">
+        <v>0</v>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212968157</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>1193601980</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>nuo</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>The Ordinary グリコリックアシッド7% エクスフォリエイティングトナー, 100ml Glycolic Acid 7% Exfoliating Toner</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F86" t="n">
+        <v>3590</v>
+      </c>
+      <c r="G86" t="n">
+        <v>2</v>
+      </c>
+      <c r="H86" t="b">
+        <v>0</v>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193601980</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>1206909143</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>nuo</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>The Ordinary グリコリックアシッド7% エクスフォリエイティングトナー, 240ml Glycolic Acid 7% Exfoliating Toner</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F87" t="n">
+        <v>4620</v>
+      </c>
+      <c r="G87" t="n">
+        <v>0</v>
+      </c>
+      <c r="H87" t="b">
+        <v>0</v>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206909143</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>1202095634</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>nuo</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>The Ordinary グリコリックアシッド7% エクスフォリエイティングトナー, 240ml Glycolic Acid 7% Exfoliating Toner</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F88" t="n">
+        <v>4020</v>
+      </c>
+      <c r="G88" t="n">
+        <v>0</v>
+      </c>
+      <c r="H88" t="b">
+        <v>0</v>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202095634</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>1205563457</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>markets7</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>ガラクトミー エンザイム ピーリングジェル, 75ml, 1個</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F89" t="n">
+        <v>1829</v>
+      </c>
+      <c r="G89" t="n">
+        <v>0</v>
+      </c>
+      <c r="H89" t="b">
+        <v>0</v>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205563457</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>1171042034</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>markets7</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>アクティブクリーンアップクレンジングパウダー酵素洗顔剤, 80g</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F90" t="n">
+        <v>4005</v>
+      </c>
+      <c r="G90" t="n">
+        <v>1</v>
+      </c>
+      <c r="H90" t="b">
+        <v>0</v>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171042034</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J73"/>
+  <autoFilter ref="A1:J90"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 15, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$90</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$105</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J90"/>
+  <dimension ref="A1:J105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4145,8 +4145,623 @@
         </is>
       </c>
     </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>1209385392</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>k-wonderland</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>アドール パフューム ヘアオイル 80ml 5種類から選べる</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>アドル</t>
+        </is>
+      </c>
+      <c r="F91" t="n">
+        <v>3456</v>
+      </c>
+      <c r="G91" t="n">
+        <v>1</v>
+      </c>
+      <c r="H91" t="b">
+        <v>0</v>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209385392</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>1206710414</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>k-wonderland</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>超高含有ヒアルロニックインテンストナー 100時間保湿持続力300g</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>セラディックス</t>
+        </is>
+      </c>
+      <c r="F92" t="n">
+        <v>3148</v>
+      </c>
+      <c r="G92" t="n">
+        <v>0</v>
+      </c>
+      <c r="H92" t="b">
+        <v>0</v>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206710414</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>1205150670</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>shoplikable</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>[1+1+ミニ6枚付き/大容量企画] ポアタイトニング トナーパッド 60枚 ダブル企画 毛穴ケア 韓国パッド 角質ケア 保湿パッド</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F93" t="n">
+        <v>4398</v>
+      </c>
+      <c r="G93" t="n">
+        <v>0</v>
+      </c>
+      <c r="H93" t="b">
+        <v>0</v>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205150670</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>1193784439</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>shoplikable</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>【大容量・本品＋詰め替え】 グローターン エクソソーム ブラシアンプル 100ml＋リフィル100ml 頭皮ケア スカルプ美容液 抜け毛・ハリコシケア</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>lily eve</t>
+        </is>
+      </c>
+      <c r="F94" t="n">
+        <v>5661</v>
+      </c>
+      <c r="G94" t="n">
+        <v>0</v>
+      </c>
+      <c r="H94" t="b">
+        <v>0</v>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193784439</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>1190305789</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>1tyoume</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>RX ザナイアシンアミド15セラム, 20ml</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F95" t="n">
+        <v>1750</v>
+      </c>
+      <c r="G95" t="n">
+        <v>0</v>
+      </c>
+      <c r="H95" t="b">
+        <v>0</v>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190305789</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>1192678454</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>olivegreen</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>【韓国皮膚科医推奨No.1】 肌荒れ・乾燥くすみ対策に！エイシカ365 トラブルリリーフセラムpH4.5 40ml 肌荒れ くすみ 乾燥 美容液</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F96" t="n">
+        <v>2910</v>
+      </c>
+      <c r="G96" t="n">
+        <v>0</v>
+      </c>
+      <c r="H96" t="b">
+        <v>0</v>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192678454</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>1192676012</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>olivegreen</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>【韓国皮膚科医推奨No.1】アトバリア365 クリーム 80mL 保湿クリーム 水分クリーム 保湿カプセル セラミド クリーム 肌荒れ 水分</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F97" t="n">
+        <v>2470</v>
+      </c>
+      <c r="G97" t="n">
+        <v>1</v>
+      </c>
+      <c r="H97" t="b">
+        <v>0</v>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192676012</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>1192160801</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>olivegreen</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>レチノール シカ リペア セラム 30mL</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>イニスフリー</t>
+        </is>
+      </c>
+      <c r="F98" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G98" t="n">
+        <v>0</v>
+      </c>
+      <c r="H98" t="b">
+        <v>0</v>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192160801</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>1150649094</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>tiaramall</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>[1+1]センテラ クイックカーミングパッド 70枚入り2個/パックパッドトナーパッド化粧水トナー鎮静水分保湿</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F99" t="n">
+        <v>3591</v>
+      </c>
+      <c r="G99" t="n">
+        <v>0</v>
+      </c>
+      <c r="H99" t="b">
+        <v>0</v>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1150649094</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>1108196605</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>tiaramall</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>[230ml]アトバリア365クリーム 80ml+ 30ml 5個</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F100" t="n">
+        <v>6678</v>
+      </c>
+      <c r="G100" t="n">
+        <v>0</v>
+      </c>
+      <c r="H100" t="b">
+        <v>0</v>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1108196605</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>1198592013</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>glovey</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>PDRN ピンクペプチドアンプル 30ml</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F101" t="n">
+        <v>3220</v>
+      </c>
+      <c r="G101" t="n">
+        <v>0</v>
+      </c>
+      <c r="H101" t="b">
+        <v>0</v>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1198592013</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>1208272698</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>glovey</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>レッドイレイジングクリーム 2.0 50ml</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F102" t="n">
+        <v>3190</v>
+      </c>
+      <c r="G102" t="n">
+        <v>0</v>
+      </c>
+      <c r="H102" t="b">
+        <v>0</v>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208272698</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>1208271013</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>glovey</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>コラーゲンジェリークリーム 110ml</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F103" t="n">
+        <v>3930</v>
+      </c>
+      <c r="G103" t="n">
+        <v>0</v>
+      </c>
+      <c r="H103" t="b">
+        <v>0</v>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208271013</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>1089059404</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>raramall</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>TXT ボディーソープ ボディソープ 500ml ホワイトムスク</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Kundal</t>
+        </is>
+      </c>
+      <c r="F104" t="n">
+        <v>1998</v>
+      </c>
+      <c r="G104" t="n">
+        <v>0</v>
+      </c>
+      <c r="H104" t="b">
+        <v>0</v>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1089059404</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>1089059413</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>raramall</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>TXT ボディーソープ ボディソープ 500ml クリーンソープ</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Kundal</t>
+        </is>
+      </c>
+      <c r="F105" t="n">
+        <v>1998</v>
+      </c>
+      <c r="G105" t="n">
+        <v>1</v>
+      </c>
+      <c r="H105" t="b">
+        <v>0</v>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1089059413</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J90"/>
+  <autoFilter ref="A1:J105"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 18, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$105</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$122</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J105"/>
+  <dimension ref="A1:J122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4760,8 +4760,705 @@
         </is>
       </c>
     </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>1202885548</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>skingallery</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>リアルカレンデュラ ヒアルロニック トナーパッド 140g/60枚*2 / 毎日スキンケア！鎮静×保湿のデイリートナーパッド</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>エイプリルスキン</t>
+        </is>
+      </c>
+      <c r="F106" t="n">
+        <v>5109</v>
+      </c>
+      <c r="G106" t="n">
+        <v>0</v>
+      </c>
+      <c r="H106" t="b">
+        <v>0</v>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202885548</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>1202885476</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>skingallery</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>ネモパッド リフィル 100枚 限定企画（マデカソサイド） / リフィルでお得！やさしく整える鎮静トナーパッド</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>メディヒール</t>
+        </is>
+      </c>
+      <c r="F107" t="n">
+        <v>2862</v>
+      </c>
+      <c r="G107" t="n">
+        <v>0</v>
+      </c>
+      <c r="H107" t="b">
+        <v>0</v>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202885476</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>1166295332</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>skingallery</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>【3~4点セット 限定企画】 大容量化粧水＋美容液＋乳液＋クリームドクダミ鎮静/桃のナイアシン美 白/シラカバ保湿/クレンジング4ステップ /韓国正規品</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F108" t="n">
+        <v>7563</v>
+      </c>
+      <c r="G108" t="n">
+        <v>0</v>
+      </c>
+      <c r="H108" t="b">
+        <v>0</v>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1166295332</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>1142414152</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>SKINTALKTALK</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>[NEW] ライス スキンケア 70 グロー ミルキー トナー 250ml + 250ml / うるおい×透明感！ライス70％でしっとりツヤ肌へ導くミルキートナー</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F109" t="n">
+        <v>6363</v>
+      </c>
+      <c r="G109" t="n">
+        <v>0</v>
+      </c>
+      <c r="H109" t="b">
+        <v>0</v>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1142414152</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>1142414147</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>SKINTALKTALK</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>[NEW] ライス 4ステップ ク(レンジング パウダー +70 グロー ミルキー トナー + セラム + 70 インテンシブ モイスチャライジング ミルク)</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F110" t="n">
+        <v>10752</v>
+      </c>
+      <c r="G110" t="n">
+        <v>0</v>
+      </c>
+      <c r="H110" t="b">
+        <v>0</v>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1142414147</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>1202885059</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>SKINTALKTALK</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>コラーゲン リフティング マスク 10枚 / ハリUP！引き締めケアでぷるツヤ肌へ</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F111" t="n">
+        <v>2885</v>
+      </c>
+      <c r="G111" t="n">
+        <v>0</v>
+      </c>
+      <c r="H111" t="b">
+        <v>0</v>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202885059</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>1210573446</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>INNOSKIN</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>【正規品】TX アスタキサンチン ブライトニング セラム 30ml / 透明感のあるツヤ肌へ / 乾燥によるくすみをケア / ベタつかない軽やかな使用感</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Dr.Melaxin</t>
+        </is>
+      </c>
+      <c r="F112" t="n">
+        <v>2777</v>
+      </c>
+      <c r="G112" t="n">
+        <v>0</v>
+      </c>
+      <c r="H112" t="b">
+        <v>0</v>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210573446</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>1210573409</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>INNOSKIN</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>【1+1】【200ml】【正規品】マカダミア ダメージケア ソリューション プレミアム ヘアエッセンスオイル 金木犀（キンモクセイ）の香り 100ml × 2本 / ダメージヘアをしっとり補修</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Kundal</t>
+        </is>
+      </c>
+      <c r="F113" t="n">
+        <v>3728</v>
+      </c>
+      <c r="G113" t="n">
+        <v>0</v>
+      </c>
+      <c r="H113" t="b">
+        <v>0</v>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210573409</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>1211721947</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>SOULPRISM</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>ポアタイトニング クレンジングバーム 50ml × 2個セット</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F114" t="n">
+        <v>7482</v>
+      </c>
+      <c r="G114" t="n">
+        <v>0</v>
+      </c>
+      <c r="H114" t="b">
+        <v>0</v>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211721947</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>1137919225</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>SOULPRISM</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>パンテノール クリームウォッシュ 300ml × 2本</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>アトパーム</t>
+        </is>
+      </c>
+      <c r="F115" t="n">
+        <v>6253</v>
+      </c>
+      <c r="G115" t="n">
+        <v>0</v>
+      </c>
+      <c r="H115" t="b">
+        <v>0</v>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1137919225</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>1211388494</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>SOULPRISM</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>ウォーターカプセル サンセラム SPF50+ / PA+++ 40ml × 2個セット</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F116" t="n">
+        <v>7482</v>
+      </c>
+      <c r="G116" t="n">
+        <v>0</v>
+      </c>
+      <c r="H116" t="b">
+        <v>0</v>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211388494</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>1179005673</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>ByU</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>1025 Dokdo Water Gel 10枚 保湿マスク 水光肌 敏感肌 韓国人気</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F117" t="n">
+        <v>4500</v>
+      </c>
+      <c r="G117" t="n">
+        <v>0</v>
+      </c>
+      <c r="H117" t="b">
+        <v>0</v>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1179005673</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>1210143539</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>seoulcosme</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>【正規品】アゼライン酸10 ヒアルロン レッドネス スージングセラム 30ml / 肌荒れ・乾燥ケアにおすすめ</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F118" t="n">
+        <v>3877</v>
+      </c>
+      <c r="G118" t="n">
+        <v>0</v>
+      </c>
+      <c r="H118" t="b">
+        <v>0</v>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210143539</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>1210322268</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>seoulcosme</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>【正規品】セルメイジング 低分子コラーゲン 毛穴弾力アンプル 30ml / 毛穴・ハリ・弾力を同時ケア/ しっとりうるおう保湿アンプル</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>トリデン</t>
+        </is>
+      </c>
+      <c r="F119" t="n">
+        <v>2877</v>
+      </c>
+      <c r="G119" t="n">
+        <v>0</v>
+      </c>
+      <c r="H119" t="b">
+        <v>0</v>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210322268</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>1202573713</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>dermadalia</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>【1+1】顔汗対策 シート スウェトロール 10枚入(5枚×2) 汗ケア 顔用 メイク崩れ防止 夏対策 正規品保証</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>東亜製薬</t>
+        </is>
+      </c>
+      <c r="F120" t="n">
+        <v>4546</v>
+      </c>
+      <c r="G120" t="n">
+        <v>0</v>
+      </c>
+      <c r="H120" t="b">
+        <v>0</v>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202573713</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>1202572261</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>dermadalia</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>顔汗対策 シート 汗ケア 汗拭きシート 5枚入 顔用 メイク崩れ防止 夏対策 スウェトロール 【正規品保証】</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>東亜製薬</t>
+        </is>
+      </c>
+      <c r="F121" t="n">
+        <v>2503</v>
+      </c>
+      <c r="G121" t="n">
+        <v>0</v>
+      </c>
+      <c r="H121" t="b">
+        <v>0</v>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202572261</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>1203205247</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>vanguardvista</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>[正規品] 人気 おすすめ 韓国 クリーム Rx 30ml+7ml セット スキンケア クリーム ギフト</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>ドミナス</t>
+        </is>
+      </c>
+      <c r="F122" t="n">
+        <v>5820</v>
+      </c>
+      <c r="G122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H122" t="b">
+        <v>0</v>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203205247</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J105"/>
+  <autoFilter ref="A1:J122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 21, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$122</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$134</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J122"/>
+  <dimension ref="A1:J134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5457,8 +5457,500 @@
         </is>
       </c>
     </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>1208548847</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>DIONEL</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>【公式】加齢臭・体臭ケア パフュームボディウォッシュ 1000mL 大容量 ボディソープ 韓国コスメ 選べる3種の香り</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>ディオネル</t>
+        </is>
+      </c>
+      <c r="F123" t="n">
+        <v>2900</v>
+      </c>
+      <c r="G123" t="n">
+        <v>0</v>
+      </c>
+      <c r="H123" t="b">
+        <v>0</v>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208548847</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>1208555932</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>DIONEL</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>【公式】チュベローズソープ ボディウォッシュ 1000mL 大容量 加齢臭・体臭ケア パフュームボディソープ 韓国ボディケア 正規品</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>ディオネル</t>
+        </is>
+      </c>
+      <c r="F124" t="n">
+        <v>2900</v>
+      </c>
+      <c r="G124" t="n">
+        <v>0</v>
+      </c>
+      <c r="H124" t="b">
+        <v>0</v>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208555932</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>1208297278</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>DIONEL</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>【公式】インナーパフューム デリケートゾーン 香水 フェミニンケア シークレットラブ ピオニア 5ml 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>ディオネル</t>
+        </is>
+      </c>
+      <c r="F125" t="n">
+        <v>2600</v>
+      </c>
+      <c r="G125" t="n">
+        <v>1</v>
+      </c>
+      <c r="H125" t="b">
+        <v>0</v>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208297278</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>1202055978</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>yeppun</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>UVクリーム SPF50+ PA ++++ 敏感肌向けトーンアップ韓国コスメの人気日焼け止め</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F126" t="n">
+        <v>4370</v>
+      </c>
+      <c r="G126" t="n">
+        <v>0</v>
+      </c>
+      <c r="H126" t="b">
+        <v>0</v>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202055978</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>1174315936</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>yeppun</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>1. マデカラボ マスク 10枚×2箱（リンクル リバイタライズ）</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>センテリアン24</t>
+        </is>
+      </c>
+      <c r="F127" t="n">
+        <v>3800</v>
+      </c>
+      <c r="G127" t="n">
+        <v>0</v>
+      </c>
+      <c r="H127" t="b">
+        <v>0</v>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174315936</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>1207330609</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>joohoh2</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>[メンズ オールインワン 限定企画3種セット] アクアパワー オールインワン 200ml セット ＋クレンザー40ml／オールインワン20ml 付き</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>ビオテルム</t>
+        </is>
+      </c>
+      <c r="F128" t="n">
+        <v>5292</v>
+      </c>
+      <c r="G128" t="n">
+        <v>0</v>
+      </c>
+      <c r="H128" t="b">
+        <v>0</v>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207330609</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>1189316227</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>theories</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>[PDRN 限定セット] ダーマヒーラーポアタイトニングアンプル30ml + トナーパッド2枚 X 6ea</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F129" t="n">
+        <v>5157</v>
+      </c>
+      <c r="G129" t="n">
+        <v>0</v>
+      </c>
+      <c r="H129" t="b">
+        <v>0</v>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189316227</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>1178929059</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>theories</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>[男女共用ヘアラインクッション] デイリースリムクイックヘアーラインクッション/2タイプ から選択</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>ダシュ</t>
+        </is>
+      </c>
+      <c r="F130" t="n">
+        <v>2403</v>
+      </c>
+      <c r="G130" t="n">
+        <v>0</v>
+      </c>
+      <c r="H130" t="b">
+        <v>0</v>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1178929059</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>1152467548</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>theories</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>[40代女性 シワケア必須アイテム] リンクル リペア ほうれい線 パッチ 36個入り</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>MARSHIQUE</t>
+        </is>
+      </c>
+      <c r="F131" t="n">
+        <v>1651</v>
+      </c>
+      <c r="G131" t="n">
+        <v>0</v>
+      </c>
+      <c r="H131" t="b">
+        <v>0</v>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1152467548</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>1072009140</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>KOR--STORE</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>バイオ スキン クレンジング パッド 6g 30枚入 x 2</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>EKE</t>
+        </is>
+      </c>
+      <c r="F132" t="n">
+        <v>5250</v>
+      </c>
+      <c r="G132" t="n">
+        <v>0</v>
+      </c>
+      <c r="H132" t="b">
+        <v>0</v>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1072009140</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>1079690675</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>KOR--STORE</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>CELL LINE PRO リペアクリーム [100口] 半永久化粧材料 アフターケア 1g100個入り</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Clear_pro</t>
+        </is>
+      </c>
+      <c r="F133" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G133" t="n">
+        <v>0</v>
+      </c>
+      <c r="H133" t="b">
+        <v>0</v>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1079690675</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>1132024666</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>happybear</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>[MARTINA GEBHARDT] アボカド アイクリーム 15ml</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>マルティナ</t>
+        </is>
+      </c>
+      <c r="F134" t="n">
+        <v>2790</v>
+      </c>
+      <c r="G134" t="n">
+        <v>1</v>
+      </c>
+      <c r="H134" t="b">
+        <v>0</v>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1132024666</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J122"/>
+  <autoFilter ref="A1:J134"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 24, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$134</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$157</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J134"/>
+  <dimension ref="A1:J157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5949,8 +5949,951 @@
         </is>
       </c>
     </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>1134061516</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>helenskin</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>[2+1]ROSE PDRN EXOSOME MIST, ROSE REPAIR CREAM MIST 80ml, 確かなきらめき, もちっとしたチャオルム</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>EXO HIGHEST+</t>
+        </is>
+      </c>
+      <c r="F135" t="n">
+        <v>15000</v>
+      </c>
+      <c r="G135" t="n">
+        <v>1</v>
+      </c>
+      <c r="H135" t="b">
+        <v>0</v>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1134061516</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>1152064671</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>helenskin</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>ステムセルライン スキンセラムクリーム [中·乾燥肌用3種]</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>ronas</t>
+        </is>
+      </c>
+      <c r="F136" t="n">
+        <v>20700</v>
+      </c>
+      <c r="G136" t="n">
+        <v>0</v>
+      </c>
+      <c r="H136" t="b">
+        <v>0</v>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1152064671</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>1172038726</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>helenskin</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>正規品 VITA-C RETURN SKIN 160ml + SERUM 50ml + RETURN CREAM 100ml</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Merikit</t>
+        </is>
+      </c>
+      <c r="F137" t="n">
+        <v>13500</v>
+      </c>
+      <c r="G137" t="n">
+        <v>0</v>
+      </c>
+      <c r="H137" t="b">
+        <v>0</v>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172038726</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>1150322959</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>helenskin</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Stem Cell Coconut Balm 100ml + Ampoule Essence 150ml 2種</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>ronas</t>
+        </is>
+      </c>
+      <c r="F138" t="n">
+        <v>13000</v>
+      </c>
+      <c r="G138" t="n">
+        <v>2</v>
+      </c>
+      <c r="H138" t="b">
+        <v>0</v>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1150322959</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>1158685803</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>hahahaya</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>グリコリック アシッド 7% エクスポリエイティングトナー 100ml</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F139" t="n">
+        <v>1860</v>
+      </c>
+      <c r="G139" t="n">
+        <v>1</v>
+      </c>
+      <c r="H139" t="b">
+        <v>0</v>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1158685803</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>1169175843</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>leewoostore</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>メイジング グレイス バレエローズ EDT 60ml</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>Bella Philosophy</t>
+        </is>
+      </c>
+      <c r="F140" t="n">
+        <v>12947</v>
+      </c>
+      <c r="G140" t="n">
+        <v>0</v>
+      </c>
+      <c r="H140" t="b">
+        <v>0</v>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1169175843</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>1211844368</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>leewoostore</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>ティーツリー シカ クーリング サンスティック リフィル企画 (20g+20g)</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>bring green</t>
+        </is>
+      </c>
+      <c r="F141" t="n">
+        <v>3429</v>
+      </c>
+      <c r="G141" t="n">
+        <v>0</v>
+      </c>
+      <c r="H141" t="b">
+        <v>0</v>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211844368</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>1210078286</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>leewoostore</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>[目元ケア] カフェインソリューション 5% + EGCG 30ml</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F142" t="n">
+        <v>2745</v>
+      </c>
+      <c r="G142" t="n">
+        <v>0</v>
+      </c>
+      <c r="H142" t="b">
+        <v>0</v>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210078286</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>1210837026</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>leewoostore</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>セラムフィット UVプロテクター 01 クリア 50ml（SPF50+/PA++++)</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>ByUR</t>
+        </is>
+      </c>
+      <c r="F143" t="n">
+        <v>3211</v>
+      </c>
+      <c r="G143" t="n">
+        <v>0</v>
+      </c>
+      <c r="H143" t="b">
+        <v>0</v>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210837026</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>1163545805</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>frombeauty</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>水分バリアPANGヒアルロン酸パンテノールアンプル 100ml</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>EDIT.B</t>
+        </is>
+      </c>
+      <c r="F144" t="n">
+        <v>1995</v>
+      </c>
+      <c r="G144" t="n">
+        <v>0</v>
+      </c>
+      <c r="H144" t="b">
+        <v>0</v>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1163545805</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>1132572987</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>frombeauty</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>サロン10アンプルヘアミスト 200ml</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>ミジャンセン</t>
+        </is>
+      </c>
+      <c r="F145" t="n">
+        <v>2090</v>
+      </c>
+      <c r="G145" t="n">
+        <v>0</v>
+      </c>
+      <c r="H145" t="b">
+        <v>0</v>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1132572987</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>1207185783</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>hadaluv</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>アロエエッセンスマスクパック1個入り50個</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>NatureBy</t>
+        </is>
+      </c>
+      <c r="F146" t="n">
+        <v>3525</v>
+      </c>
+      <c r="G146" t="n">
+        <v>0</v>
+      </c>
+      <c r="H146" t="b">
+        <v>0</v>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207185783</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>1207185764</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>hadaluv</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>ラグジュアリー24kゴールドアンプル100ml 1個</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F147" t="n">
+        <v>2585</v>
+      </c>
+      <c r="G147" t="n">
+        <v>0</v>
+      </c>
+      <c r="H147" t="b">
+        <v>0</v>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207185764</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>1207185727</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>hadaluv</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>アロエ97％スーディングジェル300ml 2個入りポムポムプリン</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>bring green</t>
+        </is>
+      </c>
+      <c r="F148" t="n">
+        <v>4747</v>
+      </c>
+      <c r="G148" t="n">
+        <v>0</v>
+      </c>
+      <c r="H148" t="b">
+        <v>0</v>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207185727</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>1207183624</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>hadaluv</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>ブライトニングヒアルロンフィリングジェル170ml 2個</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>トニーモリー</t>
+        </is>
+      </c>
+      <c r="F149" t="n">
+        <v>2867</v>
+      </c>
+      <c r="G149" t="n">
+        <v>0</v>
+      </c>
+      <c r="H149" t="b">
+        <v>0</v>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207183624</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>1163571137</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>K-BEAUTYBOX</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>グッセラスーパーセラミドクリーム 60ml 2個 高保湿クリームナイトケア</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>ホリカホリカ</t>
+        </is>
+      </c>
+      <c r="F150" t="n">
+        <v>4584</v>
+      </c>
+      <c r="G150" t="n">
+        <v>0</v>
+      </c>
+      <c r="H150" t="b">
+        <v>0</v>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1163571137</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>1210121103</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>ttonce-korea</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>ウォータープルーフ プロ サンクリーム 50g 2個 ト ラベル スポーツ日焼け止め,DEWYTREE ACディープ熱感カーミングマスク 1枚プレゼント</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>BUSHMAN</t>
+        </is>
+      </c>
+      <c r="F151" t="n">
+        <v>6383</v>
+      </c>
+      <c r="G151" t="n">
+        <v>0</v>
+      </c>
+      <c r="H151" t="b">
+        <v>0</v>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210121103</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>1202343508</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>ttonce-korea</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>フットパウダー 35g 3種類から1つ選択（オリジナル・オレンジ・ペパーミント）トラベル【プレゼント】シューズクリーナー3枚 足臭対策 消臭パウダー</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>GRAN'S REMEDY</t>
+        </is>
+      </c>
+      <c r="F152" t="n">
+        <v>3979</v>
+      </c>
+      <c r="G152" t="n">
+        <v>0</v>
+      </c>
+      <c r="H152" t="b">
+        <v>0</v>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202343508</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>1189270361</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>SeoulOppaShop</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>【Wid】 フォリゲン トニック 120ml 2個セット・頭皮ケア・ヘアトニック・抜け毛予防・頭皮栄養・スカルプケア</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Dr.FORHAIR</t>
+        </is>
+      </c>
+      <c r="F153" t="n">
+        <v>5287</v>
+      </c>
+      <c r="G153" t="n">
+        <v>0</v>
+      </c>
+      <c r="H153" t="b">
+        <v>0</v>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189270361</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>1188452071</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>SeoulOppaShop</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>【Wid】 アスコルビルテトラィソパルミテート ソリューション 20% イン ビタミンF / 30ml / 1個 / ビタミンC美容液 / オイル美容液 / 透明感 / ハリケア</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F154" t="n">
+        <v>5841</v>
+      </c>
+      <c r="G154" t="n">
+        <v>0</v>
+      </c>
+      <c r="H154" t="b">
+        <v>0</v>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188452071</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>1188452072</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>SeoulOppaShop</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>【Wid】 グリコール酸 7% エクスフォリエイティング トナー / 240ml / 2個セット / ふき取り化粧水 / 角質ケア / 肌キメ整え / ツヤ肌</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F155" t="n">
+        <v>6385</v>
+      </c>
+      <c r="G155" t="n">
+        <v>0</v>
+      </c>
+      <c r="H155" t="b">
+        <v>0</v>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188452072</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>1179809144</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>SeoulOppaShop</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>[角質ケア] マンデル酸 10％ + HA 30ml 毛穴ケア つるつる美肌 セラム</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F156" t="n">
+        <v>2485</v>
+      </c>
+      <c r="G156" t="n">
+        <v>0</v>
+      </c>
+      <c r="H156" t="b">
+        <v>0</v>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1179809144</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>1209779514</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>J_Beauty_Korea</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>【JTra】 プレミアム ヴィーガン トーンアップ サンクリーム 50ml・SPF50+ PA++++・紫外線対策・肌色補正・保湿</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>dinsee</t>
+        </is>
+      </c>
+      <c r="F157" t="n">
+        <v>3168</v>
+      </c>
+      <c r="G157" t="n">
+        <v>0</v>
+      </c>
+      <c r="H157" t="b">
+        <v>0</v>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209779514</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J134"/>
+  <autoFilter ref="A1:J157"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 27, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$157</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$169</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J157"/>
+  <dimension ref="A1:J169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6892,8 +6892,500 @@
         </is>
       </c>
     </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>1171040599</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>LUnBLOOM</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>ジェントル リフレッシング ボディウォッシュ 1L / 大容量 / 敏感肌用 / 低刺激</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>セタフィル</t>
+        </is>
+      </c>
+      <c r="F158" t="n">
+        <v>3050</v>
+      </c>
+      <c r="G158" t="n">
+        <v>0</v>
+      </c>
+      <c r="H158" t="b">
+        <v>0</v>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171040599</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>1165615884</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>yunimaru</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>ゼロ毛穴パッド2.0 70枚1セット</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F159" t="n">
+        <v>3372</v>
+      </c>
+      <c r="G159" t="n">
+        <v>0</v>
+      </c>
+      <c r="H159" t="b">
+        <v>0</v>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1165615884</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>1207138612</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>yunimaru</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>ビーネイチャー バナナ ホワイト マスクパック 10枚入</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>JM solution</t>
+        </is>
+      </c>
+      <c r="F160" t="n">
+        <v>2422</v>
+      </c>
+      <c r="G160" t="n">
+        <v>0</v>
+      </c>
+      <c r="H160" t="b">
+        <v>0</v>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207138612</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>1207138588</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>yunimaru</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>プランシナジー シルキー マスクパック 10枚入</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>JM solution</t>
+        </is>
+      </c>
+      <c r="F161" t="n">
+        <v>3087</v>
+      </c>
+      <c r="G161" t="n">
+        <v>0</v>
+      </c>
+      <c r="H161" t="b">
+        <v>0</v>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207138588</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>1165228864</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>yunimaru</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>ザリアルノニエネルギーアンプル30ml 1個</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F162" t="n">
+        <v>3087</v>
+      </c>
+      <c r="G162" t="n">
+        <v>0</v>
+      </c>
+      <c r="H162" t="b">
+        <v>0</v>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1165228864</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>1196852846</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>shoppingtree</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>AC ディープカミング ポア サンスティック 20g x 1個 / SPF 50+ PA++++</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>デューイーツリー</t>
+        </is>
+      </c>
+      <c r="F163" t="n">
+        <v>2700</v>
+      </c>
+      <c r="G163" t="n">
+        <v>0</v>
+      </c>
+      <c r="H163" t="b">
+        <v>0</v>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196852846</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>1132737248</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>shoppingtree</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>バランシウム セラミド 高保湿シート マスク 26ml x 10枚</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F164" t="n">
+        <v>3960</v>
+      </c>
+      <c r="G164" t="n">
+        <v>2</v>
+      </c>
+      <c r="H164" t="b">
+        <v>0</v>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1132737248</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>1130447122</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>shoppingtree</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>3番 結果いっぱいのエッセンス トナー 200ml (50種類の発酵/肌の輝き/弾力)</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F165" t="n">
+        <v>3420</v>
+      </c>
+      <c r="G165" t="n">
+        <v>0</v>
+      </c>
+      <c r="H165" t="b">
+        <v>0</v>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1130447122</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>1209269112</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>shoppingtree</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>【1+1】マデカソサイド保湿サンスリーム 痕跡リペア 50+50g / SPF 50+ PA++++</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>メディヒール</t>
+        </is>
+      </c>
+      <c r="F166" t="n">
+        <v>4320</v>
+      </c>
+      <c r="G166" t="n">
+        <v>0</v>
+      </c>
+      <c r="H166" t="b">
+        <v>0</v>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209269112</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>1209886899</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>osondoson7</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>もちもちチョコ 餅パイ 大容量 40個入り 860g</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>チョンウ食品</t>
+        </is>
+      </c>
+      <c r="F167" t="n">
+        <v>3042</v>
+      </c>
+      <c r="G167" t="n">
+        <v>0</v>
+      </c>
+      <c r="H167" t="b">
+        <v>0</v>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209886899</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>1180517208</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>osondoson7</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>レッドブレミッシュクリアヒアルシカスーディングセラム50ml1個</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>ドクタージー</t>
+        </is>
+      </c>
+      <c r="F168" t="n">
+        <v>2400</v>
+      </c>
+      <c r="G168" t="n">
+        <v>0</v>
+      </c>
+      <c r="H168" t="b">
+        <v>0</v>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180517208</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>1211803487</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>osondoson7</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>ベビー＆キッズ低刺激武器車車サンクッションSPF50+ PA++++</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>AVCA</t>
+        </is>
+      </c>
+      <c r="F169" t="n">
+        <v>2172</v>
+      </c>
+      <c r="G169" t="n">
+        <v>0</v>
+      </c>
+      <c r="H169" t="b">
+        <v>0</v>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211803487</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J157"/>
+  <autoFilter ref="A1:J169"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 30, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$169</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$175</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J169"/>
+  <dimension ref="A1:J175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7384,8 +7384,254 @@
         </is>
       </c>
     </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>1193127526</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>bify</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>ルートブースター シャンプー 500ml 頭皮ケア ボリュームタイプ</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>グラフェン</t>
+        </is>
+      </c>
+      <c r="F170" t="n">
+        <v>3679</v>
+      </c>
+      <c r="G170" t="n">
+        <v>0</v>
+      </c>
+      <c r="H170" t="b">
+        <v>0</v>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193127526</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>1062391008</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>hellojp</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>マスターズ プロパッチ 8g + 日焼け止め SPF50 + PA +++ 1.5mL 4セット</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>AHC</t>
+        </is>
+      </c>
+      <c r="F171" t="n">
+        <v>2164</v>
+      </c>
+      <c r="G171" t="n">
+        <v>0</v>
+      </c>
+      <c r="H171" t="b">
+        <v>0</v>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1062391008</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>1191147845</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>studio501</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>ザ ビタ A レティナル ショット タイトニング ブースター15ml</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F172" t="n">
+        <v>1720</v>
+      </c>
+      <c r="G172" t="n">
+        <v>0</v>
+      </c>
+      <c r="H172" t="b">
+        <v>0</v>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191147845</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>1174945980</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>studio501</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>ナイアシンアミド10 TXA 4ダークスポットコレクションセラム30mL</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F173" t="n">
+        <v>2470</v>
+      </c>
+      <c r="G173" t="n">
+        <v>0</v>
+      </c>
+      <c r="H173" t="b">
+        <v>0</v>
+      </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174945980</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>1202768424</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>studio501</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>ポア＋ダークスポット ブライトニングセラム 30ml</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F174" t="n">
+        <v>2090</v>
+      </c>
+      <c r="G174" t="n">
+        <v>1</v>
+      </c>
+      <c r="H174" t="b">
+        <v>0</v>
+      </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202768424</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>1194319670</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>studio501</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>バランスフルシカトナーパッド 60枚</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>トリデン</t>
+        </is>
+      </c>
+      <c r="F175" t="n">
+        <v>1997</v>
+      </c>
+      <c r="G175" t="n">
+        <v>0</v>
+      </c>
+      <c r="H175" t="b">
+        <v>0</v>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194319670</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J169"/>
+  <autoFilter ref="A1:J175"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 33, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$175</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$192</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J175"/>
+  <dimension ref="A1:J192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7630,8 +7630,705 @@
         </is>
       </c>
     </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>1205030887</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>mrm</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>シラカバ保湿サンスティック + シラカバ水分サンクリーム [韓国サンスティック]</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F176" t="n">
+        <v>7380</v>
+      </c>
+      <c r="G176" t="n">
+        <v>2</v>
+      </c>
+      <c r="H176" t="b">
+        <v>0</v>
+      </c>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205030887</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>1201003595</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>mrm</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>PDRN ヒアルロン酸カプセル100 セラム 30ml + PDRN ヒアルロン酸 水分カプセルミスト 100ml</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F177" t="n">
+        <v>6980</v>
+      </c>
+      <c r="G177" t="n">
+        <v>2</v>
+      </c>
+      <c r="H177" t="b">
+        <v>0</v>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201003595</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>1209320737</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>FaceiD</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>[2PACK] クリーンイットゼロ 抹茶クレンジングバーム 100ml</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>バニラコ</t>
+        </is>
+      </c>
+      <c r="F178" t="n">
+        <v>4555</v>
+      </c>
+      <c r="G178" t="n">
+        <v>0</v>
+      </c>
+      <c r="H178" t="b">
+        <v>0</v>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209320737</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>1201575924</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>FaceiD</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>[26SS/New]ピーチフェア ビーガン トーンアップ カプセルサンスクリーン 50ml #SPF50+ PA++++ #グルタチオン #ナイアシンアミド</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>ホイップド</t>
+        </is>
+      </c>
+      <c r="F179" t="n">
+        <v>3353</v>
+      </c>
+      <c r="G179" t="n">
+        <v>0</v>
+      </c>
+      <c r="H179" t="b">
+        <v>0</v>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201575924</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>1201571343</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>FaceiD</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>[25SS/新作]4GF ザマ リペア ハイドロ セラム 30ml #エクソソーム #ナイアシンアミド #ペプチド #ノンコメドジェニック</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>CELORABY</t>
+        </is>
+      </c>
+      <c r="F180" t="n">
+        <v>5397</v>
+      </c>
+      <c r="G180" t="n">
+        <v>0</v>
+      </c>
+      <c r="H180" t="b">
+        <v>0</v>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201571343</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>1203144925</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>ohnewcompany</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>【企画】オールアバウト グロウ カバークリーム (35g) + 大王パフ 1枚付き SPF50+ PA++++ 韓国コスメ ベースメイク 24時間持続 崩れない</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>CHASIN’ RABBITS</t>
+        </is>
+      </c>
+      <c r="F181" t="n">
+        <v>1946</v>
+      </c>
+      <c r="G181" t="n">
+        <v>1</v>
+      </c>
+      <c r="H181" t="b">
+        <v>0</v>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203144925</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>1212016450</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>ohnewcompany</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>薬手名家 Vハン リフティングパッチ PDRN 10K (5枚入) / オリヤン単独企画 二重顎 Vライン 集中ケア 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>YAKSON BEAUTY</t>
+        </is>
+      </c>
+      <c r="F182" t="n">
+        <v>3050</v>
+      </c>
+      <c r="G182" t="n">
+        <v>0</v>
+      </c>
+      <c r="H182" t="b">
+        <v>0</v>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212016450</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>1203335944</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>dreem</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>ボディローション ホワイトマスク520ml /韓国コスメ 韓国スキンケア</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>ブーケガルニ</t>
+        </is>
+      </c>
+      <c r="F183" t="n">
+        <v>2020</v>
+      </c>
+      <c r="G183" t="n">
+        <v>0</v>
+      </c>
+      <c r="H183" t="b">
+        <v>0</v>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203335944</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>1196699361</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>dreem</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>蓮花PDRNヒアルロン光彩セラム 30ml 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>ハンスキン</t>
+        </is>
+      </c>
+      <c r="F184" t="n">
+        <v>5039</v>
+      </c>
+      <c r="G184" t="n">
+        <v>0</v>
+      </c>
+      <c r="H184" t="b">
+        <v>0</v>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196699361</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>1193167209</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>dreem</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>パンテノール クリーム 100ml 韓国スキンケア 韓国 コスメ #水分#保湿 毛穴ケア</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>アトパーム</t>
+        </is>
+      </c>
+      <c r="F185" t="n">
+        <v>4504</v>
+      </c>
+      <c r="G185" t="n">
+        <v>1</v>
+      </c>
+      <c r="H185" t="b">
+        <v>0</v>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193167209</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>1182429127</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>rseed</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>【PDRNマスクパック 1枚GIFT】PDRNヒアルロン酸カプセル 100セラム, 本品 30ml(シートマスク贈呈！) orレフィル 30ml 水光注射 弾力 保湿 ツヤ</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F186" t="n">
+        <v>1770</v>
+      </c>
+      <c r="G186" t="n">
+        <v>3</v>
+      </c>
+      <c r="H186" t="b">
+        <v>0</v>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1182429127</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>1194502685</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>sizuccu</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>[NEW/透明ケア] スキン＆ラボ グルタチオントナー 200ml 1個</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>スキンアンドラブ</t>
+        </is>
+      </c>
+      <c r="F187" t="n">
+        <v>5100</v>
+      </c>
+      <c r="G187" t="n">
+        <v>0</v>
+      </c>
+      <c r="H187" t="b">
+        <v>0</v>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J187" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194502685</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>1158942439</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>sizuccu</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>マダガスカル センテラクイックカミングパッド1個</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F188" t="n">
+        <v>4800</v>
+      </c>
+      <c r="G188" t="n">
+        <v>0</v>
+      </c>
+      <c r="H188" t="b">
+        <v>0</v>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1158942439</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>1156741239</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>sizuccu</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>ドクダミヒアルロンスージング アンプル50ml</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>グーダル</t>
+        </is>
+      </c>
+      <c r="F189" t="n">
+        <v>4460</v>
+      </c>
+      <c r="G189" t="n">
+        <v>0</v>
+      </c>
+      <c r="H189" t="b">
+        <v>0</v>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1156741239</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>1171947071</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>CallaBoutique</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>【正規品】 デイリートナーパッド 80枚</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>NEEDLY</t>
+        </is>
+      </c>
+      <c r="F190" t="n">
+        <v>1990</v>
+      </c>
+      <c r="G190" t="n">
+        <v>0</v>
+      </c>
+      <c r="H190" t="b">
+        <v>0</v>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171947071</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>1171946936</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>CallaBoutique</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>【正規品】 センテラクイックカーミングパッド 70枚</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F191" t="n">
+        <v>1590</v>
+      </c>
+      <c r="G191" t="n">
+        <v>3</v>
+      </c>
+      <c r="H191" t="b">
+        <v>0</v>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J191" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171946936</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>1197892266</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>CallaBoutique</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>【正規品】 グロウクリーミーボディスクラブ ヌバニラ 300ml</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>UNOVE</t>
+        </is>
+      </c>
+      <c r="F192" t="n">
+        <v>3090</v>
+      </c>
+      <c r="G192" t="n">
+        <v>0</v>
+      </c>
+      <c r="H192" t="b">
+        <v>0</v>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197892266</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J175"/>
+  <autoFilter ref="A1:J192"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 36, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$192</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$201</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J192"/>
+  <dimension ref="A1:J201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8327,8 +8327,377 @@
         </is>
       </c>
     </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>1160418590</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>julynana</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>[2種セット]ブリングリーン ティーツリー シカスージングトナー 250ml + クリーム100ml</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>bring green</t>
+        </is>
+      </c>
+      <c r="F193" t="n">
+        <v>3510</v>
+      </c>
+      <c r="G193" t="n">
+        <v>0</v>
+      </c>
+      <c r="H193" t="b">
+        <v>0</v>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1160418590</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>1152030824</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>julynana</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>[人気2種セット]ホワイトトリュフファーストスプレーセラム 100ml +ウォータフルトーンアップサンクリーム50ml</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F194" t="n">
+        <v>5640</v>
+      </c>
+      <c r="G194" t="n">
+        <v>0</v>
+      </c>
+      <c r="H194" t="b">
+        <v>0</v>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1152030824</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>1196415617</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Widgo2</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>【WiD2】 AHA・BHA配合 28デイズヒアルクリーム (30ml) ザラつきOFF！なめらか透明肌へ 1個</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F195" t="n">
+        <v>2020</v>
+      </c>
+      <c r="G195" t="n">
+        <v>1</v>
+      </c>
+      <c r="H195" t="b">
+        <v>0</v>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196415617</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>1196366572</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Widgo2</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>【WiD2】 ガラクトナイアシンエッセンスマスク 10枚入り 肌をクリアに・高保湿・エイジングケア</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F196" t="n">
+        <v>2851</v>
+      </c>
+      <c r="G196" t="n">
+        <v>0</v>
+      </c>
+      <c r="H196" t="b">
+        <v>0</v>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J196" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196366572</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>1210829738</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>beautyluv</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>プレミアムもちソープ[グリーン], 120g</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>アレンシア</t>
+        </is>
+      </c>
+      <c r="F197" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G197" t="n">
+        <v>1</v>
+      </c>
+      <c r="H197" t="b">
+        <v>0</v>
+      </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210829738</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>1213607022</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>beautyluv</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>リアルマットメイクアップセッティングフィックスミスト, 75ml</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>ソーナチュラル</t>
+        </is>
+      </c>
+      <c r="F198" t="n">
+        <v>2397</v>
+      </c>
+      <c r="G198" t="n">
+        <v>0</v>
+      </c>
+      <c r="H198" t="b">
+        <v>0</v>
+      </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213607022</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>1211081043</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>beautyluv</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>PDRNアイパッチ</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>アビブ</t>
+        </is>
+      </c>
+      <c r="F199" t="n">
+        <v>2469</v>
+      </c>
+      <c r="G199" t="n">
+        <v>0</v>
+      </c>
+      <c r="H199" t="b">
+        <v>0</v>
+      </c>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211081043</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>1095687901</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>JUJUHONG</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>[KERASYS] ADVANCED KERAMIDE トリートメント！ ヘアパック！ シャンプー！ 人気商品集電線 1+1 [正規品] 韓国ブランド(鎮静/弾力/保湿/栄養供給/活力)</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>ケラシス</t>
+        </is>
+      </c>
+      <c r="F200" t="n">
+        <v>2980</v>
+      </c>
+      <c r="G200" t="n">
+        <v>0</v>
+      </c>
+      <c r="H200" t="b">
+        <v>0</v>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1095687901</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>1101562835</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>JUJUHONG</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>ビフィダ バイオーム アンプル パッド 70枚</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F201" t="n">
+        <v>2970</v>
+      </c>
+      <c r="G201" t="n">
+        <v>1</v>
+      </c>
+      <c r="H201" t="b">
+        <v>0</v>
+      </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1101562835</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J192"/>
+  <autoFilter ref="A1:J201"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 39, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$201</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$208</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J201"/>
+  <dimension ref="A1:J208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8696,8 +8696,295 @@
         </is>
       </c>
     </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>1191662969</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>bloomingseoul</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>ブルービーン B5-PDRN マイルドローション 230ml(+ブルービーンクリーム7ml)</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>bring green</t>
+        </is>
+      </c>
+      <c r="F202" t="n">
+        <v>2374</v>
+      </c>
+      <c r="G202" t="n">
+        <v>3</v>
+      </c>
+      <c r="H202" t="b">
+        <v>0</v>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191662969</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>1191426823</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>todaymart</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>ダメージセラピーノーウォッシュトリートメントEXトゥルーミー(パープル) 250ml + 250ml(詰め替え)</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>GROWUS</t>
+        </is>
+      </c>
+      <c r="F203" t="n">
+        <v>3190</v>
+      </c>
+      <c r="G203" t="n">
+        <v>2</v>
+      </c>
+      <c r="H203" t="b">
+        <v>0</v>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191426823</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>1191773279</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>todaymart</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>オードパルファム ローズウッド 30ml　香水／韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>pleuvoir</t>
+        </is>
+      </c>
+      <c r="F204" t="n">
+        <v>4990</v>
+      </c>
+      <c r="G204" t="n">
+        <v>2</v>
+      </c>
+      <c r="H204" t="b">
+        <v>0</v>
+      </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191773279</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>1190357115</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>lifetipsshop</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>アゼライン酸CICAスキンクリアトナー 250ml</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F205" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G205" t="n">
+        <v>0</v>
+      </c>
+      <c r="H205" t="b">
+        <v>0</v>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190357115</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>1157789377</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>lifetipsshop</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>ドクダミLHAモイスチャーピーリングジェル 120ml</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F206" t="n">
+        <v>1710</v>
+      </c>
+      <c r="G206" t="n">
+        <v>0</v>
+      </c>
+      <c r="H206" t="b">
+        <v>0</v>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1157789377</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>1203834476</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>KORESHOP</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>白樺水分サンクッション 15g</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F207" t="n">
+        <v>2109</v>
+      </c>
+      <c r="G207" t="n">
+        <v>3</v>
+      </c>
+      <c r="H207" t="b">
+        <v>0</v>
+      </c>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203834476</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>1162429093</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>yoo_k1120</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>コダリビノパーフェクトラジアンズセラム30mlホワイト ニングホワイト ニングアンプル（フランスセラム）</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>コーダリー</t>
+        </is>
+      </c>
+      <c r="F208" t="n">
+        <v>7340</v>
+      </c>
+      <c r="G208" t="n">
+        <v>1</v>
+      </c>
+      <c r="H208" t="b">
+        <v>0</v>
+      </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1162429093</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J201"/>
+  <autoFilter ref="A1:J208"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 42, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$208</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$221</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J208"/>
+  <dimension ref="A1:J221"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8983,8 +8983,541 @@
         </is>
       </c>
     </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>1206600283</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>LovingYou</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>PDRNヒアルロン酸ハイドレイティングミスト, 100ml</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F209" t="n">
+        <v>2250</v>
+      </c>
+      <c r="G209" t="n">
+        <v>0</v>
+      </c>
+      <c r="H209" t="b">
+        <v>0</v>
+      </c>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206600283</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>1205881900</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>LovingYou</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>PDRNヒアルロン酸カプセル100セラム 30ml</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F210" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G210" t="n">
+        <v>0</v>
+      </c>
+      <c r="H210" t="b">
+        <v>0</v>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205881900</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>1204898098</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>LovingYou</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>PDRNヒアルロン酸カプセル100セラム, 30ml, 2個</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F211" t="n">
+        <v>3830</v>
+      </c>
+      <c r="G211" t="n">
+        <v>0</v>
+      </c>
+      <c r="H211" t="b">
+        <v>0</v>
+      </c>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J211" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204898098</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>1204581160</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>LovingYou</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>PDRNヒアルロン酸ハイドレイティングミスト, 100ml, 2個</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F212" t="n">
+        <v>4500</v>
+      </c>
+      <c r="G212" t="n">
+        <v>0</v>
+      </c>
+      <c r="H212" t="b">
+        <v>0</v>
+      </c>
+      <c r="I212" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J212" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204581160</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>1203907708</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>LovingYou</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>トーンブライトニングカプセルアンプル, 100ml, 2個 美容液 セラム センテラ 敏感肌 毛穴ケア 保湿 くすみ ツボクサ 低刺激 弱酸性 ナイアシンアミド 大容量 トラブルケア トラネキサム酸</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F213" t="n">
+        <v>4996</v>
+      </c>
+      <c r="G213" t="n">
+        <v>0</v>
+      </c>
+      <c r="H213" t="b">
+        <v>0</v>
+      </c>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203907708</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>1151747985</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Luminomarket</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>ヒーティングガードノーウォッシュトリートメント, 147ml</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>UNOVE</t>
+        </is>
+      </c>
+      <c r="F214" t="n">
+        <v>2396</v>
+      </c>
+      <c r="G214" t="n">
+        <v>1</v>
+      </c>
+      <c r="H214" t="b">
+        <v>0</v>
+      </c>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1151747985</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>1213236507</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Luminomarket</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>ディープダメージトリートメントEX, 207ml</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>UNOVE</t>
+        </is>
+      </c>
+      <c r="F215" t="n">
+        <v>2195</v>
+      </c>
+      <c r="G215" t="n">
+        <v>0</v>
+      </c>
+      <c r="H215" t="b">
+        <v>0</v>
+      </c>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J215" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213236507</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>1210877861</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>K_Beauty_Station</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>【NEW・化粧ノリUPミスト】シェイキングシナジーミスト 50ml 3種</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>フィー</t>
+        </is>
+      </c>
+      <c r="F216" t="n">
+        <v>2438</v>
+      </c>
+      <c r="G216" t="n">
+        <v>0</v>
+      </c>
+      <c r="H216" t="b">
+        <v>0</v>
+      </c>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J216" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210877861</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>1197720706</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>K_Beauty_Station</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>【今だけ限定！企画】キャロットカロテンカーミングウォーターパッド, 60枚</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>スキンフード</t>
+        </is>
+      </c>
+      <c r="F217" t="n">
+        <v>1964</v>
+      </c>
+      <c r="G217" t="n">
+        <v>3</v>
+      </c>
+      <c r="H217" t="b">
+        <v>0</v>
+      </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197720706</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>1188680603</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>relationmarketing</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>プラスリストア UVローション日焼け止めローション SPF50+ PA++++30ml</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>プラスリストア</t>
+        </is>
+      </c>
+      <c r="F218" t="n">
+        <v>3391</v>
+      </c>
+      <c r="G218" t="n">
+        <v>1</v>
+      </c>
+      <c r="H218" t="b">
+        <v>0</v>
+      </c>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J218" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188680603</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>1200553566</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>relationmarketing</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>ルベル IAU イオ クレンジング リラックスメント シャンプー 1000ml＆イオ クリーム シルキーリペア トリートメント1000ml 詰め替え セット</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>イオ</t>
+        </is>
+      </c>
+      <c r="F219" t="n">
+        <v>7733</v>
+      </c>
+      <c r="G219" t="n">
+        <v>0</v>
+      </c>
+      <c r="H219" t="b">
+        <v>0</v>
+      </c>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J219" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200553566</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>1188922874</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>guangjingyouxiang1</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>ビオデルマ サンシビオ エイチツーオーD 500ml</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>ビオデルマ</t>
+        </is>
+      </c>
+      <c r="F220" t="n">
+        <v>3052</v>
+      </c>
+      <c r="G220" t="n">
+        <v>0</v>
+      </c>
+      <c r="H220" t="b">
+        <v>0</v>
+      </c>
+      <c r="I220" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J220" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188922874</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>1143959163</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>ggoolnim</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>ロレアルパリトタルリフェア5モイスチャークリームプロエックスヘアローション 110g x 1個 あるいは 2個 選択</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>アモーレパシフィック</t>
+        </is>
+      </c>
+      <c r="F221" t="n">
+        <v>2950</v>
+      </c>
+      <c r="G221" t="n">
+        <v>1</v>
+      </c>
+      <c r="H221" t="b">
+        <v>0</v>
+      </c>
+      <c r="I221" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J221" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1143959163</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J208"/>
+  <autoFilter ref="A1:J221"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 45, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$221</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$232</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J221"/>
+  <dimension ref="A1:J232"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9516,8 +9516,459 @@
         </is>
       </c>
     </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>1187759601</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>joungho</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>【韓国旅行の定番】垢すり石鹸＆グローブ6個セットまるで韓国エステ！自宅で叶う極上のツルツル美肌体験</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>ダイソー</t>
+        </is>
+      </c>
+      <c r="F222" t="n">
+        <v>2990</v>
+      </c>
+      <c r="G222" t="n">
+        <v>2</v>
+      </c>
+      <c r="H222" t="b">
+        <v>0</v>
+      </c>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J222" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1187759601</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>1194068552</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>joungho</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>韓国国民アイテム キュアアルファカーミングアロエクリーム 50g 2個</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>CURE</t>
+        </is>
+      </c>
+      <c r="F223" t="n">
+        <v>2990</v>
+      </c>
+      <c r="G223" t="n">
+        <v>0</v>
+      </c>
+      <c r="H223" t="b">
+        <v>0</v>
+      </c>
+      <c r="I223" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J223" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194068552</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>1102236597</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>MACARON-CAT</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>チョゴンジン クレンジング フォーム 150ml / 洗顔フォーム/ 洗顔料/ メイク落とし/ 化粧落とし/ クレンジング/ 毛穴ケア/ 乾燥肌/ 保湿ケア/ 肌荒れ/ ツヤ/ スキンケア</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>ミシャ</t>
+        </is>
+      </c>
+      <c r="F224" t="n">
+        <v>2399</v>
+      </c>
+      <c r="G224" t="n">
+        <v>0</v>
+      </c>
+      <c r="H224" t="b">
+        <v>0</v>
+      </c>
+      <c r="I224" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J224" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1102236597</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>1112935346</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>puerueme</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>【選べる2個セット】デビルズ パフュームファンタジーシャンプー &amp;amp; コンディショナー, 1L+1L</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>ケラシス</t>
+        </is>
+      </c>
+      <c r="F225" t="n">
+        <v>3300</v>
+      </c>
+      <c r="G225" t="n">
+        <v>1</v>
+      </c>
+      <c r="H225" t="b">
+        <v>0</v>
+      </c>
+      <c r="I225" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1112935346</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>1084157476</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>puerueme</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>【NEW COLOR】イージーブロウトーンチェンジャー (5回分) /ブリーチ / 眉毛脱色 /眉カラーケア</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>サムバイミー</t>
+        </is>
+      </c>
+      <c r="F226" t="n">
+        <v>4110</v>
+      </c>
+      <c r="G226" t="n">
+        <v>0</v>
+      </c>
+      <c r="H226" t="b">
+        <v>0</v>
+      </c>
+      <c r="I226" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J226" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1084157476</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>1194225739</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>misssk</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>ソリッドパフューム7g 香り : レモンビヌ&amp;nbsp;/ バニラパーク 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>SENNOK</t>
+        </is>
+      </c>
+      <c r="F227" t="n">
+        <v>5366</v>
+      </c>
+      <c r="G227" t="n">
+        <v>0</v>
+      </c>
+      <c r="H227" t="b">
+        <v>0</v>
+      </c>
+      <c r="I227" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J227" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194225739</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>1173671918</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>misssk</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>ジェントルスキンクレンザー 473ml 大容量 コスパ 低刺激 乾燥肌 洗顔 敏感肌 クレンジング 肌荒れ /韓国コスメ/韓国スキンケア</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>セタフィル</t>
+        </is>
+      </c>
+      <c r="F228" t="n">
+        <v>2198</v>
+      </c>
+      <c r="G228" t="n">
+        <v>1</v>
+      </c>
+      <c r="H228" t="b">
+        <v>0</v>
+      </c>
+      <c r="I228" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J228" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1173671918</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>1118867909</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>k-seoul</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>グリコリックアシッド7%エクスポリエイティングトナー 100ml韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F229" t="n">
+        <v>2346</v>
+      </c>
+      <c r="G229" t="n">
+        <v>0</v>
+      </c>
+      <c r="H229" t="b">
+        <v>0</v>
+      </c>
+      <c r="I229" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J229" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1118867909</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>1188512361</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>k-seoul</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>ノニアクネバブルクレンザー, 155ml /韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F230" t="n">
+        <v>2360</v>
+      </c>
+      <c r="G230" t="n">
+        <v>0</v>
+      </c>
+      <c r="H230" t="b">
+        <v>0</v>
+      </c>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J230" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188512361</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>1130886239</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>k-seoul</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>バイオガ ビオチン ダメージヘア改善 脱毛緩和シャンプー 1000ml /韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>BIORGA</t>
+        </is>
+      </c>
+      <c r="F231" t="n">
+        <v>5000</v>
+      </c>
+      <c r="G231" t="n">
+        <v>0</v>
+      </c>
+      <c r="H231" t="b">
+        <v>0</v>
+      </c>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J231" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1130886239</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>1097276457</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>k-seoul</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>リアルカレンデュラピールオフパック, 100g 韓国スキンケア 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>エイプリルスキン</t>
+        </is>
+      </c>
+      <c r="F232" t="n">
+        <v>3109</v>
+      </c>
+      <c r="G232" t="n">
+        <v>1</v>
+      </c>
+      <c r="H232" t="b">
+        <v>0</v>
+      </c>
+      <c r="I232" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J232" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1097276457</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J221"/>
+  <autoFilter ref="A1:J232"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 48, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$232</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$242</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J232"/>
+  <dimension ref="A1:J242"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9967,8 +9967,418 @@
         </is>
       </c>
     </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>1115638534</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>dal25</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>旅行用ヘアボディ5種+コットンポーチ1セット 韓国シャンプー 純正品 旅行キット トラベルキット トリートメント ボディウォッシュ ボディローション クレンジングフォーム 旅行 携帯用シャンプー</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>NARD</t>
+        </is>
+      </c>
+      <c r="F233" t="n">
+        <v>2690</v>
+      </c>
+      <c r="G233" t="n">
+        <v>0</v>
+      </c>
+      <c r="H233" t="b">
+        <v>0</v>
+      </c>
+      <c r="I233" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J233" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1115638534</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>1147146315</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>jinytrading</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>PDRN ピンク グルタチオン セラム ミスト 100ml 水分 保湿 弾力 韓国化粧品 韓国美容ギフト</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F234" t="n">
+        <v>2961</v>
+      </c>
+      <c r="G234" t="n">
+        <v>0</v>
+      </c>
+      <c r="H234" t="b">
+        <v>0</v>
+      </c>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J234" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1147146315</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>1159784308</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>jinytrading</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>ビタCプラス アスコルビン酸 クリアコンプレクション フォーミングクレンザー 120ml 高濃度ビタミンC フォームクレンジング 水分 保湿 韓国化粧品 韓国美容ギフト</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>ミシャ</t>
+        </is>
+      </c>
+      <c r="F235" t="n">
+        <v>1971</v>
+      </c>
+      <c r="G235" t="n">
+        <v>0</v>
+      </c>
+      <c r="H235" t="b">
+        <v>0</v>
+      </c>
+      <c r="I235" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J235" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1159784308</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>1170826458</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>kseoulshop</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>[コラーゲン美容液]椿 ディープコラーゲン 弾力アンプル 30ml/美容液/コラーゲン/エイジングケア・ハリ・たるみ・毛穴ケア・毛穴たるみ・キメを整える・リフトアップ・保湿・水分ケア・韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F236" t="n">
+        <v>4765</v>
+      </c>
+      <c r="G236" t="n">
+        <v>1</v>
+      </c>
+      <c r="H236" t="b">
+        <v>0</v>
+      </c>
+      <c r="I236" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J236" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1170826458</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>1182484329</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>kseoulshop</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>[企画セット]桃エキス モイスチャーマスク 5枚入り＋1枚プレゼント企画セット/パック・マスクパック・シートマスクパック・韓国パック・保湿ケアパック・トーンケア・トーンアップ</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F237" t="n">
+        <v>2816</v>
+      </c>
+      <c r="G237" t="n">
+        <v>2</v>
+      </c>
+      <c r="H237" t="b">
+        <v>0</v>
+      </c>
+      <c r="I237" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J237" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1182484329</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>1176474050</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>kseoulshop</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>[ハリケア]シカ コラーゲン マスク 30枚入／シートマスクパック・パック・韓国パック・エイジングケア・ハリ・たるみ・赤みケア・ニキビケア・トラブルケア・弾力・リフトアップパック</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F238" t="n">
+        <v>3733</v>
+      </c>
+      <c r="G238" t="n">
+        <v>1</v>
+      </c>
+      <c r="H238" t="b">
+        <v>0</v>
+      </c>
+      <c r="I238" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J238" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1176474050</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>1212714696</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>cosmefuku</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>シェイキングミスト 50ml 全3種(フローズンゼリー/パールグロウ/パウダーキープ) 韓国コスメ ベースメイクキープミスト</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>フィー</t>
+        </is>
+      </c>
+      <c r="F239" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G239" t="n">
+        <v>0</v>
+      </c>
+      <c r="H239" t="b">
+        <v>0</v>
+      </c>
+      <c r="I239" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J239" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212714696</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>1207120098</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>LUNORASELECT</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>マスターズ エアリッチ サンスティック 22g 2個 セット ポケモン エディション 日焼け止め UVカット 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>AHC</t>
+        </is>
+      </c>
+      <c r="F240" t="n">
+        <v>4836</v>
+      </c>
+      <c r="G240" t="n">
+        <v>1</v>
+      </c>
+      <c r="H240" t="b">
+        <v>0</v>
+      </c>
+      <c r="I240" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J240" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207120098</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>1208245842</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>rarakr</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>コラーゲン バウンシング スリーピング＆ウォッシュオフ マスク (100ml) 弾力・保湿</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>GIK</t>
+        </is>
+      </c>
+      <c r="F241" t="n">
+        <v>2709</v>
+      </c>
+      <c r="G241" t="n">
+        <v>0</v>
+      </c>
+      <c r="H241" t="b">
+        <v>0</v>
+      </c>
+      <c r="I241" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J241" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208245842</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>1208668038</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>rarakr</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>フレッシュ クラウド ボディ＆スカルプ スクラブ (ラベンダー＆ペア) 260g ヴィーガン 頭皮ケア 角質ケア 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>アレンシア</t>
+        </is>
+      </c>
+      <c r="F242" t="n">
+        <v>3680</v>
+      </c>
+      <c r="G242" t="n">
+        <v>0</v>
+      </c>
+      <c r="H242" t="b">
+        <v>0</v>
+      </c>
+      <c r="I242" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J242" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208668038</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J232"/>
+  <autoFilter ref="A1:J242"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 51, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$242</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$251</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J242"/>
+  <dimension ref="A1:J251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10377,8 +10377,377 @@
         </is>
       </c>
     </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>1117552337</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>rivina84</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>韓国スキンケア レチノエート X8 プロ ディープリンクル スキンソフナー 150ml ハリと弾力のある潤い肌のためのエッセンス</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>エンプラニ</t>
+        </is>
+      </c>
+      <c r="F243" t="n">
+        <v>7900</v>
+      </c>
+      <c r="G243" t="n">
+        <v>0</v>
+      </c>
+      <c r="H243" t="b">
+        <v>0</v>
+      </c>
+      <c r="I243" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1117552337</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>1166659309</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>rivina84</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>秘貼(ビチョプ) ディスカバリーセット/ アンプル / トナー / エマルジョン / クレンジングフォーム / 韓国コスメ 下地 角質 キメケア エイジングケア</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>THE WHOO</t>
+        </is>
+      </c>
+      <c r="F244" t="n">
+        <v>12000</v>
+      </c>
+      <c r="G244" t="n">
+        <v>0</v>
+      </c>
+      <c r="H244" t="b">
+        <v>0</v>
+      </c>
+      <c r="I244" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J244" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1166659309</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>1180354766</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>risingmother</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>[1+1/限定企画] スキンフード キャロット カロチン カミング ウォーターパッド 60枚 ダブル企画</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>スキンフード</t>
+        </is>
+      </c>
+      <c r="F245" t="n">
+        <v>6791</v>
+      </c>
+      <c r="G245" t="n">
+        <v>0</v>
+      </c>
+      <c r="H245" t="b">
+        <v>0</v>
+      </c>
+      <c r="I245" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J245" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180354766</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>1207273381</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>risingmother</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>PDRN ピンク コラーゲン バーム セラム 95ml 炭酸 泡 美容液 水光肌 弾力 ほうれい線 乾燥肌 エイジングケア 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F246" t="n">
+        <v>5049</v>
+      </c>
+      <c r="G246" t="n">
+        <v>0</v>
+      </c>
+      <c r="H246" t="b">
+        <v>0</v>
+      </c>
+      <c r="I246" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J246" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207273381</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>1097848142</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>sundaykoreatown</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>ローズペール ヘアケアセット シャンプー300ml+トリートメント300ml</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>ノンフィクション</t>
+        </is>
+      </c>
+      <c r="F247" t="n">
+        <v>10440</v>
+      </c>
+      <c r="G247" t="n">
+        <v>2</v>
+      </c>
+      <c r="H247" t="b">
+        <v>0</v>
+      </c>
+      <c r="I247" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J247" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1097848142</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>1195385472</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>sundaykoreatown</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>[NEW] メディヒール マデカソサイド UVカット アウトドアサンパッチ [ワイドプロテクション]</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>メディヒール</t>
+        </is>
+      </c>
+      <c r="F248" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G248" t="n">
+        <v>0</v>
+      </c>
+      <c r="H248" t="b">
+        <v>0</v>
+      </c>
+      <c r="I248" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J248" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195385472</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>1190175660</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>flymong-korea</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>マダガスカルセントラアンプル 55ml, 1個</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F249" t="n">
+        <v>2795</v>
+      </c>
+      <c r="G249" t="n">
+        <v>1</v>
+      </c>
+      <c r="H249" t="b">
+        <v>0</v>
+      </c>
+      <c r="I249" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J249" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190175660</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>1190175438</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>flymong-korea</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>ノーセバム サンクッション EX SPF50+ PA++++, 1個</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>イニスフリー</t>
+        </is>
+      </c>
+      <c r="F250" t="n">
+        <v>2215</v>
+      </c>
+      <c r="G250" t="n">
+        <v>0</v>
+      </c>
+      <c r="H250" t="b">
+        <v>0</v>
+      </c>
+      <c r="I250" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J250" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190175438</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>1190295644</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>puchimochi_lab</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>ダーマヒーラー 毛穴引き締めアンプル 30ml【陶器肌／毛穴キュッとPDRN】</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F251" t="n">
+        <v>4225</v>
+      </c>
+      <c r="G251" t="n">
+        <v>0</v>
+      </c>
+      <c r="H251" t="b">
+        <v>0</v>
+      </c>
+      <c r="I251" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J251" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190295644</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J242"/>
+  <autoFilter ref="A1:J251"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 54, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$251</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$264</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J251"/>
+  <dimension ref="A1:J264"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10746,8 +10746,541 @@
         </is>
       </c>
     </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>1145594895</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>sinature22</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>【正規品扱い店】【1+1】【本品+レフィル】ダイブイン低分子ヒアルロン酸セラム, 50mL*2</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>トリデン</t>
+        </is>
+      </c>
+      <c r="F252" t="n">
+        <v>4879</v>
+      </c>
+      <c r="G252" t="n">
+        <v>0</v>
+      </c>
+      <c r="H252" t="b">
+        <v>0</v>
+      </c>
+      <c r="I252" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J252" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1145594895</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>1145594718</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>sinature22</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>【韓国コスメ】【正規品扱い店】シルクペプチドインテンシブリフティングアンプル35ML</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>Sung Boon Editor</t>
+        </is>
+      </c>
+      <c r="F253" t="n">
+        <v>2407</v>
+      </c>
+      <c r="G253" t="n">
+        <v>0</v>
+      </c>
+      <c r="H253" t="b">
+        <v>0</v>
+      </c>
+      <c r="I253" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J253" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1145594718</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>1174312286</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>sinature23</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>【1+1】【韓国コスメ】【正規品扱い店】[病院専用] ラポラピルナトックス 50ml - シミ改善＆肌トーンアップの機能性クリーム！</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>Dermagen</t>
+        </is>
+      </c>
+      <c r="F254" t="n">
+        <v>7128</v>
+      </c>
+      <c r="G254" t="n">
+        <v>0</v>
+      </c>
+      <c r="H254" t="b">
+        <v>0</v>
+      </c>
+      <c r="I254" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J254" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174312286</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>1146499682</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>sinature23</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>【韓国コスメ】【正規品扱い店】タイムエナジーリセッティングエマルジョン 120ml - 時間を超える美肌の秘訣！</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>sum37</t>
+        </is>
+      </c>
+      <c r="F255" t="n">
+        <v>4781</v>
+      </c>
+      <c r="G255" t="n">
+        <v>0</v>
+      </c>
+      <c r="H255" t="b">
+        <v>0</v>
+      </c>
+      <c r="I255" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J255" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1146499682</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>1146499598</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>sinature23</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>【韓国コスメ】【正規品扱い店】[5番企画セット] 白玉リンガーグルタチオンCトナー200ML ＋ 白玉グルタチオンC美容液30ML - 輝く美肌へ導く！</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F256" t="n">
+        <v>7013</v>
+      </c>
+      <c r="G256" t="n">
+        <v>0</v>
+      </c>
+      <c r="H256" t="b">
+        <v>0</v>
+      </c>
+      <c r="I256" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J256" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1146499598</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>1207091316</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>manmulsang</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>レチノールスーパーバウンスセラム 20ml＋15ml 企画セット 初めてのレチノールケア 昼夜使いやすい 美容液 メイク前 なめらか肌印象 韓国コスメ スポイトタイプ 水分感 クリーム前 スキンケア</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>アイオペ</t>
+        </is>
+      </c>
+      <c r="F257" t="n">
+        <v>5324</v>
+      </c>
+      <c r="G257" t="n">
+        <v>0</v>
+      </c>
+      <c r="H257" t="b">
+        <v>0</v>
+      </c>
+      <c r="I257" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J257" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207091316</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>1210268653</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>SCH</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>アゼライン酸ナイアシンアミドクリアトナー, 250ml</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F258" t="n">
+        <v>2420</v>
+      </c>
+      <c r="G258" t="n">
+        <v>0</v>
+      </c>
+      <c r="H258" t="b">
+        <v>0</v>
+      </c>
+      <c r="I258" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J258" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210268653</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>1204022304</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>SCH</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>ステイフレッシュトーンアップサンクリーム パープル, 50ml</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>Beauty of Joseon</t>
+        </is>
+      </c>
+      <c r="F259" t="n">
+        <v>2526</v>
+      </c>
+      <c r="G259" t="n">
+        <v>0</v>
+      </c>
+      <c r="H259" t="b">
+        <v>0</v>
+      </c>
+      <c r="I259" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J259" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204022304</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>1201368379</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>SCH</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>THEVITAレチナールショットタイトニングブースター 15ml</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F260" t="n">
+        <v>2140</v>
+      </c>
+      <c r="G260" t="n">
+        <v>0</v>
+      </c>
+      <c r="H260" t="b">
+        <v>0</v>
+      </c>
+      <c r="I260" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J260" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201368379</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>1106986645</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>TeaTime</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>【2個セット】シークレット マルチバーム 7g×2 発酵保湿スティック 韓国コスメ 携帯用 高保湿 ツヤ肌 ハリケア</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>sum37</t>
+        </is>
+      </c>
+      <c r="F261" t="n">
+        <v>4399</v>
+      </c>
+      <c r="G261" t="n">
+        <v>0</v>
+      </c>
+      <c r="H261" t="b">
+        <v>0</v>
+      </c>
+      <c r="I261" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J261" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1106986645</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>1060687901</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>gugumile</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>Uriage ユリアージュ バリアダム シカクリーム 40ml [製造国 フランス]</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>Uriage</t>
+        </is>
+      </c>
+      <c r="F262" t="n">
+        <v>3156</v>
+      </c>
+      <c r="G262" t="n">
+        <v>0</v>
+      </c>
+      <c r="H262" t="b">
+        <v>0</v>
+      </c>
+      <c r="I262" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J262" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1060687901</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>1059767256</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>gugumile</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>ROUND LAB ラウンドラップ 1025 独島 クレンザー 150ml</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F263" t="n">
+        <v>1680</v>
+      </c>
+      <c r="G263" t="n">
+        <v>1</v>
+      </c>
+      <c r="H263" t="b">
+        <v>0</v>
+      </c>
+      <c r="I263" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J263" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1059767256</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>1210577063</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>wingkone</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>【正規品】【NEW】【脱色/染め】 眉毛脱色 イージーブロウトーンチェンジャー 5回分 / イージーブロウムードチェンジャー 5回分 / アイブロウ / 韓国コスメ / 眉毛</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>コスノリ</t>
+        </is>
+      </c>
+      <c r="F264" t="n">
+        <v>1810</v>
+      </c>
+      <c r="G264" t="n">
+        <v>3</v>
+      </c>
+      <c r="H264" t="b">
+        <v>0</v>
+      </c>
+      <c r="I264" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J264" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210577063</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J251"/>
+  <autoFilter ref="A1:J264"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 57, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$264</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$275</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J264"/>
+  <dimension ref="A1:J275"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11279,8 +11279,459 @@
         </is>
       </c>
     </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>1152724729</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>MAYSHOP</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>ドクダミ77%スージングトナー, 250ml</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F265" t="n">
+        <v>1760</v>
+      </c>
+      <c r="G265" t="n">
+        <v>0</v>
+      </c>
+      <c r="H265" t="b">
+        <v>0</v>
+      </c>
+      <c r="I265" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J265" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1152724729</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>1191147953</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>MAYSHOP</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>ピュア ボディミスト ベビーパウダーの香り 128ml 2個</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>Kundal</t>
+        </is>
+      </c>
+      <c r="F266" t="n">
+        <v>1867</v>
+      </c>
+      <c r="G266" t="n">
+        <v>1</v>
+      </c>
+      <c r="H266" t="b">
+        <v>0</v>
+      </c>
+      <c r="I266" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J266" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191147953</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>1185851789</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>MAYSHOP</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>[1+1] レッド ラクト コラーゲン ラッピング マスクパック 70ml *2 + ブラシ</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F267" t="n">
+        <v>3587</v>
+      </c>
+      <c r="G267" t="n">
+        <v>1</v>
+      </c>
+      <c r="H267" t="b">
+        <v>0</v>
+      </c>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J267" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1185851789</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>1152724831</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>MAYSHOP</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>6番 爆睡マスクパックセラム50ml</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F268" t="n">
+        <v>2360</v>
+      </c>
+      <c r="G268" t="n">
+        <v>0</v>
+      </c>
+      <c r="H268" t="b">
+        <v>0</v>
+      </c>
+      <c r="I268" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J268" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1152724831</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>1209321763</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>5708</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>【GIFT】[プレミアムPDRN セット] (トナー/アンプル/クリーム) 最大3種フル構成+パック1枚贈呈/MEDICUBE</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F269" t="n">
+        <v>4300</v>
+      </c>
+      <c r="G269" t="n">
+        <v>0</v>
+      </c>
+      <c r="H269" t="b">
+        <v>0</v>
+      </c>
+      <c r="I269" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J269" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209321763</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>1211863823</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>5708</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>【選べる】リードルショット 100 / 300 / 700 + AHCアイクリーム本品付き (韓国大人気スキンケアセット)</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F270" t="n">
+        <v>2700</v>
+      </c>
+      <c r="G270" t="n">
+        <v>0</v>
+      </c>
+      <c r="H270" t="b">
+        <v>0</v>
+      </c>
+      <c r="I270" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J270" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211863823</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>1209714705</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>5708</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>【GIFT】PDRNヒアルロン酸カプセル100セラム, 30ml[プレミアムPDRN セット]ピンクPDRN 基礎セット (アンプル)</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F271" t="n">
+        <v>3500</v>
+      </c>
+      <c r="G271" t="n">
+        <v>0</v>
+      </c>
+      <c r="H271" t="b">
+        <v>0</v>
+      </c>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J271" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209714705</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>1209150921</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>5708</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>【GIFT】【選べる1+1】 自分好みに選ぶ セラム4種セット / 桃セラム ドクダミ ナイアシン PDRN 水光肌 ハリ 弾力 ケア</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F272" t="n">
+        <v>2800</v>
+      </c>
+      <c r="G272" t="n">
+        <v>0</v>
+      </c>
+      <c r="H272" t="b">
+        <v>0</v>
+      </c>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J272" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209150921</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>1191691008</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>HANAK-BEAUTYSHOP</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>[1位サンベース]ウォータフルビタカプセルエイジングケアサンクリーム, 50ml/日焼け止め 日焼けどめ ビタミンC 美白 低刺激 紫外線対策 UVカット 日焼け対策 韓国コスメ 化粧下地 プライマー</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F273" t="n">
+        <v>4532</v>
+      </c>
+      <c r="G273" t="n">
+        <v>0</v>
+      </c>
+      <c r="H273" t="b">
+        <v>0</v>
+      </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J273" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191691008</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>1168503263</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>modepick</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>ハンドウォッシュ LUCIEN CARR 450ml 正規品 ハンドソープ おしゃれな香り 韓国コスメ 韓国人気アイテム</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>GRANHAND</t>
+        </is>
+      </c>
+      <c r="F274" t="n">
+        <v>3630</v>
+      </c>
+      <c r="G274" t="n">
+        <v>0</v>
+      </c>
+      <c r="H274" t="b">
+        <v>0</v>
+      </c>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J274" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168503263</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>1194081987</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>modepick</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>【SEVENTEEN ミンギュ着用】半袖Tシャツ マルチーズ グラフィック プリント YK23HSTS12-1 韓国ファッション オーバーサイズ ユニセックス</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>WaiKei</t>
+        </is>
+      </c>
+      <c r="F275" t="n">
+        <v>4260</v>
+      </c>
+      <c r="G275" t="n">
+        <v>1</v>
+      </c>
+      <c r="H275" t="b">
+        <v>0</v>
+      </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J275" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194081987</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J264"/>
+  <autoFilter ref="A1:J275"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 60, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$275</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$284</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J275"/>
+  <dimension ref="A1:J284"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11730,8 +11730,377 @@
         </is>
       </c>
     </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>1199411031</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>Seoullys</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>[2+2] 白樺 水分 日焼け止めスプレー, 100ml 4ea(SPF 50 + PA ++++)</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F276" t="n">
+        <v>6007</v>
+      </c>
+      <c r="G276" t="n">
+        <v>0</v>
+      </c>
+      <c r="H276" t="b">
+        <v>0</v>
+      </c>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J276" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199411031</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>1149907926</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>sssemibeauty</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>ブラックシュガーパーフェクトファーストセラム 150ml</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>スキンフード</t>
+        </is>
+      </c>
+      <c r="F277" t="n">
+        <v>2299</v>
+      </c>
+      <c r="G277" t="n">
+        <v>0</v>
+      </c>
+      <c r="H277" t="b">
+        <v>0</v>
+      </c>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J277" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1149907926</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>1172085888</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>sssemibeauty</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>フルフィットプロポリスライトアンプル, 30ml</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F278" t="n">
+        <v>2337</v>
+      </c>
+      <c r="G278" t="n">
+        <v>0</v>
+      </c>
+      <c r="H278" t="b">
+        <v>0</v>
+      </c>
+      <c r="I278" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J278" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172085888</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>1172312020</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>hokkorikorea</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>【SALE】【毛穴ケア】PDRN毛穴弾力パッド 100枚 ハリ感 キメ整う エイジングケア ツヤ肌 角質ケア うるおい 人気 韓国コスメ 大容量 毎日ケア 時短 敏感肌OK 透明感 キメケア 保湿</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>メディヒール</t>
+        </is>
+      </c>
+      <c r="F279" t="n">
+        <v>3006</v>
+      </c>
+      <c r="G279" t="n">
+        <v>0</v>
+      </c>
+      <c r="H279" t="b">
+        <v>0</v>
+      </c>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J279" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172312020</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>1118545938</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>ksco</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>センテラライトクレンジングオイル, 200ml</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F280" t="n">
+        <v>2210</v>
+      </c>
+      <c r="G280" t="n">
+        <v>0</v>
+      </c>
+      <c r="H280" t="b">
+        <v>0</v>
+      </c>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J280" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1118545938</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>1199379098</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>ksco</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>ゼリーセラムミスト, 50ml</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>Biodance</t>
+        </is>
+      </c>
+      <c r="F281" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G281" t="n">
+        <v>0</v>
+      </c>
+      <c r="H281" t="b">
+        <v>0</v>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J281" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199379098</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>1163668247</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>ksco</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>シューマジゴールド糸ラッピングマスク, 90g</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>メディテラピー</t>
+        </is>
+      </c>
+      <c r="F282" t="n">
+        <v>5580</v>
+      </c>
+      <c r="G282" t="n">
+        <v>0</v>
+      </c>
+      <c r="H282" t="b">
+        <v>0</v>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J282" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1163668247</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>1169199883</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>COCO-Beauty</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>【正規品】エッセンシャルムルマイクロフィッティングミスト, 55ml</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>ジョンセンムル</t>
+        </is>
+      </c>
+      <c r="F283" t="n">
+        <v>1808</v>
+      </c>
+      <c r="G283" t="n">
+        <v>2</v>
+      </c>
+      <c r="H283" t="b">
+        <v>0</v>
+      </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J283" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1169199883</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>1170526082</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>COCO-Beauty</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>【正規品】セラミッククリーム, 100ml</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>ティルティル</t>
+        </is>
+      </c>
+      <c r="F284" t="n">
+        <v>5287</v>
+      </c>
+      <c r="G284" t="n">
+        <v>0</v>
+      </c>
+      <c r="H284" t="b">
+        <v>0</v>
+      </c>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J284" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1170526082</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J275"/>
+  <autoFilter ref="A1:J284"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 63, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$284</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$297</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J284"/>
+  <dimension ref="A1:J297"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12099,8 +12099,541 @@
         </is>
       </c>
     </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>1196192763</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>HLINEINTERNATIONAL</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>デオドラント ロールオン 50ml</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>イソップ</t>
+        </is>
+      </c>
+      <c r="F285" t="n">
+        <v>5800</v>
+      </c>
+      <c r="G285" t="n">
+        <v>0</v>
+      </c>
+      <c r="H285" t="b">
+        <v>0</v>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J285" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196192763</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>1085260269</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>HLINEINTERNATIONAL</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>アーモンドミルク ボディモイスチャライザー 250ml</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>ロクシタン</t>
+        </is>
+      </c>
+      <c r="F286" t="n">
+        <v>5580</v>
+      </c>
+      <c r="G286" t="n">
+        <v>0</v>
+      </c>
+      <c r="H286" t="b">
+        <v>0</v>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J286" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1085260269</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>1081721110</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>HLINEINTERNATIONAL</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>ボディ フィット 200ml</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>クラランス</t>
+        </is>
+      </c>
+      <c r="F287" t="n">
+        <v>6820</v>
+      </c>
+      <c r="G287" t="n">
+        <v>1</v>
+      </c>
+      <c r="H287" t="b">
+        <v>0</v>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J287" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1081721110</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>1212749170</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>easyworld</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>restore pha facial r 200ml</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>ネオストラータ</t>
+        </is>
+      </c>
+      <c r="F288" t="n">
+        <v>4920</v>
+      </c>
+      <c r="G288" t="n">
+        <v>0</v>
+      </c>
+      <c r="H288" t="b">
+        <v>0</v>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J288" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212749170</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>1122993259</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>easyworld</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>ジェントル クレンジング ジェル 500ml</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>ムステラ</t>
+        </is>
+      </c>
+      <c r="F289" t="n">
+        <v>1890</v>
+      </c>
+      <c r="G289" t="n">
+        <v>1</v>
+      </c>
+      <c r="H289" t="b">
+        <v>0</v>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J289" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1122993259</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>1205868858</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>easyworld</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>パーフェクトuv サンスクリーン スキンケアジェル spf50 90g</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>アネッサ</t>
+        </is>
+      </c>
+      <c r="F290" t="n">
+        <v>3780</v>
+      </c>
+      <c r="G290" t="n">
+        <v>0</v>
+      </c>
+      <c r="H290" t="b">
+        <v>0</v>
+      </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J290" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205868858</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>1023263418</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>SWNO1</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>【即納】【正規品】【最新製造日】 1個目 2個目 パースピレックス オリジナル デオドラント ロールオン 脇汗 ワキガ 制汗剤 20ml</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>パースピレックス</t>
+        </is>
+      </c>
+      <c r="F291" t="n">
+        <v>2230</v>
+      </c>
+      <c r="G291" t="n">
+        <v>0</v>
+      </c>
+      <c r="H291" t="b">
+        <v>0</v>
+      </c>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J291" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1023263418</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>1016471395</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>SWNO1</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>【即納】【正規品】【最新製造日】 1個目 パースピレックス ストロング デオドラント ロールオン 脇汗 ワキガ 制汗剤 20ml</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>パースピレックス</t>
+        </is>
+      </c>
+      <c r="F292" t="n">
+        <v>2230</v>
+      </c>
+      <c r="G292" t="n">
+        <v>0</v>
+      </c>
+      <c r="H292" t="b">
+        <v>0</v>
+      </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J292" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1016471395</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>1200694196</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>SWNO1</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>【即納】【正規品】【最新製造日】 1個目 2個目 パースピレックス デオドラント ロールオン 脇汗 ワキガ 制汗剤 20ml</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>パースピレックス</t>
+        </is>
+      </c>
+      <c r="F293" t="n">
+        <v>3660</v>
+      </c>
+      <c r="G293" t="n">
+        <v>1</v>
+      </c>
+      <c r="H293" t="b">
+        <v>0</v>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J293" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200694196</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>1213379918</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>KOOKA</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>エルセブ トータルリペア 5 インスタントミラクルヘアパック400ml 2個</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>LOREAL PARIS</t>
+        </is>
+      </c>
+      <c r="F294" t="n">
+        <v>4444</v>
+      </c>
+      <c r="G294" t="n">
+        <v>0</v>
+      </c>
+      <c r="H294" t="b">
+        <v>0</v>
+      </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J294" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213379918</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>1212659970</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>KOOKA</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>サロン10プロテインシャンプーダメージヘア用990ml1個</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>ミジャンセン</t>
+        </is>
+      </c>
+      <c r="F295" t="n">
+        <v>3018</v>
+      </c>
+      <c r="G295" t="n">
+        <v>0</v>
+      </c>
+      <c r="H295" t="b">
+        <v>0</v>
+      </c>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J295" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212659970</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>1212659429</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>KOOKA</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>サロン10 プロテイントリートメント ダメージヘア用250ml 3個</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>ミジャンセン</t>
+        </is>
+      </c>
+      <c r="F296" t="n">
+        <v>3956</v>
+      </c>
+      <c r="G296" t="n">
+        <v>0</v>
+      </c>
+      <c r="H296" t="b">
+        <v>0</v>
+      </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J296" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212659429</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>1212659125</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>KOOKA</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>サロン10プロテインヘアトリートメント極ダメージヘア用250ml1個</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>ミジャンセン</t>
+        </is>
+      </c>
+      <c r="F297" t="n">
+        <v>1806</v>
+      </c>
+      <c r="G297" t="n">
+        <v>0</v>
+      </c>
+      <c r="H297" t="b">
+        <v>0</v>
+      </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J297" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212659125</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J284"/>
+  <autoFilter ref="A1:J297"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 66, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$297</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$309</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J297"/>
+  <dimension ref="A1:J309"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12632,8 +12632,500 @@
         </is>
       </c>
     </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>1194458592</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>kiseki-trend</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>資生堂 サブリミック ワンダーシールド h レフィル 110mL 詰め替え用 洗い流さないトリートメント ヘアプロテクター ツヤケア 美容室専売品</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>資生堂</t>
+        </is>
+      </c>
+      <c r="F298" t="n">
+        <v>2032</v>
+      </c>
+      <c r="G298" t="n">
+        <v>0</v>
+      </c>
+      <c r="H298" t="b">
+        <v>0</v>
+      </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J298" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194458592</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>1173903686</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>bettysbeauty</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>レプリカ ハンドクリーム レイジーサンデー モーニング 50ml/1.6fl.oz.</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>メゾンマルジェラ</t>
+        </is>
+      </c>
+      <c r="F299" t="n">
+        <v>4191</v>
+      </c>
+      <c r="G299" t="n">
+        <v>1</v>
+      </c>
+      <c r="H299" t="b">
+        <v>0</v>
+      </c>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J299" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1173903686</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>638382548</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>bettysbeauty</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>ヴァーベナ ボディローション 250ml</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>ロクシタン</t>
+        </is>
+      </c>
+      <c r="F300" t="n">
+        <v>3135</v>
+      </c>
+      <c r="G300" t="n">
+        <v>2</v>
+      </c>
+      <c r="H300" t="b">
+        <v>0</v>
+      </c>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J300" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=638382548</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>1203744619</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>treasurebeauty</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>ベルベット クレンジング ミルク 200ml x 2 お得な2個セット</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>クラランス</t>
+        </is>
+      </c>
+      <c r="F301" t="n">
+        <v>6230</v>
+      </c>
+      <c r="G301" t="n">
+        <v>0</v>
+      </c>
+      <c r="H301" t="b">
+        <v>0</v>
+      </c>
+      <c r="I301" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J301" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203744619</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>1173946856</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>treasurebeauty</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>デイリーPD 50ml/1.7fl.oz.</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>ZO SKIN</t>
+        </is>
+      </c>
+      <c r="F302" t="n">
+        <v>21465</v>
+      </c>
+      <c r="G302" t="n">
+        <v>0</v>
+      </c>
+      <c r="H302" t="b">
+        <v>0</v>
+      </c>
+      <c r="I302" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J302" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1173946856</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>1154827017</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>treasurebeauty</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>メン ハード バーム 60g</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>アリミノ</t>
+        </is>
+      </c>
+      <c r="F303" t="n">
+        <v>1979</v>
+      </c>
+      <c r="G303" t="n">
+        <v>0</v>
+      </c>
+      <c r="H303" t="b">
+        <v>0</v>
+      </c>
+      <c r="I303" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J303" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1154827017</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>1162075812</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>goingover</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>JEANNE ARTHES(ジャンヌ・アルテス) ジャンヌ・アルテス スルタン オードパルファム 1</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>ジャンヌアルテス</t>
+        </is>
+      </c>
+      <c r="F304" t="n">
+        <v>4144</v>
+      </c>
+      <c r="G304" t="n">
+        <v>3</v>
+      </c>
+      <c r="H304" t="b">
+        <v>0</v>
+      </c>
+      <c r="I304" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J304" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1162075812</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>1163081544</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>goingover</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>ラ・カスタ アロマエステ ヘアローション スムース リフィル(詰め替え用) *髪用ローション*</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>ラ・カスタ</t>
+        </is>
+      </c>
+      <c r="F305" t="n">
+        <v>2312</v>
+      </c>
+      <c r="G305" t="n">
+        <v>1</v>
+      </c>
+      <c r="H305" t="b">
+        <v>0</v>
+      </c>
+      <c r="I305" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J305" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1163081544</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>1213367912</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>spklbzr</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>ルベル イオ クリーム メルトリペア ヘアトリートメント 200g 赤 684</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>イオ</t>
+        </is>
+      </c>
+      <c r="F306" t="n">
+        <v>1755</v>
+      </c>
+      <c r="G306" t="n">
+        <v>0</v>
+      </c>
+      <c r="H306" t="b">
+        <v>0</v>
+      </c>
+      <c r="I306" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J306" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213367912</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>1185299459</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>nokotan</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>ululis ウルリス VITA.C 乾燥・パサつきケア の ビタシー ウォーターコンク EXリペア ヘアオイル 100mL</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>ululis</t>
+        </is>
+      </c>
+      <c r="F307" t="n">
+        <v>1894</v>
+      </c>
+      <c r="G307" t="n">
+        <v>3</v>
+      </c>
+      <c r="H307" t="b">
+        <v>0</v>
+      </c>
+      <c r="I307" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J307" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1185299459</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>1129386950</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>--HAPPYBUNNY--</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>GIVENCHY【大人気】ジバンシイ プリズム リーブル ミニパウダー No0/No1/No2/No3/No4 ジバンシイ プリズム リーブル PRISME LIBRE ルース パウダー</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>ナンバースリー</t>
+        </is>
+      </c>
+      <c r="F308" t="n">
+        <v>7441</v>
+      </c>
+      <c r="G308" t="n">
+        <v>0</v>
+      </c>
+      <c r="H308" t="b">
+        <v>0</v>
+      </c>
+      <c r="I308" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J308" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1129386950</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>1114825811</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>--HAPPYBUNNY--</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>【大人気】拭き取りトナーパッド 化粧水（プランプハニー/スージンググリーン/ビタギビング）</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>ByUR</t>
+        </is>
+      </c>
+      <c r="F309" t="n">
+        <v>4060</v>
+      </c>
+      <c r="G309" t="n">
+        <v>0</v>
+      </c>
+      <c r="H309" t="b">
+        <v>0</v>
+      </c>
+      <c r="I309" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J309" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1114825811</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J297"/>
+  <autoFilter ref="A1:J309"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 69, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$309</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$321</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J309"/>
+  <dimension ref="A1:J321"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13124,8 +13124,500 @@
         </is>
       </c>
     </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>1155003250</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>royalshop</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>つや米 トーンアップ 水分 サンクリーム 日焼け止め 化粧下地 UVカット SPF50+ PA++++ 韓国コスメ [ロイヤルショップ] 100mL</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>シンムルナラ</t>
+        </is>
+      </c>
+      <c r="F310" t="n">
+        <v>3413</v>
+      </c>
+      <c r="G310" t="n">
+        <v>0</v>
+      </c>
+      <c r="H310" t="b">
+        <v>0</v>
+      </c>
+      <c r="I310" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J310" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1155003250</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>1157009011</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>royalshop</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>エアライン KF94 黄砂・飛沫対策 3Dマスク 大型サイズ 韓国マスク 100枚セット（25枚×4袋）［ホワイト/ブラック］</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>URBANWIZ</t>
+        </is>
+      </c>
+      <c r="F311" t="n">
+        <v>2477</v>
+      </c>
+      <c r="G311" t="n">
+        <v>0</v>
+      </c>
+      <c r="H311" t="b">
+        <v>0</v>
+      </c>
+      <c r="I311" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J311" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1157009011</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>1193058658</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>akiaki</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>レッドイッチ ケアクリーム 330ml（20mlオイル付き）</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>イリユン</t>
+        </is>
+      </c>
+      <c r="F312" t="n">
+        <v>3500</v>
+      </c>
+      <c r="G312" t="n">
+        <v>0</v>
+      </c>
+      <c r="H312" t="b">
+        <v>0</v>
+      </c>
+      <c r="I312" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J312" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193058658</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>1212341086</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>akiaki</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>【BLACKPINK ジェニー PICK】【NEW】ヴァセリン グルタヒヤ セラム ボディローション 3種 300ml</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>ヴァセリン</t>
+        </is>
+      </c>
+      <c r="F313" t="n">
+        <v>1850</v>
+      </c>
+      <c r="G313" t="n">
+        <v>0</v>
+      </c>
+      <c r="H313" t="b">
+        <v>0</v>
+      </c>
+      <c r="I313" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J313" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212341086</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>1190762638</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>pureco</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>Wonjungyo (ウォンジョンヨ) モイスト アップ レディ スキン パック 50枚</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>ウォンジョンヨ</t>
+        </is>
+      </c>
+      <c r="F314" t="n">
+        <v>1689</v>
+      </c>
+      <c r="G314" t="n">
+        <v>2</v>
+      </c>
+      <c r="H314" t="b">
+        <v>0</v>
+      </c>
+      <c r="I314" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J314" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190762638</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>1213602528</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>pureco</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>コーセー コスメデコルテ ルース パウダー 6g #02 lucent lilac 【限定】</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>Kose</t>
+        </is>
+      </c>
+      <c r="F315" t="n">
+        <v>3207</v>
+      </c>
+      <c r="G315" t="n">
+        <v>0</v>
+      </c>
+      <c r="H315" t="b">
+        <v>0</v>
+      </c>
+      <c r="I315" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J315" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213602528</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>1154113008</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>myroom</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>【プレステージEXキット贈呈】 プリステージEXトナー 130ml</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>エルツティン</t>
+        </is>
+      </c>
+      <c r="F316" t="n">
+        <v>9490</v>
+      </c>
+      <c r="G316" t="n">
+        <v>1</v>
+      </c>
+      <c r="H316" t="b">
+        <v>0</v>
+      </c>
+      <c r="I316" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J316" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1154113008</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>1139814745</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>vip_s</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>ティルティールオフザサンエアムース/ 40ml/ 1個</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>ティルティル</t>
+        </is>
+      </c>
+      <c r="F317" t="n">
+        <v>2247</v>
+      </c>
+      <c r="G317" t="n">
+        <v>0</v>
+      </c>
+      <c r="H317" t="b">
+        <v>0</v>
+      </c>
+      <c r="I317" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J317" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1139814745</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>1151569871</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>vip_s</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>デイリー アンチヘアロス タンパク質 トリートメント 500ml</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>ダシュ</t>
+        </is>
+      </c>
+      <c r="F318" t="n">
+        <v>3048</v>
+      </c>
+      <c r="G318" t="n">
+        <v>0</v>
+      </c>
+      <c r="H318" t="b">
+        <v>0</v>
+      </c>
+      <c r="I318" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J318" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1151569871</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>1138225289</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>dreamus</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>シグネチャーパルファム, 50ml, 1個</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>FORMENT</t>
+        </is>
+      </c>
+      <c r="F319" t="n">
+        <v>5517</v>
+      </c>
+      <c r="G319" t="n">
+        <v>0</v>
+      </c>
+      <c r="H319" t="b">
+        <v>0</v>
+      </c>
+      <c r="I319" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J319" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1138225289</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>1139807140</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>gpgp</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>パルファムボディウォッシュ/ 500ml/ 2個</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>ミルクバオバブ</t>
+        </is>
+      </c>
+      <c r="F320" t="n">
+        <v>3492</v>
+      </c>
+      <c r="G320" t="n">
+        <v>0</v>
+      </c>
+      <c r="H320" t="b">
+        <v>0</v>
+      </c>
+      <c r="I320" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J320" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1139807140</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>1139805675</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>gpgp</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>オードパルファム(07シュガーフローラル)/ 25ml/ 1個</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>After blow</t>
+        </is>
+      </c>
+      <c r="F321" t="n">
+        <v>5505</v>
+      </c>
+      <c r="G321" t="n">
+        <v>1</v>
+      </c>
+      <c r="H321" t="b">
+        <v>0</v>
+      </c>
+      <c r="I321" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J321" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1139805675</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J309"/>
+  <autoFilter ref="A1:J321"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 72, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$321</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$333</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J321"/>
+  <dimension ref="A1:J333"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13616,8 +13616,500 @@
         </is>
       </c>
     </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>1106939117</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>HARUMAL__</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>【正規品】[ユーチューバー おすすめアイテム] ホワイトトリュフ ファーストスプレー ミストセラム 100ml</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F322" t="n">
+        <v>3057</v>
+      </c>
+      <c r="G322" t="n">
+        <v>0</v>
+      </c>
+      <c r="H322" t="b">
+        <v>0</v>
+      </c>
+      <c r="I322" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J322" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1106939117</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>1205747267</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>kshopofficial</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>アクニDr.ファーストブラックディープクレンジングフォーム 75ml</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>アイソイ</t>
+        </is>
+      </c>
+      <c r="F323" t="n">
+        <v>2286</v>
+      </c>
+      <c r="G323" t="n">
+        <v>0</v>
+      </c>
+      <c r="H323" t="b">
+        <v>0</v>
+      </c>
+      <c r="I323" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J323" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205747267</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>1205744981</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>kshopofficial</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>シカカーミングパウダーウォッシュ 50g</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>TOCOBO</t>
+        </is>
+      </c>
+      <c r="F324" t="n">
+        <v>2200</v>
+      </c>
+      <c r="G324" t="n">
+        <v>0</v>
+      </c>
+      <c r="H324" t="b">
+        <v>0</v>
+      </c>
+      <c r="I324" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J324" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205744981</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>1210161140</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>kshopofficial</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>3番キメブースター時短バブルパック 90ml</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F325" t="n">
+        <v>2496</v>
+      </c>
+      <c r="G325" t="n">
+        <v>0</v>
+      </c>
+      <c r="H325" t="b">
+        <v>0</v>
+      </c>
+      <c r="I325" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J325" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210161140</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>1209641531</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>angelskinmall</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>[1+]NEWサイトカインブースタープロ 70ml＋70ml</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>Refilled</t>
+        </is>
+      </c>
+      <c r="F326" t="n">
+        <v>5039</v>
+      </c>
+      <c r="G326" t="n">
+        <v>0</v>
+      </c>
+      <c r="H326" t="b">
+        <v>0</v>
+      </c>
+      <c r="I326" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J326" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209641531</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>1209148971</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>angelskinmall</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>【韓国正規品/NEW】Gureum o de perfume EDP 50ml</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>BiBiANG</t>
+        </is>
+      </c>
+      <c r="F327" t="n">
+        <v>11419</v>
+      </c>
+      <c r="G327" t="n">
+        <v>0</v>
+      </c>
+      <c r="H327" t="b">
+        <v>0</v>
+      </c>
+      <c r="I327" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J327" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209148971</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>1206526891</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>angelskinmall</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>[NEW]エアロクーリングシャンプー 400ml＋70ml / -5.2度急速冷却</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>Dr.FORHAIR</t>
+        </is>
+      </c>
+      <c r="F328" t="n">
+        <v>3859</v>
+      </c>
+      <c r="G328" t="n">
+        <v>0</v>
+      </c>
+      <c r="H328" t="b">
+        <v>0</v>
+      </c>
+      <c r="I328" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J328" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206526891</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>1196819316</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>ktrendmall</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>グルタチオンビタシートマスク デイリーピック 30枚</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>アビブ</t>
+        </is>
+      </c>
+      <c r="F329" t="n">
+        <v>2734</v>
+      </c>
+      <c r="G329" t="n">
+        <v>0</v>
+      </c>
+      <c r="H329" t="b">
+        <v>0</v>
+      </c>
+      <c r="I329" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J329" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196819316</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>1182043662</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>ktrendmall</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>エクソソームシカ ツボクサ鎮静クリーム 50ml</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F330" t="n">
+        <v>3290</v>
+      </c>
+      <c r="G330" t="n">
+        <v>0</v>
+      </c>
+      <c r="H330" t="b">
+        <v>0</v>
+      </c>
+      <c r="I330" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J330" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1182043662</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>1197915395</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>GHMKOREA</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>ボディウォッシュ 保湿 敏感肌 乾燥肌用 532ml×2本 大容量 ポンプ式 デイリーモイスチャライジング</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>アビーノ</t>
+        </is>
+      </c>
+      <c r="F331" t="n">
+        <v>4990</v>
+      </c>
+      <c r="G331" t="n">
+        <v>0</v>
+      </c>
+      <c r="H331" t="b">
+        <v>0</v>
+      </c>
+      <c r="I331" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J331" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197915395</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>1208263731</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>GHMKOREA</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>パフューム シャルマン ムスク シャンプー＆コンディショナーセット 600ml×3本（シャンプー2本＋コンディショナー1本）フローラルムスクの香り 韓国人気ヘアケア</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>ケラシス</t>
+        </is>
+      </c>
+      <c r="F332" t="n">
+        <v>4091</v>
+      </c>
+      <c r="G332" t="n">
+        <v>0</v>
+      </c>
+      <c r="H332" t="b">
+        <v>0</v>
+      </c>
+      <c r="I332" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J332" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208263731</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>1199673717</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>GHMKOREA</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>Nature Skin フェイスマスク 100枚セット シートマスク 100枚 大容量 フェイスパック 16種類から選べる 保湿ケア デイリー スキンケア 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>FOODAHOLIC</t>
+        </is>
+      </c>
+      <c r="F333" t="n">
+        <v>4378</v>
+      </c>
+      <c r="G333" t="n">
+        <v>0</v>
+      </c>
+      <c r="H333" t="b">
+        <v>0</v>
+      </c>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J333" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199673717</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J321"/>
+  <autoFilter ref="A1:J333"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 75, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$333</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$350</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J333"/>
+  <dimension ref="A1:J350"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14108,8 +14108,705 @@
         </is>
       </c>
     </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>1201633330</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>kurashiben</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>ナノバブル バブルエッセンス 95ml NANO BUBBLES 泡タイプ美容液 バブルエッセンス 乾燥ケア REVI 基礎化粧品 フェイシャルケア ホームケア ホームエステ</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>REVI</t>
+        </is>
+      </c>
+      <c r="F334" t="n">
+        <v>4480</v>
+      </c>
+      <c r="G334" t="n">
+        <v>0</v>
+      </c>
+      <c r="H334" t="b">
+        <v>0</v>
+      </c>
+      <c r="I334" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J334" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201633330</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>1203041614</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>mayjoy</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>ドンア ノスカルナジェル ニキビ跡手術痕ケロイド赤褐色色素沈着のあるニキビ跡に／韓国・ソウル産</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>東亜製薬</t>
+        </is>
+      </c>
+      <c r="F335" t="n">
+        <v>1590</v>
+      </c>
+      <c r="G335" t="n">
+        <v>0</v>
+      </c>
+      <c r="H335" t="b">
+        <v>0</v>
+      </c>
+      <c r="I335" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J335" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203041614</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>1209154400</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>AnchorBlue</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>[密着ハリツヤ/5枚入] コラーゲン 100 メルティング シート マスク 2.5g x 5枚 / 濃密 潤い 水分 パッチ 弾力 肌キメ ス킨케어 高保湿 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F336" t="n">
+        <v>7376</v>
+      </c>
+      <c r="G336" t="n">
+        <v>0</v>
+      </c>
+      <c r="H336" t="b">
+        <v>0</v>
+      </c>
+      <c r="I336" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J336" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209154400</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>1208338165</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>AnchorBlue</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>[サロン級ホームケア] エクストリーム ダメージ クリニック ヘア アンプル 10ml 9個入り / 傷んだ髪 高濃縮 補修 保湿 ツヤ髪 トリートメント 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>ケラシス</t>
+        </is>
+      </c>
+      <c r="F337" t="n">
+        <v>3818</v>
+      </c>
+      <c r="G337" t="n">
+        <v>0</v>
+      </c>
+      <c r="H337" t="b">
+        <v>0</v>
+      </c>
+      <c r="I337" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J337" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208338165</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>1193433365</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>pharmesthetic</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>【公式】 コナピディル フィクシカ CONAPIDIL Fixcica 13g</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>CONAPIDIL</t>
+        </is>
+      </c>
+      <c r="F338" t="n">
+        <v>7700</v>
+      </c>
+      <c r="G338" t="n">
+        <v>3</v>
+      </c>
+      <c r="H338" t="b">
+        <v>0</v>
+      </c>
+      <c r="I338" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J338" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193433365</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>1193433355</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>pharmesthetic</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>【公式】 コナピディル グリーンボクシン CONAPIDIL Greenboxin 150ml</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>CONAPIDIL</t>
+        </is>
+      </c>
+      <c r="F339" t="n">
+        <v>9200</v>
+      </c>
+      <c r="G339" t="n">
+        <v>2</v>
+      </c>
+      <c r="H339" t="b">
+        <v>0</v>
+      </c>
+      <c r="I339" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J339" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193433355</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>1193433366</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>pharmesthetic</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>【公式】 コナピディル フィニッシュローション CONAPIDIL Finish Lotion 20g</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>CONAPIDIL</t>
+        </is>
+      </c>
+      <c r="F340" t="n">
+        <v>9800</v>
+      </c>
+      <c r="G340" t="n">
+        <v>1</v>
+      </c>
+      <c r="H340" t="b">
+        <v>0</v>
+      </c>
+      <c r="I340" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J340" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193433366</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>1193433359</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>pharmesthetic</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>【公式】 アクセンダ ルティナー aXENDA Routiner 15ml</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>aXENDA</t>
+        </is>
+      </c>
+      <c r="F341" t="n">
+        <v>9100</v>
+      </c>
+      <c r="G341" t="n">
+        <v>2</v>
+      </c>
+      <c r="H341" t="b">
+        <v>0</v>
+      </c>
+      <c r="I341" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J341" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193433359</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>1210385244</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>pharma21</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>【日本メーカ―公式】ファーマ21 モイストリペアヘアマスク 乾燥ケア しっとり保湿 髪質ケア パサつき・広がり対策 サロン品質 ヘアトリートメント ヘアパック 230g</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>PHARMA21</t>
+        </is>
+      </c>
+      <c r="F342" t="n">
+        <v>2970</v>
+      </c>
+      <c r="G342" t="n">
+        <v>0</v>
+      </c>
+      <c r="H342" t="b">
+        <v>0</v>
+      </c>
+      <c r="I342" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J342" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210385244</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>1210384486</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>pharma21</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>【日本メーカー公式】ファーマ21 ラグジュリアスリペアヘアマスク 年齢髪ケア 髪質改善 ダメージ補修 美容液成分配合 しっとりまとまる髪 サロン品質 ヘアトリートメント ヘアパック 230g</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>PHARMA21</t>
+        </is>
+      </c>
+      <c r="F343" t="n">
+        <v>2970</v>
+      </c>
+      <c r="G343" t="n">
+        <v>0</v>
+      </c>
+      <c r="H343" t="b">
+        <v>0</v>
+      </c>
+      <c r="I343" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J343" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210384486</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>1210384445</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>pharma21</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>【日本メーカー公式】ファーマ21 シルキーグロスリペアヘアマスク 湿気対策 髪質改善 くせ毛・うねり・広がり・パサつき・絡まりケア シルクのようなツヤ髪へ サロン品質 ヘアトリートメント ヘアパック</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>PHARMA21</t>
+        </is>
+      </c>
+      <c r="F344" t="n">
+        <v>2750</v>
+      </c>
+      <c r="G344" t="n">
+        <v>0</v>
+      </c>
+      <c r="H344" t="b">
+        <v>0</v>
+      </c>
+      <c r="I344" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J344" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210384445</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>1199000651</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>pharma21</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>【日本メーカー公式】ファーマ21 すっきりヘアコアシャンプー フケかゆみ 芯から補修 パサつき抑え もこもこ泡 摩擦レス 軽やか指通り 爽快感 低刺激 無添加 445mL</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>PHARMA21</t>
+        </is>
+      </c>
+      <c r="F345" t="n">
+        <v>2750</v>
+      </c>
+      <c r="G345" t="n">
+        <v>0</v>
+      </c>
+      <c r="H345" t="b">
+        <v>0</v>
+      </c>
+      <c r="I345" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J345" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199000651</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>1173839691</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>enseoul</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>酵素ピーリングジェル ガラクトミー成分配合 75mL×3個セット</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F346" t="n">
+        <v>4174</v>
+      </c>
+      <c r="G346" t="n">
+        <v>1</v>
+      </c>
+      <c r="H346" t="b">
+        <v>0</v>
+      </c>
+      <c r="I346" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J346" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1173839691</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>1190324743</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>enseoul</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>ゼロ クレンジングバーム ブライトニング 100mL 3本セット</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>バニラコ</t>
+        </is>
+      </c>
+      <c r="F347" t="n">
+        <v>9248</v>
+      </c>
+      <c r="G347" t="n">
+        <v>1</v>
+      </c>
+      <c r="H347" t="b">
+        <v>0</v>
+      </c>
+      <c r="I347" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J347" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190324743</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>1169332727</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>enseoul</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>炭酸パウダー洗顔 濃密泡 毛穴ケア しっとり洗い上がり 150mL 2本セット</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F348" t="n">
+        <v>4949</v>
+      </c>
+      <c r="G348" t="n">
+        <v>1</v>
+      </c>
+      <c r="H348" t="b">
+        <v>0</v>
+      </c>
+      <c r="I348" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J348" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1169332727</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>1163294474</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>enseoul</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>韓蘭 保湿化粧水 170mL 2本セット</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>イニスフリー</t>
+        </is>
+      </c>
+      <c r="F349" t="n">
+        <v>5820</v>
+      </c>
+      <c r="G349" t="n">
+        <v>1</v>
+      </c>
+      <c r="H349" t="b">
+        <v>0</v>
+      </c>
+      <c r="I349" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J349" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1163294474</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>1161207715</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>enseoul</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>しっとり水分保護 5種ヒアルロン酸×緑茶保湿クリーム 50mL x3</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>イニスフリー</t>
+        </is>
+      </c>
+      <c r="F350" t="n">
+        <v>9631</v>
+      </c>
+      <c r="G350" t="n">
+        <v>0</v>
+      </c>
+      <c r="H350" t="b">
+        <v>0</v>
+      </c>
+      <c r="I350" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J350" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1161207715</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J333"/>
+  <autoFilter ref="A1:J350"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 78, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$350</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$368</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J350"/>
+  <dimension ref="A1:J368"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14805,8 +14805,746 @@
         </is>
       </c>
     </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>1209121752</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>LANLANCOSME</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>【2本セット・2026年新発売・国内正規品】イドラクラリティ 薬用 ブライトニング エッセンス ウォーター 医薬部外品 200ml 美容液 化粧水 ローション エッセンス 潤い 保湿</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>コスメデコルテ</t>
+        </is>
+      </c>
+      <c r="F351" t="n">
+        <v>13902</v>
+      </c>
+      <c r="G351" t="n">
+        <v>0</v>
+      </c>
+      <c r="H351" t="b">
+        <v>0</v>
+      </c>
+      <c r="I351" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J351" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209121752</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>1200341995</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>LANLANCOSME</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>【国内正規品】コスメデコルテ AQ 毛穴美容液オイル 40mL クレンジング オイルクレンジング うるおい 美容液 クレンジング美容液 なめらかな肌 フェイスオイル スキンケア 美容液オイル</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>コスメデコルテ</t>
+        </is>
+      </c>
+      <c r="F352" t="n">
+        <v>10859</v>
+      </c>
+      <c r="G352" t="n">
+        <v>0</v>
+      </c>
+      <c r="H352" t="b">
+        <v>0</v>
+      </c>
+      <c r="I352" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J352" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200341995</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>1160784536</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>LANLANCOSME</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>MONNALI MIHATSU モナリ ミハツ カバートリートメント 200g ブラックシリーズ 黒いトリートメント ヘアケア エイジングケア スカルプケア メンズ レディース</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>MONNALI</t>
+        </is>
+      </c>
+      <c r="F353" t="n">
+        <v>3902</v>
+      </c>
+      <c r="G353" t="n">
+        <v>0</v>
+      </c>
+      <c r="H353" t="b">
+        <v>0</v>
+      </c>
+      <c r="I353" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J353" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1160784536</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>1160784512</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>LANLANCOSME</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>【2点セット】MONNALI MIHATSU モナリ ミハツ クレンジングシャンプー 350ml+トリートメント 200g+ ブラックシリーズ 黒いシャンプー ヘアケア エイジ</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>MONNALI</t>
+        </is>
+      </c>
+      <c r="F354" t="n">
+        <v>9295</v>
+      </c>
+      <c r="G354" t="n">
+        <v>0</v>
+      </c>
+      <c r="H354" t="b">
+        <v>0</v>
+      </c>
+      <c r="I354" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J354" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1160784512</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>1199692215</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>lasana</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>ラサーナ 海藻 ヘア セラム ミスト（200ml）</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>ラサーナ</t>
+        </is>
+      </c>
+      <c r="F355" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G355" t="n">
+        <v>0</v>
+      </c>
+      <c r="H355" t="b">
+        <v>0</v>
+      </c>
+      <c r="I355" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J355" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199692215</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>1199692156</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>lasana</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>ラサーナ 海藻 海泥 シャンプー＆トリートメント セット（空ボトル付き）</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>ラサーナ</t>
+        </is>
+      </c>
+      <c r="F356" t="n">
+        <v>7300</v>
+      </c>
+      <c r="G356" t="n">
+        <v>0</v>
+      </c>
+      <c r="H356" t="b">
+        <v>0</v>
+      </c>
+      <c r="I356" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J356" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199692156</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>1199692199</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>lasana</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>ラサーナ 海藻 ヘア セラム ミルク 120g</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>ラサーナ</t>
+        </is>
+      </c>
+      <c r="F357" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G357" t="n">
+        <v>0</v>
+      </c>
+      <c r="H357" t="b">
+        <v>0</v>
+      </c>
+      <c r="I357" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J357" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199692199</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>1199692158</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>lasana</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>ラサーナ プレミオール ホワイトティーの香り 2点セット シャンプー＆トリートメントセット（空ボトル付き）</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>ラサーナ</t>
+        </is>
+      </c>
+      <c r="F358" t="n">
+        <v>7940</v>
+      </c>
+      <c r="G358" t="n">
+        <v>1</v>
+      </c>
+      <c r="H358" t="b">
+        <v>0</v>
+      </c>
+      <c r="I358" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J358" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199692158</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>1157639375</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>fnehqld</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>[正規品] PDRNエッセンス100+PDRN ハイドロゲルマスク, 1枚/韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F359" t="n">
+        <v>5032</v>
+      </c>
+      <c r="G359" t="n">
+        <v>0</v>
+      </c>
+      <c r="H359" t="b">
+        <v>0</v>
+      </c>
+      <c r="I359" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J359" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1157639375</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>1196602352</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>fnehqld</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>DW-EGFメラワンデーセラムシカアロエ15mLX2個/EGF/シミ/色素沈着 ニキビ跡 メラトーニンアンプル シカ 毛穴/アロエエクソソーム</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>イージーデュー</t>
+        </is>
+      </c>
+      <c r="F360" t="n">
+        <v>9060</v>
+      </c>
+      <c r="G360" t="n">
+        <v>0</v>
+      </c>
+      <c r="H360" t="b">
+        <v>0</v>
+      </c>
+      <c r="I360" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J360" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196602352</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>1196592902</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>fnehqld</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>[大容量] 4世代グローターンエクソソームヘアアンプル130ml+ミニ 30ml 贈呈/ オリーブヤング企画/ヘアケア /抜け毛ケア/脱毛ケア/頭皮ケア/韓国コスメ/グローターン</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>lily eve</t>
+        </is>
+      </c>
+      <c r="F361" t="n">
+        <v>5695</v>
+      </c>
+      <c r="G361" t="n">
+        <v>0</v>
+      </c>
+      <c r="H361" t="b">
+        <v>0</v>
+      </c>
+      <c r="I361" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J361" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196592902</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>1158739035</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>kirakiranandemoya</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>ドリームグロウマスク RR (6枚入り+1購入贈呈) シートマスク 保湿 ツヤ肌 ブライトニング 敏感肌 韓国コスメ 正規品</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>ファミュ</t>
+        </is>
+      </c>
+      <c r="F362" t="n">
+        <v>5760</v>
+      </c>
+      <c r="G362" t="n">
+        <v>0</v>
+      </c>
+      <c r="H362" t="b">
+        <v>0</v>
+      </c>
+      <c r="I362" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J362" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1158739035</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>1196695553</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>kirakiranandemoya</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>ボーンパンテノールピールトナー 180ml / 拭き取り化粧水 角質ケア パンテノール ピーリング 導入化粧水 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>サミュ</t>
+        </is>
+      </c>
+      <c r="F363" t="n">
+        <v>4590</v>
+      </c>
+      <c r="G363" t="n">
+        <v>1</v>
+      </c>
+      <c r="H363" t="b">
+        <v>0</v>
+      </c>
+      <c r="I363" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J363" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196695553</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>1195196973</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>HIHYMY26</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>1秒 ダメージケア マーブル ヘアパック 300g LPP プロテイン トリートメント</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>BIORECIPE</t>
+        </is>
+      </c>
+      <c r="F364" t="n">
+        <v>5224</v>
+      </c>
+      <c r="G364" t="n">
+        <v>0</v>
+      </c>
+      <c r="H364" t="b">
+        <v>0</v>
+      </c>
+      <c r="I364" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J364" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195196973</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>1212713877</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>Lulupi</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>【フィー】 シェイキングシナジーミスト 50ml 全3種</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>フィー</t>
+        </is>
+      </c>
+      <c r="F365" t="n">
+        <v>2654</v>
+      </c>
+      <c r="G365" t="n">
+        <v>0</v>
+      </c>
+      <c r="H365" t="b">
+        <v>0</v>
+      </c>
+      <c r="I365" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J365" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212713877</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>1191657535</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>seoulglowpick</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>シカケア クリア アンプル 30ml</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>ロベクチン</t>
+        </is>
+      </c>
+      <c r="F366" t="n">
+        <v>3290</v>
+      </c>
+      <c r="G366" t="n">
+        <v>0</v>
+      </c>
+      <c r="H366" t="b">
+        <v>0</v>
+      </c>
+      <c r="I366" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J366" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191657535</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>1191655869</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>seoulglowpick</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>[新作]オールデイ ノーセバム トーンアップ サンクッション 2種 SPF45 PA++++ lilac fog vanilla lemon</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>ミルクタッチ</t>
+        </is>
+      </c>
+      <c r="F367" t="n">
+        <v>3982</v>
+      </c>
+      <c r="G367" t="n">
+        <v>0</v>
+      </c>
+      <c r="H367" t="b">
+        <v>0</v>
+      </c>
+      <c r="I367" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J367" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191655869</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>1188483946</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>seoulglowpick</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>キャロット カロテン デイリーマスク 30枚 #毎日使える栄養たっぷりのフェイスマスク</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>スキンフード</t>
+        </is>
+      </c>
+      <c r="F368" t="n">
+        <v>3777</v>
+      </c>
+      <c r="G368" t="n">
+        <v>0</v>
+      </c>
+      <c r="H368" t="b">
+        <v>0</v>
+      </c>
+      <c r="I368" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J368" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188483946</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J350"/>
+  <autoFilter ref="A1:J368"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 81, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$368</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$384</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J368"/>
+  <dimension ref="A1:J384"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15543,8 +15543,664 @@
         </is>
       </c>
     </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>1068190736</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>arimcosmetic</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>パフュームシードライン6種 ボディウォッシュ クリーム ローション ミルク クレンザー ミスト オイル香りと保湿を一度に 5つの無添加 超微粒 バラエキス ギフト用</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>ザフェイスショップ</t>
+        </is>
+      </c>
+      <c r="F369" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G369" t="n">
+        <v>3</v>
+      </c>
+      <c r="H369" t="b">
+        <v>0</v>
+      </c>
+      <c r="I369" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J369" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1068190736</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>1120351146</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>arimcosmetic</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>【30枚】すりおろしのマスクシート 新鮮な自然植物たっぷり 高密着 無添加 保湿 栄養 水分 鎮静 アロエ キュウリ 韓国コスメマスクパックです</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>ザフェイスショップ</t>
+        </is>
+      </c>
+      <c r="F370" t="n">
+        <v>2660</v>
+      </c>
+      <c r="G370" t="n">
+        <v>1</v>
+      </c>
+      <c r="H370" t="b">
+        <v>0</v>
+      </c>
+      <c r="I370" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J370" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1120351146</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>1088835091</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>arimcosmetic</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>旅行用/ 携帯用 化粧品コレクション 韓国コスメ 1ml x 120枚 5ml x 30個 アンプル エマルジョン クリーム CC アイクリーム クレンジングフォーム セラム</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>イザノックス</t>
+        </is>
+      </c>
+      <c r="F371" t="n">
+        <v>2900</v>
+      </c>
+      <c r="G371" t="n">
+        <v>0</v>
+      </c>
+      <c r="H371" t="b">
+        <v>0</v>
+      </c>
+      <c r="I371" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J371" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1088835091</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>1195242230</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>k10shop</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>イリユン セラミドアトローション 無香料 508ml 1個</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>イリユン</t>
+        </is>
+      </c>
+      <c r="F372" t="n">
+        <v>2655</v>
+      </c>
+      <c r="G372" t="n">
+        <v>0</v>
+      </c>
+      <c r="H372" t="b">
+        <v>0</v>
+      </c>
+      <c r="I372" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J372" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195242230</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>1208323570</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>k10shop</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>SKIN1004 マダガスカルセンテラ ヒアルーシカ ウォーターフィットサンセラム 日焼け止め SPF50+ PA++++ 100ml 1個</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>ティーゼン</t>
+        </is>
+      </c>
+      <c r="F373" t="n">
+        <v>3076</v>
+      </c>
+      <c r="G373" t="n">
+        <v>0</v>
+      </c>
+      <c r="H373" t="b">
+        <v>0</v>
+      </c>
+      <c r="I373" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J373" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208323570</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>1164978194</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>peachshop</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>【ビビアン】 ニチ ルームスプレー ウォルナット クリーク グリーン 100ml 1個, 繊維香水 繊維脱臭剤 ドレスパフューム Walnut Creek Green</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>BiBiANG</t>
+        </is>
+      </c>
+      <c r="F374" t="n">
+        <v>2899</v>
+      </c>
+      <c r="G374" t="n">
+        <v>1</v>
+      </c>
+      <c r="H374" t="b">
+        <v>0</v>
+      </c>
+      <c r="I374" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J374" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1164978194</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>1095419459</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>peachshop</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>コントロールA ティーツリーメントスージング スポット 15m /Ctrl+A/ピンクパウダー/ニキビ/ニキビケア/ 薬/teatree/吹き出物/肌荒れ/集中ケア/韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>Dr.Jart+</t>
+        </is>
+      </c>
+      <c r="F375" t="n">
+        <v>3099</v>
+      </c>
+      <c r="G375" t="n">
+        <v>0</v>
+      </c>
+      <c r="H375" t="b">
+        <v>0</v>
+      </c>
+      <c r="I375" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J375" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1095419459</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>1208658337</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>supermoon</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>[Tamburins] SUMMER TAILS ディスカバリーセット</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>タンバリンズ</t>
+        </is>
+      </c>
+      <c r="F376" t="n">
+        <v>1950</v>
+      </c>
+      <c r="G376" t="n">
+        <v>0</v>
+      </c>
+      <c r="H376" t="b">
+        <v>0</v>
+      </c>
+      <c r="I376" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J376" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208658337</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>1203988364</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>supermoon</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>[大容量] オービタミネボディミルク 400ml</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>ビオテルム</t>
+        </is>
+      </c>
+      <c r="F377" t="n">
+        <v>6250</v>
+      </c>
+      <c r="G377" t="n">
+        <v>0</v>
+      </c>
+      <c r="H377" t="b">
+        <v>0</v>
+      </c>
+      <c r="I377" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J377" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203988364</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>1193624609</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>supermoon</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>TXT愛用 BOMBSHELLUTH バムシェル 10ml Oil Perfumeオイル香水</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>DANIELS TRUTH</t>
+        </is>
+      </c>
+      <c r="F378" t="n">
+        <v>6550</v>
+      </c>
+      <c r="G378" t="n">
+        <v>3</v>
+      </c>
+      <c r="H378" t="b">
+        <v>0</v>
+      </c>
+      <c r="I378" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J378" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193624609</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>1189436342</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>supermoon</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>VT リードルショット ユニバース キット 2ml × 5本 x 9種（全45本）正規品 韓国化粧品 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F379" t="n">
+        <v>3250</v>
+      </c>
+      <c r="G379" t="n">
+        <v>3</v>
+      </c>
+      <c r="H379" t="b">
+        <v>0</v>
+      </c>
+      <c r="I379" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J379" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189436342</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>1193991472</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>yujunystore</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>ティーツリーカ リリーフ アンプル,1個,100ml</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F380" t="n">
+        <v>3634</v>
+      </c>
+      <c r="G380" t="n">
+        <v>0</v>
+      </c>
+      <c r="H380" t="b">
+        <v>0</v>
+      </c>
+      <c r="I380" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J380" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193991472</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>1202091445</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>beautyokbank</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>プラミー 3-in-1マルチエフェクトグロースプレー75ml(保湿・メイクキープ・水光肌）</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>PRAMY</t>
+        </is>
+      </c>
+      <c r="F381" t="n">
+        <v>3199</v>
+      </c>
+      <c r="G381" t="n">
+        <v>0</v>
+      </c>
+      <c r="H381" t="b">
+        <v>0</v>
+      </c>
+      <c r="I381" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J381" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202091445</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>1197574204</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>sioris</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>【乾燥対策】【ミスト2本セット】タイムイズランニングアウトミスト100mlユズ果実エキス/オイルイン/べたつかない/保湿/オーガニック認証</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>シオリス</t>
+        </is>
+      </c>
+      <c r="F382" t="n">
+        <v>5544</v>
+      </c>
+      <c r="G382" t="n">
+        <v>1</v>
+      </c>
+      <c r="H382" t="b">
+        <v>0</v>
+      </c>
+      <c r="I382" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J382" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197574204</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>1197590797</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>sioris</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>【ゆらぎ肌対策】マイファーストエッセナー100ml 2本J.Y. Parkプロデュース/緑茶エキス/鎮静ブースター/オーガニック認証</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>シオリス</t>
+        </is>
+      </c>
+      <c r="F383" t="n">
+        <v>7326</v>
+      </c>
+      <c r="G383" t="n">
+        <v>0</v>
+      </c>
+      <c r="H383" t="b">
+        <v>0</v>
+      </c>
+      <c r="I383" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J383" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197590797</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>1195971817</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>sioris</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>【低刺激ミルククレンジング】クレンズ ミー ソフトリー ミルククレンザー シグニチャー 200ml低pH高保湿/ダブル洗顔不要/弱酸性/乾燥肌</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>シオリス</t>
+        </is>
+      </c>
+      <c r="F384" t="n">
+        <v>3630</v>
+      </c>
+      <c r="G384" t="n">
+        <v>2</v>
+      </c>
+      <c r="H384" t="b">
+        <v>0</v>
+      </c>
+      <c r="I384" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J384" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195971817</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J368"/>
+  <autoFilter ref="A1:J384"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 84, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$384</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$400</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J384"/>
+  <dimension ref="A1:J400"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16199,8 +16199,664 @@
         </is>
       </c>
     </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>1126626890</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>HANABEAUTY</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>超低分子 ヒアルロン酸 トナー 300ml</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>イズエンツリー</t>
+        </is>
+      </c>
+      <c r="F385" t="n">
+        <v>3286</v>
+      </c>
+      <c r="G385" t="n">
+        <v>0</v>
+      </c>
+      <c r="H385" t="b">
+        <v>0</v>
+      </c>
+      <c r="I385" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J385" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1126626890</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>1127123405</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>HANABEAUTY</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>PH センシティブ クリーム 60ml</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>サミュ</t>
+        </is>
+      </c>
+      <c r="F386" t="n">
+        <v>5309</v>
+      </c>
+      <c r="G386" t="n">
+        <v>0</v>
+      </c>
+      <c r="H386" t="b">
+        <v>0</v>
+      </c>
+      <c r="I386" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J386" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1127123405</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>1199417296</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>HANABEAUTY</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>プランプハニー セラム 美容液 30g</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>ByUR</t>
+        </is>
+      </c>
+      <c r="F387" t="n">
+        <v>4845</v>
+      </c>
+      <c r="G387" t="n">
+        <v>0</v>
+      </c>
+      <c r="H387" t="b">
+        <v>0</v>
+      </c>
+      <c r="I387" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J387" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199417296</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>1142360945</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>HANABEAUTY</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>毛髪コア強化高栄養タンパク質クリームヘアトリートメント200ml</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>ラグライア</t>
+        </is>
+      </c>
+      <c r="F388" t="n">
+        <v>2785</v>
+      </c>
+      <c r="G388" t="n">
+        <v>0</v>
+      </c>
+      <c r="H388" t="b">
+        <v>0</v>
+      </c>
+      <c r="I388" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J388" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1142360945</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>1211859799</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>ToraDepato</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>ゼロキャスト デイリー 透明 保湿サンスクリーン 50ml 1個</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F389" t="n">
+        <v>3211</v>
+      </c>
+      <c r="G389" t="n">
+        <v>0</v>
+      </c>
+      <c r="H389" t="b">
+        <v>0</v>
+      </c>
+      <c r="I389" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J389" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211859799</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>1211855765</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>ToraDepato</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>ビタC フォーストリックス トーニング セラムマスク 22ml 10枚</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F390" t="n">
+        <v>3173</v>
+      </c>
+      <c r="G390" t="n">
+        <v>0</v>
+      </c>
+      <c r="H390" t="b">
+        <v>0</v>
+      </c>
+      <c r="I390" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J390" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211855765</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>1209466651</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>ToraDepato</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>ラクトリメディ レディース カミングクリーム 15ml</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>メディオン</t>
+        </is>
+      </c>
+      <c r="F391" t="n">
+        <v>5161</v>
+      </c>
+      <c r="G391" t="n">
+        <v>1</v>
+      </c>
+      <c r="H391" t="b">
+        <v>0</v>
+      </c>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J391" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209466651</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>1209446667</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>ToraDepato</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>【クーリング/Yーンケア】ポエリエ フェミニン インナーパフューム デイリー マルチ香水</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>フォエリー</t>
+        </is>
+      </c>
+      <c r="F392" t="n">
+        <v>2331</v>
+      </c>
+      <c r="G392" t="n">
+        <v>1</v>
+      </c>
+      <c r="H392" t="b">
+        <v>0</v>
+      </c>
+      <c r="I392" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J392" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209446667</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>1188839770</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>Helenabeauty</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>[保湿 保水 栄養 シートマスク 10枚 5種類から選択] 高保湿 まとめ買い 夜用 デイリー スキンケア</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>ヴァセリン</t>
+        </is>
+      </c>
+      <c r="F393" t="n">
+        <v>1709</v>
+      </c>
+      <c r="G393" t="n">
+        <v>2</v>
+      </c>
+      <c r="H393" t="b">
+        <v>0</v>
+      </c>
+      <c r="I393" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J393" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188839770</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>1197460025</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>Helenabeauty</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>【1+1 クリームミスト 120ml】保湿ミスト 化粧水ミスト うるおいケア 整肌ケア スプレー 韓国スキンケア デイリーケア</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>バイオヒールボ</t>
+        </is>
+      </c>
+      <c r="F394" t="n">
+        <v>3899</v>
+      </c>
+      <c r="G394" t="n">
+        <v>0</v>
+      </c>
+      <c r="H394" t="b">
+        <v>0</v>
+      </c>
+      <c r="I394" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J394" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197460025</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>1188077394</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>Helenabeauty</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>[秀麗な本超保湿クリーム 50ml] 韓国漢方 高保湿 エイジングケア シワ/改/善 /弾力アップ しっとり濃密テクスチャー</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>秀麗韓</t>
+        </is>
+      </c>
+      <c r="F395" t="n">
+        <v>4427</v>
+      </c>
+      <c r="G395" t="n">
+        <v>0</v>
+      </c>
+      <c r="H395" t="b">
+        <v>0</v>
+      </c>
+      <c r="I395" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J395" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188077394</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>1176564980</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>YoungsVillage</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>[限定セール]ブランネイチャー マジックティーツリーオイル 20ml</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>ブランナチュレ</t>
+        </is>
+      </c>
+      <c r="F396" t="n">
+        <v>3844</v>
+      </c>
+      <c r="G396" t="n">
+        <v>0</v>
+      </c>
+      <c r="H396" t="b">
+        <v>0</v>
+      </c>
+      <c r="I396" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J396" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1176564980</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>1203288450</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>medifa</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>.ダヴ ふわとろクリーミースクラブ ミッドナイトラベンダー 298g Dove ダブ ボディスクラブ【P】</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>ダヴ</t>
+        </is>
+      </c>
+      <c r="F397" t="n">
+        <v>1768</v>
+      </c>
+      <c r="G397" t="n">
+        <v>0</v>
+      </c>
+      <c r="H397" t="b">
+        <v>0</v>
+      </c>
+      <c r="I397" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J397" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203288450</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>1201842300</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>medifa</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>.プロスタイル アイス美容スパークリングスプレー 95g ドライシャンプー【R】</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>プロスタイル</t>
+        </is>
+      </c>
+      <c r="F398" t="n">
+        <v>1900</v>
+      </c>
+      <c r="G398" t="n">
+        <v>0</v>
+      </c>
+      <c r="H398" t="b">
+        <v>0</v>
+      </c>
+      <c r="I398" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J398" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201842300</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>1083089713</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>fresh-aka</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>ピュアフィットシカ 弱酸性クレンジングパッド 100枚入 * 1個</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F399" t="n">
+        <v>3200</v>
+      </c>
+      <c r="G399" t="n">
+        <v>0</v>
+      </c>
+      <c r="H399" t="b">
+        <v>0</v>
+      </c>
+      <c r="I399" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J399" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1083089713</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>1082221247</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>fresh-aka</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>ムード ペブル ネイル 29種</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>ロムアンド</t>
+        </is>
+      </c>
+      <c r="F400" t="n">
+        <v>1810</v>
+      </c>
+      <c r="G400" t="n">
+        <v>0</v>
+      </c>
+      <c r="H400" t="b">
+        <v>0</v>
+      </c>
+      <c r="I400" t="inlineStr">
+        <is>
+          <t>120000021</t>
+        </is>
+      </c>
+      <c r="J400" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1082221247</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J384"/>
+  <autoFilter ref="A1:J400"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 87, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$400</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$407</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J400"/>
+  <dimension ref="A1:J407"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16855,8 +16855,295 @@
         </is>
       </c>
     </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>1172083985</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>KBEAT</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>【公式】ティーツリー グリーン ボディウォッシュ 500ml</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>原料工房</t>
+        </is>
+      </c>
+      <c r="F401" t="n">
+        <v>3739</v>
+      </c>
+      <c r="G401" t="n">
+        <v>0</v>
+      </c>
+      <c r="H401" t="b">
+        <v>0</v>
+      </c>
+      <c r="I401" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J401" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172083985</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>1152723831</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>MAYBORN</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>[NEW] リドルショット ユニバースキット スティックポーチ 45個入り (スティックポーチ 9種)</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F402" t="n">
+        <v>3370</v>
+      </c>
+      <c r="G402" t="n">
+        <v>1</v>
+      </c>
+      <c r="H402" t="b">
+        <v>0</v>
+      </c>
+      <c r="I402" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J402" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1152723831</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>1202354498</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>MAYBORN</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>ライス セラミド エッセンス トナー 250ml - 高保湿・バリアケア・ヴィーガン処方</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>FULLY</t>
+        </is>
+      </c>
+      <c r="F403" t="n">
+        <v>3264</v>
+      </c>
+      <c r="G403" t="n">
+        <v>0</v>
+      </c>
+      <c r="H403" t="b">
+        <v>0</v>
+      </c>
+      <c r="I403" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J403" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202354498</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>1188188856</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>MAYBORN</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>マダガスカル センテラ プロバイオシカ インテンシブ アンプル 50ml</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F404" t="n">
+        <v>1986</v>
+      </c>
+      <c r="G404" t="n">
+        <v>0</v>
+      </c>
+      <c r="H404" t="b">
+        <v>0</v>
+      </c>
+      <c r="I404" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J404" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188188856</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>1181822405</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>kirakirahosi</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>ACON エクオンディープ クレンジングフォーム 100mL</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>東亜製薬</t>
+        </is>
+      </c>
+      <c r="F405" t="n">
+        <v>1800</v>
+      </c>
+      <c r="G405" t="n">
+        <v>0</v>
+      </c>
+      <c r="H405" t="b">
+        <v>0</v>
+      </c>
+      <c r="I405" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J405" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1181822405</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>1181822404</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>kirakirahosi</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>コンセントレートアンプル 30ml クリニックライン</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F406" t="n">
+        <v>5300</v>
+      </c>
+      <c r="G406" t="n">
+        <v>0</v>
+      </c>
+      <c r="H406" t="b">
+        <v>0</v>
+      </c>
+      <c r="I406" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J406" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1181822404</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>1192796253</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>heyhey</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>リジュビエス　アンプル　６ml x 2本入り リジュビ-エス　リジュビーS</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F407" t="n">
+        <v>4650</v>
+      </c>
+      <c r="G407" t="n">
+        <v>3</v>
+      </c>
+      <c r="H407" t="b">
+        <v>0</v>
+      </c>
+      <c r="I407" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J407" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192796253</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J400"/>
+  <autoFilter ref="A1:J407"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 90, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$407</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$417</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J407"/>
+  <dimension ref="A1:J417"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17142,8 +17142,418 @@
         </is>
       </c>
     </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>1186319083</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>wb</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>韓国正規品 AMPLE:N ペプチドショットアンプル2X 100ml 大容量美容液 ペプチド 高保湿 ハリケア 弾力ケア 韓国コスメ 韓国直送</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>アンプルエヌ</t>
+        </is>
+      </c>
+      <c r="F408" t="n">
+        <v>2999</v>
+      </c>
+      <c r="G408" t="n">
+        <v>0</v>
+      </c>
+      <c r="H408" t="b">
+        <v>0</v>
+      </c>
+      <c r="I408" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J408" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1186319083</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>1174996099</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>wb</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>韓国正規品 3Dハリクリームセット 50ml 美容液15ml+ミスト20ml付 豪華2点特典 保湿 ハリケア 韓国コスメ 韓国直送</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>バイオヒールボ</t>
+        </is>
+      </c>
+      <c r="F409" t="n">
+        <v>3900</v>
+      </c>
+      <c r="G409" t="n">
+        <v>1</v>
+      </c>
+      <c r="H409" t="b">
+        <v>0</v>
+      </c>
+      <c r="I409" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J409" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174996099</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>1213260537</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>wb</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>韓国正規品 リニューアル MLE保湿ローション 120ml／200ml 敏感肌 乾燥肌 ベビー 全身 肌バリア 韓国直送</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>アトパーム</t>
+        </is>
+      </c>
+      <c r="F410" t="n">
+        <v>2465</v>
+      </c>
+      <c r="G410" t="n">
+        <v>0</v>
+      </c>
+      <c r="H410" t="b">
+        <v>0</v>
+      </c>
+      <c r="I410" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J410" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213260537</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>1150363013</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>ASHA_MARKET</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>サンミューズ無機自茶サンクリーム[SPF50+/PA++++], 50ml</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>ビープレーン</t>
+        </is>
+      </c>
+      <c r="F411" t="n">
+        <v>1650</v>
+      </c>
+      <c r="G411" t="n">
+        <v>0</v>
+      </c>
+      <c r="H411" t="b">
+        <v>0</v>
+      </c>
+      <c r="I411" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J411" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1150363013</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>817605715</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>greengreen-q</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>グッチ バンブー 75ML EDP SP</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>GUCCI</t>
+        </is>
+      </c>
+      <c r="F412" t="n">
+        <v>12540</v>
+      </c>
+      <c r="G412" t="n">
+        <v>2</v>
+      </c>
+      <c r="H412" t="b">
+        <v>0</v>
+      </c>
+      <c r="I412" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J412" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=817605715</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>724850594</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>greengreen-q</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>ポロ ブラック 125ML EDT SP</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>Ralph Lauren</t>
+        </is>
+      </c>
+      <c r="F413" t="n">
+        <v>7700</v>
+      </c>
+      <c r="G413" t="n">
+        <v>0</v>
+      </c>
+      <c r="H413" t="b">
+        <v>0</v>
+      </c>
+      <c r="I413" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J413" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=724850594</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>1183179464</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>telemedia</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>ハー ロンドン ドリーム EDP SP 30ml</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>Burberry</t>
+        </is>
+      </c>
+      <c r="F414" t="n">
+        <v>11198</v>
+      </c>
+      <c r="G414" t="n">
+        <v>0</v>
+      </c>
+      <c r="H414" t="b">
+        <v>0</v>
+      </c>
+      <c r="I414" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J414" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183179464</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>1065580984</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>telemedia</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>グロウ バイジェイロー EDT SP 100ml</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>ジェニファーロペス</t>
+        </is>
+      </c>
+      <c r="F415" t="n">
+        <v>4373</v>
+      </c>
+      <c r="G415" t="n">
+        <v>0</v>
+      </c>
+      <c r="H415" t="b">
+        <v>0</v>
+      </c>
+      <c r="I415" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J415" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1065580984</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>1066844135</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>telemedia</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>オードモワゼル フローラル EDT SP 100ml</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>GIVENCHY</t>
+        </is>
+      </c>
+      <c r="F416" t="n">
+        <v>12073</v>
+      </c>
+      <c r="G416" t="n">
+        <v>0</v>
+      </c>
+      <c r="H416" t="b">
+        <v>0</v>
+      </c>
+      <c r="I416" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J416" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1066844135</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>1183179421</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>telemedia</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>ポロ レッド （チューブサンプル） EDT SP 1.2ml</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>Ralph Lauren</t>
+        </is>
+      </c>
+      <c r="F417" t="n">
+        <v>2340</v>
+      </c>
+      <c r="G417" t="n">
+        <v>0</v>
+      </c>
+      <c r="H417" t="b">
+        <v>0</v>
+      </c>
+      <c r="I417" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J417" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183179421</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J407"/>
+  <autoFilter ref="A1:J417"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 93, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$417</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$431</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J417"/>
+  <dimension ref="A1:J431"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17552,8 +17552,582 @@
         </is>
       </c>
     </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>1212001587</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>wish</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>レプリカ オン ア デート EDT BT 7ml【ミニ香水 ミニボトル】【香水 メンズ レディース】</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>メゾンマルジェラ</t>
+        </is>
+      </c>
+      <c r="F418" t="n">
+        <v>1925</v>
+      </c>
+      <c r="G418" t="n">
+        <v>0</v>
+      </c>
+      <c r="H418" t="b">
+        <v>0</v>
+      </c>
+      <c r="I418" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J418" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212001587</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>1212001233</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>wish</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>アクア エッセンツィアーレ ブルー EDT SP 100ml【香水 ギフト メンズ】</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>CHANEL</t>
+        </is>
+      </c>
+      <c r="F419" t="n">
+        <v>7645</v>
+      </c>
+      <c r="G419" t="n">
+        <v>0</v>
+      </c>
+      <c r="H419" t="b">
+        <v>0</v>
+      </c>
+      <c r="I419" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J419" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212001233</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>1195231911</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>wish</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>サムライ ライト EDT SP 100ml SAMOURAI LIGHT【香水 メンズ】ALAIN DELON アラン・ドロン</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>サムライ</t>
+        </is>
+      </c>
+      <c r="F420" t="n">
+        <v>4763</v>
+      </c>
+      <c r="G420" t="n">
+        <v>0</v>
+      </c>
+      <c r="H420" t="b">
+        <v>0</v>
+      </c>
+      <c r="I420" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J420" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195231911</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>1159643310</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>cosmetch</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>ハッピー フォーメン EDC 50ml SP （香水）</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>クリニーク</t>
+        </is>
+      </c>
+      <c r="F421" t="n">
+        <v>3530</v>
+      </c>
+      <c r="G421" t="n">
+        <v>0</v>
+      </c>
+      <c r="H421" t="b">
+        <v>0</v>
+      </c>
+      <c r="I421" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J421" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1159643310</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>1158430479</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>cosmetch</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>アベンヌウォーター 300ml 3本セット （化粧水）</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>アベンヌ</t>
+        </is>
+      </c>
+      <c r="F422" t="n">
+        <v>3620</v>
+      </c>
+      <c r="G422" t="n">
+        <v>3</v>
+      </c>
+      <c r="H422" t="b">
+        <v>0</v>
+      </c>
+      <c r="I422" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J422" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1158430479</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>1192146158</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>cosmetch</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>アナスイ EDT 30ml SP （香水）</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>アナスイ</t>
+        </is>
+      </c>
+      <c r="F423" t="n">
+        <v>3020</v>
+      </c>
+      <c r="G423" t="n">
+        <v>0</v>
+      </c>
+      <c r="H423" t="b">
+        <v>0</v>
+      </c>
+      <c r="I423" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J423" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192146158</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>1189247744</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>cosmetch</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>アルティム8 スブリム ビューティクレンジングオイルn 150ml （メイク落とし） 【国内正規品】</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>シュウウエムラ</t>
+        </is>
+      </c>
+      <c r="F424" t="n">
+        <v>5610</v>
+      </c>
+      <c r="G424" t="n">
+        <v>0</v>
+      </c>
+      <c r="H424" t="b">
+        <v>0</v>
+      </c>
+      <c r="I424" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J424" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189247744</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>1138374893</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>besba</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>香栄化学 エルカラ20 400ml レフィル 詰替用</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>香栄化学</t>
+        </is>
+      </c>
+      <c r="F425" t="n">
+        <v>3657</v>
+      </c>
+      <c r="G425" t="n">
+        <v>0</v>
+      </c>
+      <c r="H425" t="b">
+        <v>0</v>
+      </c>
+      <c r="I425" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J425" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1138374893</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>1117338699</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>besba</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>ブルガリ アクア プールオム EDT オードトワレ SP 30ml 香水 BVLGARI</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>ブルガリ</t>
+        </is>
+      </c>
+      <c r="F426" t="n">
+        <v>9631</v>
+      </c>
+      <c r="G426" t="n">
+        <v>1</v>
+      </c>
+      <c r="H426" t="b">
+        <v>0</v>
+      </c>
+      <c r="I426" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J426" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1117338699</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>1117341863</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>besba</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>メゾン マルジェラ レプリカ バブル バス EDT オードトワレ SP 10ml ミニ香水 MAISON MARGIELA</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>メゾンマルジェラ</t>
+        </is>
+      </c>
+      <c r="F427" t="n">
+        <v>3821</v>
+      </c>
+      <c r="G427" t="n">
+        <v>0</v>
+      </c>
+      <c r="H427" t="b">
+        <v>0</v>
+      </c>
+      <c r="I427" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J427" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1117341863</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>1185513461</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>sellon</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>エーキュア ピュリファイング スポット クリーム 2X 30ml 1個</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>Cutem</t>
+        </is>
+      </c>
+      <c r="F428" t="n">
+        <v>3431</v>
+      </c>
+      <c r="G428" t="n">
+        <v>0</v>
+      </c>
+      <c r="H428" t="b">
+        <v>0</v>
+      </c>
+      <c r="I428" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J428" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1185513461</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>1185105694</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>sellon</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>ビール酵母 スカルプケア トリートメント 1L 2個</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>AVCA</t>
+        </is>
+      </c>
+      <c r="F429" t="n">
+        <v>4226</v>
+      </c>
+      <c r="G429" t="n">
+        <v>0</v>
+      </c>
+      <c r="H429" t="b">
+        <v>0</v>
+      </c>
+      <c r="I429" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J429" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1185105694</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>1184246186</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>sellon</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>AHA・BHA・PHA 30デイズ ミラクル トナー 150ml（1個）</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>サムバイミー</t>
+        </is>
+      </c>
+      <c r="F430" t="n">
+        <v>3885</v>
+      </c>
+      <c r="G430" t="n">
+        <v>0</v>
+      </c>
+      <c r="H430" t="b">
+        <v>0</v>
+      </c>
+      <c r="I430" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J430" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1184246186</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>1183988943</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>sellon</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>ヘアトリートメント 1000ml（大容量）LPP プロテイン集中ケア／極ダメージ補修（ベイベリーオーチャードの香り）1L × 1個</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>VADEV</t>
+        </is>
+      </c>
+      <c r="F431" t="n">
+        <v>4004</v>
+      </c>
+      <c r="G431" t="n">
+        <v>0</v>
+      </c>
+      <c r="H431" t="b">
+        <v>0</v>
+      </c>
+      <c r="I431" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J431" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183988943</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J417"/>
+  <autoFilter ref="A1:J431"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 96, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$431</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$442</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J431"/>
+  <dimension ref="A1:J442"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18126,8 +18126,459 @@
         </is>
       </c>
     </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>1123888012</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>unopick</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>リードルショット1000 エッセンス 15ml</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F432" t="n">
+        <v>5700</v>
+      </c>
+      <c r="G432" t="n">
+        <v>1</v>
+      </c>
+      <c r="H432" t="b">
+        <v>0</v>
+      </c>
+      <c r="I432" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J432" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1123888012</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>1123548274</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>unopick</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>ナイアシンアミド 10 TXA 4 ダークスポット コレクティング セラム 30ml</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F433" t="n">
+        <v>4940</v>
+      </c>
+      <c r="G433" t="n">
+        <v>0</v>
+      </c>
+      <c r="H433" t="b">
+        <v>0</v>
+      </c>
+      <c r="I433" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J433" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1123548274</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>1206936003</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>suesstore</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>NC PETRA エンリッチ カールクリーム 150g 2個 ヘアクリーム 韓国ヘアケア パーマヘア ウェーブヘア スタイリング しっとり ツヤ感 2</t>
+        </is>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>NC PETRA</t>
+        </is>
+      </c>
+      <c r="F434" t="n">
+        <v>4950</v>
+      </c>
+      <c r="G434" t="n">
+        <v>0</v>
+      </c>
+      <c r="H434" t="b">
+        <v>0</v>
+      </c>
+      <c r="I434" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J434" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206936003</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>1197607118</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>kaktas</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>【公式】リップスティック パーソナルモード 唇の色へ馴染むpH変化 メンズ メンズリップ バーム [高保湿 pH変化 血色感 クール 無香料 セミマット]</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>KAKTAS</t>
+        </is>
+      </c>
+      <c r="F435" t="n">
+        <v>2420</v>
+      </c>
+      <c r="G435" t="n">
+        <v>0</v>
+      </c>
+      <c r="H435" t="b">
+        <v>0</v>
+      </c>
+      <c r="I435" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J435" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197607118</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>1197608620</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>kaktas</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>【公式】リップスティック サイレントレッド ナチュラルに馴染む赤色 メンズ メンズリップ バーム [高保湿 血色感 ナチュラル 無香料 セミマット とろける使用感]</t>
+        </is>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t>KAKTAS</t>
+        </is>
+      </c>
+      <c r="F436" t="n">
+        <v>2420</v>
+      </c>
+      <c r="G436" t="n">
+        <v>0</v>
+      </c>
+      <c r="H436" t="b">
+        <v>0</v>
+      </c>
+      <c r="I436" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J436" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197608620</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>1119202545</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>kaktas</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>【公式】【20%増量リニューアル】オールインワンジェル 不規則な生活肌へ スキンケアこれ1本 [98%美容液成分 Wビタミンカプセル処方 寝不足の肌 セラミド5種]</t>
+        </is>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>KAKTAS</t>
+        </is>
+      </c>
+      <c r="F437" t="n">
+        <v>3300</v>
+      </c>
+      <c r="G437" t="n">
+        <v>1</v>
+      </c>
+      <c r="H437" t="b">
+        <v>0</v>
+      </c>
+      <c r="I437" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J437" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1119202545</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>1209235049</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>differNdeeper</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>【公式】メラチノール クラウドクリーム 50g /レチノール/メラニンケア/シミケア</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>DIFFER&amp;amp;DEEPER</t>
+        </is>
+      </c>
+      <c r="F438" t="n">
+        <v>4620</v>
+      </c>
+      <c r="G438" t="n">
+        <v>2</v>
+      </c>
+      <c r="H438" t="b">
+        <v>0</v>
+      </c>
+      <c r="I438" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J438" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209235049</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>1210321053</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>differNdeeper</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>【公式】メラチノール クラウドクリーム 50g＋メラティノールアンプル(2ml*7ea) /レチノール/メラニンケア/シミケア</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>DIFFER&amp;amp;DEEPER</t>
+        </is>
+      </c>
+      <c r="F439" t="n">
+        <v>7700</v>
+      </c>
+      <c r="G439" t="n">
+        <v>0</v>
+      </c>
+      <c r="H439" t="b">
+        <v>0</v>
+      </c>
+      <c r="I439" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J439" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210321053</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>1209234684</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>differNdeeper</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>【公式】ピエルトラ ファーミングバンドリフター 50ml/リフティング/肌のキメ改善/コエンザイム/顔・首のたるみケア /弾力 /シワ・たるみ改善 / 真のVラインケア</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>DIFFER&amp;amp;DEEPER</t>
+        </is>
+      </c>
+      <c r="F440" t="n">
+        <v>3680</v>
+      </c>
+      <c r="G440" t="n">
+        <v>1</v>
+      </c>
+      <c r="H440" t="b">
+        <v>0</v>
+      </c>
+      <c r="I440" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J440" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209234684</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>1206892952</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>veridel</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>[1+1] ウォーターグロウバリア TXショット 5000 美容液 30ml 2個</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>veridel</t>
+        </is>
+      </c>
+      <c r="F441" t="n">
+        <v>3888</v>
+      </c>
+      <c r="G441" t="n">
+        <v>0</v>
+      </c>
+      <c r="H441" t="b">
+        <v>0</v>
+      </c>
+      <c r="I441" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J441" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206892952</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>1025023517</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>GlowMee</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>ダイブイン 低分子 ヒアルロン酸 スージングクリーム 100ml 1個</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>トリデン</t>
+        </is>
+      </c>
+      <c r="F442" t="n">
+        <v>1913</v>
+      </c>
+      <c r="G442" t="n">
+        <v>2</v>
+      </c>
+      <c r="H442" t="b">
+        <v>0</v>
+      </c>
+      <c r="I442" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J442" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1025023517</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J431"/>
+  <autoFilter ref="A1:J442"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 99, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$442</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$455</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J442"/>
+  <dimension ref="A1:J455"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18577,8 +18577,541 @@
         </is>
       </c>
     </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>1191514399</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>Beautiful_KKK</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>ドクダミポアクレイパック100ml _Beautiful_K</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F443" t="n">
+        <v>2327</v>
+      </c>
+      <c r="G443" t="n">
+        <v>0</v>
+      </c>
+      <c r="H443" t="b">
+        <v>0</v>
+      </c>
+      <c r="I443" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J443" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191514399</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>1191514733</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>Beautiful_KKK</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>ライトウェイトスージングモイスチャーライザー, 80ml _Beautiful_K</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F444" t="n">
+        <v>2215</v>
+      </c>
+      <c r="G444" t="n">
+        <v>0</v>
+      </c>
+      <c r="H444" t="b">
+        <v>0</v>
+      </c>
+      <c r="I444" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J444" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191514733</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>1191514702</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>Beautiful_KKK</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>センテラウォーターアルコールフリートナー, 150ml _Beautiful_K</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F445" t="n">
+        <v>1759</v>
+      </c>
+      <c r="G445" t="n">
+        <v>2</v>
+      </c>
+      <c r="H445" t="b">
+        <v>0</v>
+      </c>
+      <c r="I445" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J445" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191514702</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>1191514690</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>Beautiful_KKK</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>ドクダミLHAモイスチャーピーリングジェル, 120ml _Beautiful_K</t>
+        </is>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F446" t="n">
+        <v>2327</v>
+      </c>
+      <c r="G446" t="n">
+        <v>0</v>
+      </c>
+      <c r="H446" t="b">
+        <v>0</v>
+      </c>
+      <c r="I446" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J446" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191514690</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>1191514653</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>Beautiful_KKK</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>マグワートマスク, 110g _Beautiful_K</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>アイムフロム</t>
+        </is>
+      </c>
+      <c r="F447" t="n">
+        <v>2592</v>
+      </c>
+      <c r="G447" t="n">
+        <v>1</v>
+      </c>
+      <c r="H447" t="b">
+        <v>0</v>
+      </c>
+      <c r="I447" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J447" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191514653</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>1171497230</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>K_JIKGU</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>ノスカナイントラブルセラム, 30ml</t>
+        </is>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t>パティオン</t>
+        </is>
+      </c>
+      <c r="F448" t="n">
+        <v>2954</v>
+      </c>
+      <c r="G448" t="n">
+        <v>0</v>
+      </c>
+      <c r="H448" t="b">
+        <v>0</v>
+      </c>
+      <c r="I448" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J448" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171497230</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>1171497900</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>K_JIKGU</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>ホワイトトリュフファーストアロマティックスプレーセラム, 60ml</t>
+        </is>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F449" t="n">
+        <v>2581</v>
+      </c>
+      <c r="G449" t="n">
+        <v>1</v>
+      </c>
+      <c r="H449" t="b">
+        <v>0</v>
+      </c>
+      <c r="I449" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J449" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171497900</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>1171498084</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>K_JIKGU</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>レッドアクネボディソープ, 400g</t>
+        </is>
+      </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F450" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G450" t="n">
+        <v>1</v>
+      </c>
+      <c r="H450" t="b">
+        <v>0</v>
+      </c>
+      <c r="I450" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J450" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171498084</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>1180666078</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>Beautiful_KK</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>シルクペプチド インテンシブ リフティング アンプル, 35ml _Beautiful_K</t>
+        </is>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>Sung Boon Editor</t>
+        </is>
+      </c>
+      <c r="F451" t="n">
+        <v>1615</v>
+      </c>
+      <c r="G451" t="n">
+        <v>2</v>
+      </c>
+      <c r="H451" t="b">
+        <v>0</v>
+      </c>
+      <c r="I451" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J451" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180666078</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>1203960088</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>HEYDAYS</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>345リリーフクリーム, 50ml</t>
+        </is>
+      </c>
+      <c r="E452" t="inlineStr">
+        <is>
+          <t>ドクターエルシア</t>
+        </is>
+      </c>
+      <c r="F452" t="n">
+        <v>2453</v>
+      </c>
+      <c r="G452" t="n">
+        <v>0</v>
+      </c>
+      <c r="H452" t="b">
+        <v>0</v>
+      </c>
+      <c r="I452" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J452" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203960088</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>1192047927</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>HEYDAYS</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>グリコリックアシッド7%トーニングソリューション 240ml トーニング ソリューション</t>
+        </is>
+      </c>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F453" t="n">
+        <v>2216</v>
+      </c>
+      <c r="G453" t="n">
+        <v>2</v>
+      </c>
+      <c r="H453" t="b">
+        <v>0</v>
+      </c>
+      <c r="I453" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J453" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192047927</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>1133764204</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>shintenchi</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>バイオコラーゲンリアルディープマスク, 4枚</t>
+        </is>
+      </c>
+      <c r="E454" t="inlineStr">
+        <is>
+          <t>Biodance</t>
+        </is>
+      </c>
+      <c r="F454" t="n">
+        <v>2120</v>
+      </c>
+      <c r="G454" t="n">
+        <v>0</v>
+      </c>
+      <c r="H454" t="b">
+        <v>0</v>
+      </c>
+      <c r="I454" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J454" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1133764204</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>1207544119</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>shintenchi</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>エキスパートマデカクリームリニューPDRN, 50ml</t>
+        </is>
+      </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>センテリアン24</t>
+        </is>
+      </c>
+      <c r="F455" t="n">
+        <v>2330</v>
+      </c>
+      <c r="G455" t="n">
+        <v>0</v>
+      </c>
+      <c r="H455" t="b">
+        <v>0</v>
+      </c>
+      <c r="I455" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J455" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207544119</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J442"/>
+  <autoFilter ref="A1:J455"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 102, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$455</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$467</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J455"/>
+  <dimension ref="A1:J467"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19110,8 +19110,500 @@
         </is>
       </c>
     </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>1209812267</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>thebest_mall</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>SOSセラム, 50ml</t>
+        </is>
+      </c>
+      <c r="E456" t="inlineStr">
+        <is>
+          <t>ティルティル</t>
+        </is>
+      </c>
+      <c r="F456" t="n">
+        <v>3524</v>
+      </c>
+      <c r="G456" t="n">
+        <v>0</v>
+      </c>
+      <c r="H456" t="b">
+        <v>0</v>
+      </c>
+      <c r="I456" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J456" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209812267</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>1213161313</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>pinnacosme</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>アンリミテッドメイクアップフィックスミストマット, 100ml</t>
+        </is>
+      </c>
+      <c r="E457" t="inlineStr">
+        <is>
+          <t>シュウウエムラ</t>
+        </is>
+      </c>
+      <c r="F457" t="n">
+        <v>3980</v>
+      </c>
+      <c r="G457" t="n">
+        <v>0</v>
+      </c>
+      <c r="H457" t="b">
+        <v>0</v>
+      </c>
+      <c r="I457" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J457" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213161313</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>1164572296</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>finca</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>サンダルウッド SANDALWOOD 神ノ白檀 オードトワレ 30mL 白檀の香り 香水</t>
+        </is>
+      </c>
+      <c r="E458" t="inlineStr">
+        <is>
+          <t>FINCA</t>
+        </is>
+      </c>
+      <c r="F458" t="n">
+        <v>3300</v>
+      </c>
+      <c r="G458" t="n">
+        <v>0</v>
+      </c>
+      <c r="H458" t="b">
+        <v>0</v>
+      </c>
+      <c r="I458" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J458" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1164572296</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>1164631585</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>finca</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>ストロベリースイート イチゴのささやき オードトワレ 30mL いちごの香り 香水</t>
+        </is>
+      </c>
+      <c r="E459" t="inlineStr">
+        <is>
+          <t>FINCA</t>
+        </is>
+      </c>
+      <c r="F459" t="n">
+        <v>3300</v>
+      </c>
+      <c r="G459" t="n">
+        <v>0</v>
+      </c>
+      <c r="H459" t="b">
+        <v>0</v>
+      </c>
+      <c r="I459" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J459" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1164631585</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>1164565336</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>finca</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>【新型ボトル】オスマンサスナイト 金木犀の夜更かし オードトワレ 30mL キンモクセイの香り 香水</t>
+        </is>
+      </c>
+      <c r="E460" t="inlineStr">
+        <is>
+          <t>FINCA</t>
+        </is>
+      </c>
+      <c r="F460" t="n">
+        <v>3300</v>
+      </c>
+      <c r="G460" t="n">
+        <v>3</v>
+      </c>
+      <c r="H460" t="b">
+        <v>0</v>
+      </c>
+      <c r="I460" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J460" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1164565336</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>1164543671</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>finca</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>リュンクス 愛しい猫 オードトワレ　30mL　シトラスフローラルの香り 香水</t>
+        </is>
+      </c>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>FINCA</t>
+        </is>
+      </c>
+      <c r="F461" t="n">
+        <v>3300</v>
+      </c>
+      <c r="G461" t="n">
+        <v>0</v>
+      </c>
+      <c r="H461" t="b">
+        <v>0</v>
+      </c>
+      <c r="I461" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J461" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1164543671</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>1164543260</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>finca</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>【新型ボトル】リラッサンテコーヒー 時の味わい オードトワレ 30mL コーヒーの香り 香水</t>
+        </is>
+      </c>
+      <c r="E462" t="inlineStr">
+        <is>
+          <t>FINCA</t>
+        </is>
+      </c>
+      <c r="F462" t="n">
+        <v>3300</v>
+      </c>
+      <c r="G462" t="n">
+        <v>0</v>
+      </c>
+      <c r="H462" t="b">
+        <v>0</v>
+      </c>
+      <c r="I462" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J462" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1164543260</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>1203203087</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>mrelephant</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>スキンケアパッド 4種 (各タイプ別)/シラカバ]潤い水分/セリ カミング鎮静/ユジャC トーンアップ(ブライトニング)/ザクロ ハリ弾力パーミング/</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>コアコス</t>
+        </is>
+      </c>
+      <c r="F463" t="n">
+        <v>1890</v>
+      </c>
+      <c r="G463" t="n">
+        <v>0</v>
+      </c>
+      <c r="H463" t="b">
+        <v>0</v>
+      </c>
+      <c r="I463" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J463" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203203087</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>1195547873</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>mrelephant</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>SOS メガ Mケア ソリューションアンプル 30ml</t>
+        </is>
+      </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>MOJELIM</t>
+        </is>
+      </c>
+      <c r="F464" t="n">
+        <v>2210</v>
+      </c>
+      <c r="G464" t="n">
+        <v>0</v>
+      </c>
+      <c r="H464" t="b">
+        <v>0</v>
+      </c>
+      <c r="I464" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J464" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195547873</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>1183054314</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>jkmtr-jp</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>Round Lab（ラウンドラボ）1025 ドクド クリーム 80ml ― 5種セラミドで内側まで満たす鎮静×保湿クリーム</t>
+        </is>
+      </c>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F465" t="n">
+        <v>2300</v>
+      </c>
+      <c r="G465" t="n">
+        <v>0</v>
+      </c>
+      <c r="H465" t="b">
+        <v>0</v>
+      </c>
+      <c r="I465" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J465" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183054314</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>1156238215</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>jkmtr-jp</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>[正規品/ 公式] ブッシュマン ウォータープルーフ プロ 日焼け止め 50g SPF50+ PA++++ 1個</t>
+        </is>
+      </c>
+      <c r="E466" t="inlineStr">
+        <is>
+          <t>BUSHMAN</t>
+        </is>
+      </c>
+      <c r="F466" t="n">
+        <v>3590</v>
+      </c>
+      <c r="G466" t="n">
+        <v>0</v>
+      </c>
+      <c r="H466" t="b">
+        <v>0</v>
+      </c>
+      <c r="I466" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J466" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1156238215</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>1197007088</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>baell</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>ファッロ 超強力 鎮静 トナーパッド 大容量 150枚 敏感肌 低刺激 赤み消し クーリング 急速冷却 肌荒れ 救急 毛穴 水分爆弾 古代穀物 パック 超密着 ピタッと</t>
+        </is>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>BAELL</t>
+        </is>
+      </c>
+      <c r="F467" t="n">
+        <v>2875</v>
+      </c>
+      <c r="G467" t="n">
+        <v>2</v>
+      </c>
+      <c r="H467" t="b">
+        <v>0</v>
+      </c>
+      <c r="I467" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J467" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197007088</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J455"/>
+  <autoFilter ref="A1:J467"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 105, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$467</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$485</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J467"/>
+  <dimension ref="A1:J485"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19602,8 +19602,746 @@
         </is>
       </c>
     </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>1142237251</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>otonari</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>BTSジョングクPerfume 50ml / フォルメント コットンハグ BTS ジョングク</t>
+        </is>
+      </c>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>FORMENT</t>
+        </is>
+      </c>
+      <c r="F468" t="n">
+        <v>4700</v>
+      </c>
+      <c r="G468" t="n">
+        <v>1</v>
+      </c>
+      <c r="H468" t="b">
+        <v>0</v>
+      </c>
+      <c r="I468" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J468" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1142237251</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>1159827458</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>otonari</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>クリーンイットゼロ ピンク 水分 トナー パッド</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>バニラコ</t>
+        </is>
+      </c>
+      <c r="F469" t="n">
+        <v>2300</v>
+      </c>
+      <c r="G469" t="n">
+        <v>0</v>
+      </c>
+      <c r="H469" t="b">
+        <v>0</v>
+      </c>
+      <c r="I469" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J469" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1159827458</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>1080079065</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>otonari</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>デイリー マスクパック 30枚</t>
+        </is>
+      </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>メディヒール</t>
+        </is>
+      </c>
+      <c r="F470" t="n">
+        <v>3550</v>
+      </c>
+      <c r="G470" t="n">
+        <v>1</v>
+      </c>
+      <c r="H470" t="b">
+        <v>0</v>
+      </c>
+      <c r="I470" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J470" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1080079065</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>1181847777</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>RARI</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>【ポムポムプリンコラボ】ライティングトーンアップサンクッション/ヴィーガンリリーフサンクリーム/サンエッセンス/オーセンティックリップグロイバーム/セット企画 / オリーブヤング限定</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>アッテ</t>
+        </is>
+      </c>
+      <c r="F471" t="n">
+        <v>2890</v>
+      </c>
+      <c r="G471" t="n">
+        <v>2</v>
+      </c>
+      <c r="H471" t="b">
+        <v>0</v>
+      </c>
+      <c r="I471" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J471" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1181847777</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>1189371186</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>RARI</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>【NEW!】 シェイキングミスト</t>
+        </is>
+      </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>フィー</t>
+        </is>
+      </c>
+      <c r="F472" t="n">
+        <v>2856</v>
+      </c>
+      <c r="G472" t="n">
+        <v>0</v>
+      </c>
+      <c r="H472" t="b">
+        <v>0</v>
+      </c>
+      <c r="I472" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J472" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189371186</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>1213323194</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>RARI</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>【ピングーコラボ】全種まとめ ポストアルファクーリングパッド 70枚+70枚 / クーリングペプチドアンプル 30ml / ファーストクーリングマスク 5+3枚 / シカクーリングマスク 5+3枚</t>
+        </is>
+      </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>セルフュージョンC</t>
+        </is>
+      </c>
+      <c r="F473" t="n">
+        <v>2310</v>
+      </c>
+      <c r="G473" t="n">
+        <v>0</v>
+      </c>
+      <c r="H473" t="b">
+        <v>0</v>
+      </c>
+      <c r="I473" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J473" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213323194</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>1191474301</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>KBEAUTYOFFICIALSTORE</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>REJURAN 公式 リジュラン PDRN (c-PDRN) ポアタイトニングトナーパッド 60枚 トナーパッド パック</t>
+        </is>
+      </c>
+      <c r="E474" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F474" t="n">
+        <v>4490</v>
+      </c>
+      <c r="G474" t="n">
+        <v>0</v>
+      </c>
+      <c r="H474" t="b">
+        <v>0</v>
+      </c>
+      <c r="I474" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J474" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191474301</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>1193834173</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>KBEAUTYOFFICIALSTORE</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>dAlba 公式 ダルバ 下地 グリーン ウォータフル トーンアップサンクリーム 50ml 5種 ピンク パープル カバーベージュ 21号 23号 日焼け止め</t>
+        </is>
+      </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F475" t="n">
+        <v>4290</v>
+      </c>
+      <c r="G475" t="n">
+        <v>0</v>
+      </c>
+      <c r="H475" t="b">
+        <v>0</v>
+      </c>
+      <c r="I475" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J475" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193834173</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>1193834160</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>KBEAUTYOFFICIALSTORE</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>BRINGGREEN 公式 ブリングリーン ティーツリーシカセンシティブクレンジングウォーター 500ml BRINGGREEN 洗顔 クレンジング</t>
+        </is>
+      </c>
+      <c r="E476" t="inlineStr">
+        <is>
+          <t>bring green</t>
+        </is>
+      </c>
+      <c r="F476" t="n">
+        <v>2990</v>
+      </c>
+      <c r="G476" t="n">
+        <v>1</v>
+      </c>
+      <c r="H476" t="b">
+        <v>0</v>
+      </c>
+      <c r="I476" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J476" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193834160</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>1191474305</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>KBEAUTYOFFICIALSTORE</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>Rejuran 公式 リジュラン リバランシング トナー 120ml+120ml PDRN ( c-PDRN ) 化粧水 口コミ</t>
+        </is>
+      </c>
+      <c r="E477" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F477" t="n">
+        <v>5990</v>
+      </c>
+      <c r="G477" t="n">
+        <v>0</v>
+      </c>
+      <c r="H477" t="b">
+        <v>0</v>
+      </c>
+      <c r="I477" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J477" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191474305</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>1203766483</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>tbas</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>ウォータープルーフ サーフィン サンスティック 20g</t>
+        </is>
+      </c>
+      <c r="E478" t="inlineStr">
+        <is>
+          <t>BUSHMAN</t>
+        </is>
+      </c>
+      <c r="F478" t="n">
+        <v>3201</v>
+      </c>
+      <c r="G478" t="n">
+        <v>0</v>
+      </c>
+      <c r="H478" t="b">
+        <v>0</v>
+      </c>
+      <c r="I478" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J478" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203766483</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>1096782550</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>tbas</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>アクア ヒアルロニック エッセンス 大容量, 250ml</t>
+        </is>
+      </c>
+      <c r="E479" t="inlineStr">
+        <is>
+          <t>ロベクチン</t>
+        </is>
+      </c>
+      <c r="F479" t="n">
+        <v>3888</v>
+      </c>
+      <c r="G479" t="n">
+        <v>0</v>
+      </c>
+      <c r="H479" t="b">
+        <v>0</v>
+      </c>
+      <c r="I479" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J479" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1096782550</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>1211243856</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>Seoulika</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>【クレヨンしんちゃんコラボ】 スーパーメルティングセバムソフトナー 150ml 企画セット (+ステッカー2種+ブラックヘッドリムーバー+コットン40枚)</t>
+        </is>
+      </c>
+      <c r="E480" t="inlineStr">
+        <is>
+          <t>ilso</t>
+        </is>
+      </c>
+      <c r="F480" t="n">
+        <v>2669</v>
+      </c>
+      <c r="G480" t="n">
+        <v>1</v>
+      </c>
+      <c r="H480" t="b">
+        <v>0</v>
+      </c>
+      <c r="I480" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J480" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211243856</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>1207298088</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>Seoulika</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>[ポケモン コラボ] グロウターン 3Dボリュームシャンプー 大容量 500ml 企画 セット(+100ml+キーホルダーポーチ)</t>
+        </is>
+      </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>lily eve</t>
+        </is>
+      </c>
+      <c r="F481" t="n">
+        <v>3092</v>
+      </c>
+      <c r="G481" t="n">
+        <v>0</v>
+      </c>
+      <c r="H481" t="b">
+        <v>0</v>
+      </c>
+      <c r="I481" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J481" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207298088</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>1093898160</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>PeonyAgit</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>発酵豆 バウンス タンパク質 エッセンス 80ml/低刺激/保湿/水分/韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>フラスキン</t>
+        </is>
+      </c>
+      <c r="F482" t="n">
+        <v>4372</v>
+      </c>
+      <c r="G482" t="n">
+        <v>0</v>
+      </c>
+      <c r="H482" t="b">
+        <v>0</v>
+      </c>
+      <c r="I482" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J482" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1093898160</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>1096256291</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>PeonyAgit</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>【正規品】コラーゲンプロフェッショナルプログラムセット (マイクロコラーゲン200mg*4ea+アクティベーションブースター30ml+ドロッパー4ea)/コラーゲン/光沢/高栄養/活力/弾力</t>
+        </is>
+      </c>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>LAVIEN</t>
+        </is>
+      </c>
+      <c r="F483" t="n">
+        <v>15010</v>
+      </c>
+      <c r="G483" t="n">
+        <v>0</v>
+      </c>
+      <c r="H483" t="b">
+        <v>0</v>
+      </c>
+      <c r="I483" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J483" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1096256291</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>1094315646</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>PeonyAgit</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>【1+1】ブイ コラーゲン ハートフィット マルチバーム 10g/肌バリアケア/ スローエイジング/ 高濃縮/ 弾力/ 水分バリア/ 鎮静/ 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F484" t="n">
+        <v>6786</v>
+      </c>
+      <c r="G484" t="n">
+        <v>1</v>
+      </c>
+      <c r="H484" t="b">
+        <v>0</v>
+      </c>
+      <c r="I484" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J484" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1094315646</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>1093734916</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>PeonyAgit</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>【1+1】スピキュールセラム(ニードルアクション100) 30ml/ 塗る毛穴セラム針 / ニードルショット / ブースティングセラム / 肌のキメ改善 / 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>BIOME ACTIVATE</t>
+        </is>
+      </c>
+      <c r="F485" t="n">
+        <v>3995</v>
+      </c>
+      <c r="G485" t="n">
+        <v>0</v>
+      </c>
+      <c r="H485" t="b">
+        <v>0</v>
+      </c>
+      <c r="I485" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J485" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1093734916</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J467"/>
+  <autoFilter ref="A1:J485"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 108, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$485</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$499</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J485"/>
+  <dimension ref="A1:J499"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20340,8 +20340,582 @@
         </is>
       </c>
     </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>1201105046</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>onsensou</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>シャンプー トリートメント セット KABOSU 【LDK A評価・ランキング1位】 ヘアケア ギフト 乾燥 パサつき 切れ毛・枝毛を防ぐ 12種アミノ酸 セラミド配合 ノンシリコン オーガニック発想</t>
+        </is>
+      </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>オンセンソウ</t>
+        </is>
+      </c>
+      <c r="F486" t="n">
+        <v>4026</v>
+      </c>
+      <c r="G486" t="n">
+        <v>0</v>
+      </c>
+      <c r="H486" t="b">
+        <v>0</v>
+      </c>
+      <c r="I486" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J486" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201105046</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>1205625745</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>COSNRM</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>パンテノールクリーム 80ml</t>
+        </is>
+      </c>
+      <c r="E487" t="inlineStr">
+        <is>
+          <t>アトパーム</t>
+        </is>
+      </c>
+      <c r="F487" t="n">
+        <v>2882</v>
+      </c>
+      <c r="G487" t="n">
+        <v>0</v>
+      </c>
+      <c r="H487" t="b">
+        <v>0</v>
+      </c>
+      <c r="I487" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J487" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205625745</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>1201757060</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>COSNRM</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>マルチペプチドセラムフォーヘアデンシティ 60ml 2個 ヘアケア</t>
+        </is>
+      </c>
+      <c r="E488" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F488" t="n">
+        <v>8612</v>
+      </c>
+      <c r="G488" t="n">
+        <v>0</v>
+      </c>
+      <c r="H488" t="b">
+        <v>0</v>
+      </c>
+      <c r="I488" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J488" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201757060</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>1194137533</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>COSNRM</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>ルティナー マルチバーム 15ml</t>
+        </is>
+      </c>
+      <c r="E489" t="inlineStr">
+        <is>
+          <t>aXENDA</t>
+        </is>
+      </c>
+      <c r="F489" t="n">
+        <v>4232</v>
+      </c>
+      <c r="G489" t="n">
+        <v>1</v>
+      </c>
+      <c r="H489" t="b">
+        <v>0</v>
+      </c>
+      <c r="I489" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J489" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194137533</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>1194137521</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>COSNRM</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>ユース シナジー リフティング ファーストエッセンス 100ml</t>
+        </is>
+      </c>
+      <c r="E490" t="inlineStr">
+        <is>
+          <t>メディヒール</t>
+        </is>
+      </c>
+      <c r="F490" t="n">
+        <v>6573</v>
+      </c>
+      <c r="G490" t="n">
+        <v>0</v>
+      </c>
+      <c r="H490" t="b">
+        <v>0</v>
+      </c>
+      <c r="I490" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J490" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194137521</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>1209961997</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>WISEPICK0423</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>レチノール0.2%のスクワランセラム_30ml_1個</t>
+        </is>
+      </c>
+      <c r="E491" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F491" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G491" t="n">
+        <v>0</v>
+      </c>
+      <c r="H491" t="b">
+        <v>0</v>
+      </c>
+      <c r="I491" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J491" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209961997</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>1209962351</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>WISEPICK0423</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>ヒアルロン酸2% + B5セラム_30ml_1個</t>
+        </is>
+      </c>
+      <c r="E492" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F492" t="n">
+        <v>2784</v>
+      </c>
+      <c r="G492" t="n">
+        <v>0</v>
+      </c>
+      <c r="H492" t="b">
+        <v>0</v>
+      </c>
+      <c r="I492" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J492" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209962351</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>1209956990</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>WISEPICK0423</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>ナイアシンアミド10% + ジンク1%エッセンス_30ml_1個</t>
+        </is>
+      </c>
+      <c r="E493" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F493" t="n">
+        <v>1509</v>
+      </c>
+      <c r="G493" t="n">
+        <v>0</v>
+      </c>
+      <c r="H493" t="b">
+        <v>0</v>
+      </c>
+      <c r="I493" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J493" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209956990</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>1196826611</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>OliveYouth</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>ブルービーン B5-PDRN マイルドローション 230ml / 保湿乳液 敏感肌対応 うるおいケア スキンケアローション 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E494" t="inlineStr">
+        <is>
+          <t>bring green</t>
+        </is>
+      </c>
+      <c r="F494" t="n">
+        <v>2999</v>
+      </c>
+      <c r="G494" t="n">
+        <v>3</v>
+      </c>
+      <c r="H494" t="b">
+        <v>0</v>
+      </c>
+      <c r="I494" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J494" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196826611</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>1164705875</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>OliveYouth</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>ウォータープルーフプロ日焼け止め 50g+サンスティック 20g / アウトドア スポーツ対応UVクリーム 汗・水に強いスティックタイプ 手を汚さない</t>
+        </is>
+      </c>
+      <c r="E495" t="inlineStr">
+        <is>
+          <t>BUSHMAN</t>
+        </is>
+      </c>
+      <c r="F495" t="n">
+        <v>5499</v>
+      </c>
+      <c r="G495" t="n">
+        <v>1</v>
+      </c>
+      <c r="H495" t="b">
+        <v>0</v>
+      </c>
+      <c r="I495" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J495" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1164705875</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>1146818611</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>thesugar</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>ペプチドショットアンプル 100ml x 2ea [大容量] / 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E496" t="inlineStr">
+        <is>
+          <t>アンプルエヌ</t>
+        </is>
+      </c>
+      <c r="F496" t="n">
+        <v>2899</v>
+      </c>
+      <c r="G496" t="n">
+        <v>3</v>
+      </c>
+      <c r="H496" t="b">
+        <v>0</v>
+      </c>
+      <c r="I496" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J496" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1146818611</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>1213387450</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>Crystal_K</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>THEVITAレチナールショットタイトニングブースター, 15ml, 2個</t>
+        </is>
+      </c>
+      <c r="E497" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F497" t="n">
+        <v>4800</v>
+      </c>
+      <c r="G497" t="n">
+        <v>0</v>
+      </c>
+      <c r="H497" t="b">
+        <v>0</v>
+      </c>
+      <c r="I497" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J497" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213387450</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>1123317400</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>withgaia</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>[1+1]レッド センテラカ マスク 10枚</t>
+        </is>
+      </c>
+      <c r="E498" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F498" t="n">
+        <v>7390</v>
+      </c>
+      <c r="G498" t="n">
+        <v>1</v>
+      </c>
+      <c r="H498" t="b">
+        <v>0</v>
+      </c>
+      <c r="I498" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J498" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1123317400</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>1133684811</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>withgaia</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>プレミアムブリリアントミスト, 90ml</t>
+        </is>
+      </c>
+      <c r="E499" t="inlineStr">
+        <is>
+          <t>Kopher</t>
+        </is>
+      </c>
+      <c r="F499" t="n">
+        <v>5350</v>
+      </c>
+      <c r="G499" t="n">
+        <v>0</v>
+      </c>
+      <c r="H499" t="b">
+        <v>0</v>
+      </c>
+      <c r="I499" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J499" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1133684811</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J485"/>
+  <autoFilter ref="A1:J499"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 111, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$499</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$501</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J499"/>
+  <dimension ref="A1:J501"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20914,8 +20914,90 @@
         </is>
       </c>
     </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>1160698268</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>DRsChoice</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>ドルコ PACE7II FRESH カミソリ メンズ 12個</t>
+        </is>
+      </c>
+      <c r="E500" t="inlineStr">
+        <is>
+          <t>ドルコ</t>
+        </is>
+      </c>
+      <c r="F500" t="n">
+        <v>4920</v>
+      </c>
+      <c r="G500" t="n">
+        <v>0</v>
+      </c>
+      <c r="H500" t="b">
+        <v>0</v>
+      </c>
+      <c r="I500" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J500" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1160698268</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>1174362545</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>vivienpink_SG_jp</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>ブライトニング毛穴ジャブティパッド本品40枚+10枚（追加贈呈）</t>
+        </is>
+      </c>
+      <c r="E501" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F501" t="n">
+        <v>3890</v>
+      </c>
+      <c r="G501" t="n">
+        <v>3</v>
+      </c>
+      <c r="H501" t="b">
+        <v>0</v>
+      </c>
+      <c r="I501" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J501" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174362545</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J499"/>
+  <autoFilter ref="A1:J501"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 1, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$307</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$316</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J307"/>
+  <dimension ref="A1:J316"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13042,8 +13042,377 @@
         </is>
       </c>
     </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>1158926077</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>kireinare</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>イポケアEX　角質 角質粒 顔 首 肩 胸 角質ケア 簡単・塗るだけ 専用美容液 イポケア</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>イポケア</t>
+        </is>
+      </c>
+      <c r="F308" t="n">
+        <v>2200</v>
+      </c>
+      <c r="G308" t="n">
+        <v>5</v>
+      </c>
+      <c r="H308" t="b">
+        <v>0</v>
+      </c>
+      <c r="I308" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J308" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1158926077</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>1195426254</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>kireinare</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>ソープ　100g　ソープ　トウキョウ　デリケートゾーン 石鹸 保湿 ボディケア 国産 ジャムウ石けん HPナチュラルソープ</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>東京ラブ</t>
+        </is>
+      </c>
+      <c r="F309" t="n">
+        <v>1680</v>
+      </c>
+      <c r="G309" t="n">
+        <v>0</v>
+      </c>
+      <c r="H309" t="b">
+        <v>0</v>
+      </c>
+      <c r="I309" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J309" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195426254</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>1213620539</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>KSpot</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>グリーントマト NMN ポアリフティングアンプル 40ml×2</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>グリーントマト</t>
+        </is>
+      </c>
+      <c r="F310" t="n">
+        <v>2600</v>
+      </c>
+      <c r="G310" t="n">
+        <v>0</v>
+      </c>
+      <c r="H310" t="b">
+        <v>0</v>
+      </c>
+      <c r="I310" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J310" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213620539</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>1189255608</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>hjfutures</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>VT　正規品　リードルショット100/300/700/ 韓国コスメ/7月限定</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F311" t="n">
+        <v>2780</v>
+      </c>
+      <c r="G311" t="n">
+        <v>4</v>
+      </c>
+      <c r="H311" t="b">
+        <v>0</v>
+      </c>
+      <c r="I311" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J311" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189255608</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>1072105391</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>changefit</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>[ダーマルマトリックス] エピダーマルデトキシファイングマスク (23ml*4枚)</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>Dermall-matrix</t>
+        </is>
+      </c>
+      <c r="F312" t="n">
+        <v>1950</v>
+      </c>
+      <c r="G312" t="n">
+        <v>1</v>
+      </c>
+      <c r="H312" t="b">
+        <v>0</v>
+      </c>
+      <c r="I312" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J312" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1072105391</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>1211228394</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>sallymoazen</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>ひんやりクール リカバリー グラフェンパッチ 156枚 クールタイプ</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>POWER FULX</t>
+        </is>
+      </c>
+      <c r="F313" t="n">
+        <v>3300</v>
+      </c>
+      <c r="G313" t="n">
+        <v>0</v>
+      </c>
+      <c r="H313" t="b">
+        <v>0</v>
+      </c>
+      <c r="I313" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J313" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211228394</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>1166295513</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>sallymoazen</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>【1+1】 ボリューマイジングラディアンスエッセンス all in one / シテノール(R)A 50ml オールインワン美容液 ヒアルロン酸 グルタチオン ペプチド　韓国発送</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>LAVIEN</t>
+        </is>
+      </c>
+      <c r="F314" t="n">
+        <v>15900</v>
+      </c>
+      <c r="G314" t="n">
+        <v>2</v>
+      </c>
+      <c r="H314" t="b">
+        <v>0</v>
+      </c>
+      <c r="I314" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J314" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1166295513</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>1192835408</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>premier-antiaging</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>【数量限定】 Lalaskin 白玉 ピーリングジェル 洗顔 140g ・ 水光シャワーミスト 60g セット ピーリング 洗顔ジェル ミスト化粧水 ララスキン</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>Lalaskin</t>
+        </is>
+      </c>
+      <c r="F315" t="n">
+        <v>1650</v>
+      </c>
+      <c r="G315" t="n">
+        <v>12</v>
+      </c>
+      <c r="H315" t="b">
+        <v>0</v>
+      </c>
+      <c r="I315" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J315" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192835408</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>1102313093</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>premier-antiaging</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>【医薬部外品/うるおい・肌あれケア*】 ザ 薬用クレンジングバーム バリア 18g×3/66g 医薬部外品 緑 バーム ニキビ 花粉 低刺激 敏感肌 肌荒れ 保湿 メイク落とし スキンケア</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>DUO</t>
+        </is>
+      </c>
+      <c r="F316" t="n">
+        <v>2257</v>
+      </c>
+      <c r="G316" t="n">
+        <v>15</v>
+      </c>
+      <c r="H316" t="b">
+        <v>0</v>
+      </c>
+      <c r="I316" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J316" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1102313093</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J307"/>
+  <autoFilter ref="A1:J316"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 2, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$323</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$333</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J323"/>
+  <dimension ref="A1:J333"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13698,8 +13698,418 @@
         </is>
       </c>
     </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>809443442</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>lctradinghouse</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>速達便 税込 Rexona (レクソーナ) Women Free Spirit Roll On 女性フリースピリットロールオン45ml x 5</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>レクソーナ</t>
+        </is>
+      </c>
+      <c r="F324" t="n">
+        <v>3999</v>
+      </c>
+      <c r="G324" t="n">
+        <v>8</v>
+      </c>
+      <c r="H324" t="b">
+        <v>0</v>
+      </c>
+      <c r="I324" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J324" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=809443442</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>809459822</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>lctradinghouse</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>速達便 税込 Rexona (レクソーナ) Men Quantum Dry Roll On メン量子ドライロールオン 45ml x 3</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>レクソーナ</t>
+        </is>
+      </c>
+      <c r="F325" t="n">
+        <v>3500</v>
+      </c>
+      <c r="G325" t="n">
+        <v>0</v>
+      </c>
+      <c r="H325" t="b">
+        <v>0</v>
+      </c>
+      <c r="I325" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J325" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=809459822</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>809426932</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>lctradinghouse</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>速達便 税込 Rexona (レクソーナ) Men Quantum Dry Roll On メン量子ドライロールオン 45ml x 5</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>レクソーナ</t>
+        </is>
+      </c>
+      <c r="F326" t="n">
+        <v>3999</v>
+      </c>
+      <c r="G326" t="n">
+        <v>0</v>
+      </c>
+      <c r="H326" t="b">
+        <v>0</v>
+      </c>
+      <c r="I326" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J326" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=809426932</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>1126994397</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>steambase</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>【公式】STEAMBASE TEA TREE SCALP WATER SCALER 500ML /シャンプー /韓国シャンプー/頭皮シャンプー/ヘアケア/頭皮 匂い/頭皮かゆみ/頭皮にきび/頭皮皮脂</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>STEAMBASE</t>
+        </is>
+      </c>
+      <c r="F327" t="n">
+        <v>4600</v>
+      </c>
+      <c r="G327" t="n">
+        <v>3</v>
+      </c>
+      <c r="H327" t="b">
+        <v>0</v>
+      </c>
+      <c r="I327" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J327" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1126994397</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>1159802621</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>ROAEXPO</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>CELLMEDICS セルメディクス オールデイ サンプロテクト SPF50+ PA+++（70ml) _ 皮膚科開発！1日中うるおう高機能UVケア</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>cellmedics</t>
+        </is>
+      </c>
+      <c r="F328" t="n">
+        <v>5600</v>
+      </c>
+      <c r="G328" t="n">
+        <v>0</v>
+      </c>
+      <c r="H328" t="b">
+        <v>0</v>
+      </c>
+      <c r="I328" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J328" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1159802621</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>1090489296</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>ROAEXPO</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>cellmedics インテンシブ マルチケア マスクパック 28g * 5EA病院の皮膚科様々な皮膚の悩みを一度に - 韓国生産</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>cellmedics</t>
+        </is>
+      </c>
+      <c r="F329" t="n">
+        <v>3780</v>
+      </c>
+      <c r="G329" t="n">
+        <v>0</v>
+      </c>
+      <c r="H329" t="b">
+        <v>0</v>
+      </c>
+      <c r="I329" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J329" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1090489296</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>1188946800</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>AROCELL</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>[10枚] ヒアルB5シートマスク [肌荒れ/赤み/ほてり/クーリング/シワ/ハリツヤ/弾力/鎮静/保湿/うるおい/高密着/シートマスク/栄養/お家エステ/毛穴/トナーパッド/下</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>AROCELL</t>
+        </is>
+      </c>
+      <c r="F330" t="n">
+        <v>3040</v>
+      </c>
+      <c r="G330" t="n">
+        <v>19</v>
+      </c>
+      <c r="H330" t="b">
+        <v>0</v>
+      </c>
+      <c r="I330" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J330" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188946800</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>1156884773</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>Odeloi</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>オドロイ 毛穴収縮 シカ 83.7 コラーゲン ミスト アンプル ルフティグ 100ml, Pore Tightening Cica 83.7 Collagen Mist</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>ODELOI</t>
+        </is>
+      </c>
+      <c r="F331" t="n">
+        <v>2538</v>
+      </c>
+      <c r="G331" t="n">
+        <v>9</v>
+      </c>
+      <c r="H331" t="b">
+        <v>0</v>
+      </c>
+      <c r="I331" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J331" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1156884773</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>1135008630</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>idrrjp</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>[頭皮を潤す・髪にボリューム]【公式】コットン ヘアセラム 80ml</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>IDRR</t>
+        </is>
+      </c>
+      <c r="F332" t="n">
+        <v>2900</v>
+      </c>
+      <c r="G332" t="n">
+        <v>4</v>
+      </c>
+      <c r="H332" t="b">
+        <v>0</v>
+      </c>
+      <c r="I332" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J332" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1135008630</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>1159096115</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>JayeHouse</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>[Banana Boat] スポーツウルトラ サンスクリーンスプレー SPF100 170g / 日焼け止め / 超強力UVカット/ ウォータープルーフ・アメリカ製・顔&amp;amp;全身用</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>バナナボート</t>
+        </is>
+      </c>
+      <c r="F333" t="n">
+        <v>3890</v>
+      </c>
+      <c r="G333" t="n">
+        <v>1</v>
+      </c>
+      <c r="H333" t="b">
+        <v>0</v>
+      </c>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J333" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1159096115</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J323"/>
+  <autoFilter ref="A1:J333"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 4, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$361</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$363</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J361"/>
+  <dimension ref="A1:J363"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15256,8 +15256,90 @@
         </is>
       </c>
     </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>1204214641</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>maybena</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>EGF 10ppm めもとケアクリーム 10ml</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>MAYBENA</t>
+        </is>
+      </c>
+      <c r="F362" t="n">
+        <v>4290</v>
+      </c>
+      <c r="G362" t="n">
+        <v>0</v>
+      </c>
+      <c r="H362" t="b">
+        <v>0</v>
+      </c>
+      <c r="I362" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J362" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204214641</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>1146523540</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>debeaus</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>新商品 公式 ディビュース DEBEAUS インテンシブエナジェニックマルチインディケーション マルチクッションファンデ クッションファンデーション アナザーマジック 韓国コスメ　本品</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>ディビュース</t>
+        </is>
+      </c>
+      <c r="F363" t="n">
+        <v>11000</v>
+      </c>
+      <c r="G363" t="n">
+        <v>0</v>
+      </c>
+      <c r="H363" t="b">
+        <v>0</v>
+      </c>
+      <c r="I363" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J363" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1146523540</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J361"/>
+  <autoFilter ref="A1:J363"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 5, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$363</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$364</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J363"/>
+  <dimension ref="A1:J364"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15338,8 +15338,49 @@
         </is>
       </c>
     </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>1209405922</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>buenoofficial</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>PDRNSOME 7 ペプチド スピキュールクリーム 30g [PDRN エクソソーム ナイトクリーム]</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>ブエノ</t>
+        </is>
+      </c>
+      <c r="F364" t="n">
+        <v>2400</v>
+      </c>
+      <c r="G364" t="n">
+        <v>15</v>
+      </c>
+      <c r="H364" t="b">
+        <v>0</v>
+      </c>
+      <c r="I364" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J364" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209405922</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J363"/>
+  <autoFilter ref="A1:J364"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 7, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$364</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$365</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J364"/>
+  <dimension ref="A1:J365"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15379,8 +15379,49 @@
         </is>
       </c>
     </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>1192490873</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>12est</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>[SET割] グッドナイトシカエクソソームリカバリーアンプルクリーム</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>12EST</t>
+        </is>
+      </c>
+      <c r="F365" t="n">
+        <v>5980</v>
+      </c>
+      <c r="G365" t="n">
+        <v>0</v>
+      </c>
+      <c r="H365" t="b">
+        <v>0</v>
+      </c>
+      <c r="I365" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J365" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192490873</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J364"/>
+  <autoFilter ref="A1:J365"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 8, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$365</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$366</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J365"/>
+  <dimension ref="A1:J366"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15420,8 +15420,49 @@
         </is>
       </c>
     </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>969182336</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>secondtable</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>【詰め替え用】 モイスト シャンプー 400mL 2種類のヒト幹細胞培養液配合 ヒト幹細胞シャンプー クレイシャンプー 泥シャンプー レディース メンズ ギフト</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>JOIE CELU</t>
+        </is>
+      </c>
+      <c r="F366" t="n">
+        <v>1430</v>
+      </c>
+      <c r="G366" t="n">
+        <v>6</v>
+      </c>
+      <c r="H366" t="b">
+        <v>0</v>
+      </c>
+      <c r="I366" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J366" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=969182336</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J365"/>
+  <autoFilter ref="A1:J366"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 8)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$428</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$429</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J428"/>
+  <dimension ref="A1:J429"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17868,8 +17868,49 @@
         </is>
       </c>
     </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>1215224379</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>cococielshop</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>さらさ 液体 無添加【大容量】1900g 植物由来の厳選成分配合 洗濯洗剤 詰め替え</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>さらさ</t>
+        </is>
+      </c>
+      <c r="F429" t="n">
+        <v>2694</v>
+      </c>
+      <c r="G429" t="n">
+        <v>0</v>
+      </c>
+      <c r="H429" t="b">
+        <v>0</v>
+      </c>
+      <c r="I429" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J429" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1215224379</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J428"/>
+  <autoFilter ref="A1:J429"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 14, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$430</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$431</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J430"/>
+  <dimension ref="A1:J431"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17950,8 +17950,49 @@
         </is>
       </c>
     </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>1183037325</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>39market</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>フォーデイズ　ムーサ イオ DN リッチ クリーム final</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>フォーデイズ</t>
+        </is>
+      </c>
+      <c r="F431" t="n">
+        <v>3480</v>
+      </c>
+      <c r="G431" t="n">
+        <v>0</v>
+      </c>
+      <c r="H431" t="b">
+        <v>0</v>
+      </c>
+      <c r="I431" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J431" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183037325</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J430"/>
+  <autoFilter ref="A1:J431"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 15)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$431</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$432</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J431"/>
+  <dimension ref="A1:J432"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17991,8 +17991,49 @@
         </is>
       </c>
     </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>1049528532</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>total-item-shop</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>クレンジングバーム 100g</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>ノエビア</t>
+        </is>
+      </c>
+      <c r="F432" t="n">
+        <v>5980</v>
+      </c>
+      <c r="G432" t="n">
+        <v>0</v>
+      </c>
+      <c r="H432" t="b">
+        <v>0</v>
+      </c>
+      <c r="I432" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J432" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1049528532</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J431"/>
+  <autoFilter ref="A1:J432"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 34, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$432</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$433</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J432"/>
+  <dimension ref="A1:J433"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18032,8 +18032,49 @@
         </is>
       </c>
     </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>1214609928</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>drci-labo</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>EC限定 VC100エッセンスローションEX 285mL＋VC100 エマルジョン EXパウチ ドクターシーラボビタミンC 化粧水 ポンプタイプ</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>ドクターシーラボ</t>
+        </is>
+      </c>
+      <c r="F433" t="n">
+        <v>8910</v>
+      </c>
+      <c r="G433" t="n">
+        <v>0</v>
+      </c>
+      <c r="H433" t="b">
+        <v>0</v>
+      </c>
+      <c r="I433" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J433" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1214609928</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J432"/>
+  <autoFilter ref="A1:J433"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 37, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$434</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$436</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J434"/>
+  <dimension ref="A1:J436"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18114,8 +18114,90 @@
         </is>
       </c>
     </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>1214886234</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>coscora</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>ミネラルリスト ラスティング アイライナ # ダイヤモンド 0.35g</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>ベアミネラル</t>
+        </is>
+      </c>
+      <c r="F435" t="n">
+        <v>2510</v>
+      </c>
+      <c r="G435" t="n">
+        <v>0</v>
+      </c>
+      <c r="H435" t="b">
+        <v>0</v>
+      </c>
+      <c r="I435" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J435" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1214886234</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>1214886256</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>coscora</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>メンズ制汗ロルオン 50ml</t>
+        </is>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t>クラランス</t>
+        </is>
+      </c>
+      <c r="F436" t="n">
+        <v>3240</v>
+      </c>
+      <c r="G436" t="n">
+        <v>0</v>
+      </c>
+      <c r="H436" t="b">
+        <v>0</v>
+      </c>
+      <c r="I436" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J436" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1214886256</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J434"/>
+  <autoFilter ref="A1:J436"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 53, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$437</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$438</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J437"/>
+  <dimension ref="A1:J438"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18237,8 +18237,49 @@
         </is>
       </c>
     </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>1199807022</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>kiyose-store</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>SHINY CICA 炭酸水 クレンジングフォーム 正規販売店 韓国コスメ 韓国化粧品 美肌 済州島 クレンザー スキンケア 素肌 高密度</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>SHINY Cosmetic</t>
+        </is>
+      </c>
+      <c r="F438" t="n">
+        <v>3245</v>
+      </c>
+      <c r="G438" t="n">
+        <v>1</v>
+      </c>
+      <c r="H438" t="b">
+        <v>0</v>
+      </c>
+      <c r="I438" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J438" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199807022</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J437"/>
+  <autoFilter ref="A1:J438"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 14)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$450</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$452</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J450"/>
+  <dimension ref="A1:J452"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16687,7 +16687,7 @@
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>LABASOME</t>
+          <t>LAVASOME</t>
         </is>
       </c>
       <c r="C400" t="inlineStr">
@@ -16704,7 +16704,7 @@
         <v>5900</v>
       </c>
       <c r="G400" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H400" t="b">
         <v>0</v>
@@ -18770,8 +18770,90 @@
         </is>
       </c>
     </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>1087980274</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>carabeautyconcierge</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>ディアテック ウクワ UKUWA モイストプラス 100g【3個セット】</t>
+        </is>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>ディアテック</t>
+        </is>
+      </c>
+      <c r="F451" t="n">
+        <v>4500</v>
+      </c>
+      <c r="G451" t="n">
+        <v>7</v>
+      </c>
+      <c r="H451" t="b">
+        <v>0</v>
+      </c>
+      <c r="I451" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J451" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1087980274</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>1087980242</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>carabeautyconcierge</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>ディアテック ウクワ UKUWA モイストプラス 100g　【2個セット】</t>
+        </is>
+      </c>
+      <c r="E452" t="inlineStr">
+        <is>
+          <t>ディアテック</t>
+        </is>
+      </c>
+      <c r="F452" t="n">
+        <v>3300</v>
+      </c>
+      <c r="G452" t="n">
+        <v>4</v>
+      </c>
+      <c r="H452" t="b">
+        <v>0</v>
+      </c>
+      <c r="I452" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J452" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1087980242</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J450"/>
+  <autoFilter ref="A1:J452"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 6)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$459</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$460</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J459"/>
+  <dimension ref="A1:J460"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19139,8 +19139,49 @@
         </is>
       </c>
     </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>1203606043</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>seaable</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>【トライアルセット6種組】シャンプートリートメントセット(バスグロウ3種/スーパーリッチクリスタル3種）6種各1枚 お試しサシェ6回分10mL+10mL 携帯用 旅行用</t>
+        </is>
+      </c>
+      <c r="E460" t="inlineStr">
+        <is>
+          <t>ラックス</t>
+        </is>
+      </c>
+      <c r="F460" t="n">
+        <v>860</v>
+      </c>
+      <c r="G460" t="n">
+        <v>0</v>
+      </c>
+      <c r="H460" t="b">
+        <v>0</v>
+      </c>
+      <c r="I460" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J460" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203606043</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J459"/>
+  <autoFilter ref="A1:J460"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 10, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$461</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$464</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J461"/>
+  <dimension ref="A1:J464"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19221,8 +19221,131 @@
         </is>
       </c>
     </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>1089747800</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>crossplus</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>ellips ヘアオイル シャイニーブラック(ピーチ＆シトラスの香り)50粒入 正規品 洗い流さないトリートメント ヘアビタミン 保湿 持ち運び ハリ コシ 潤い ツヤ 黒髪</t>
+        </is>
+      </c>
+      <c r="E462" t="inlineStr">
+        <is>
+          <t>エリップス</t>
+        </is>
+      </c>
+      <c r="F462" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G462" t="n">
+        <v>7</v>
+      </c>
+      <c r="H462" t="b">
+        <v>0</v>
+      </c>
+      <c r="I462" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J462" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1089747800</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>1089750324</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>crossplus</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>ellips ヘアオイル レディシャイニー(スウィートフローラルブーケの香り)50粒入 日本限定 正規品 洗い流さないトリートメント 保湿 持ち運び ハリ コシ 切毛 枝毛 ダメージケア ツヤ</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>エリップス</t>
+        </is>
+      </c>
+      <c r="F463" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G463" t="n">
+        <v>9</v>
+      </c>
+      <c r="H463" t="b">
+        <v>0</v>
+      </c>
+      <c r="I463" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J463" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1089750324</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>1089173212</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>crossplus</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>ellips ヘアオイル スムース&amp;amp;シャイニー(トロピカルフルーツの香り)50粒入 正規品 洗い流さないトリートメント ヘアビタミン サラサラ 持ち運び ダメージケア 保湿 潤い</t>
+        </is>
+      </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>エリップス</t>
+        </is>
+      </c>
+      <c r="F464" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G464" t="n">
+        <v>6</v>
+      </c>
+      <c r="H464" t="b">
+        <v>0</v>
+      </c>
+      <c r="I464" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J464" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1089173212</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J461"/>
+  <autoFilter ref="A1:J464"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 12)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$476</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$482</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J476"/>
+  <dimension ref="A1:J482"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19836,8 +19836,254 @@
         </is>
       </c>
     </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>1213011435</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>eightpointone</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>ルティナー 15ml スリープクリーム スリープバーム</t>
+        </is>
+      </c>
+      <c r="E477" t="inlineStr">
+        <is>
+          <t>aXENDA</t>
+        </is>
+      </c>
+      <c r="F477" t="n">
+        <v>5462</v>
+      </c>
+      <c r="G477" t="n">
+        <v>0</v>
+      </c>
+      <c r="H477" t="b">
+        <v>0</v>
+      </c>
+      <c r="I477" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J477" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213011435</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>1148824099</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>HappyBGLD</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>【20%OFF 全ブランド跨ぎ割引】 イロン 当帰 トナー 500ml+マスクパックをプレゼント</t>
+        </is>
+      </c>
+      <c r="E478" t="inlineStr">
+        <is>
+          <t>ILLON</t>
+        </is>
+      </c>
+      <c r="F478" t="n">
+        <v>7790</v>
+      </c>
+      <c r="G478" t="n">
+        <v>9</v>
+      </c>
+      <c r="H478" t="b">
+        <v>0</v>
+      </c>
+      <c r="I478" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J478" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1148824099</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>1102128974</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>HappyBGLD</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>【20%OFF 全ブランド跨ぎ割引】ボラヨン ヒアロテン パウダー(水分/鎮静) クーリングモデリングパック 500g+パック道具+ マスクパック追加贈呈</t>
+        </is>
+      </c>
+      <c r="E479" t="inlineStr">
+        <is>
+          <t>volayon</t>
+        </is>
+      </c>
+      <c r="F479" t="n">
+        <v>4199</v>
+      </c>
+      <c r="G479" t="n">
+        <v>4</v>
+      </c>
+      <c r="H479" t="b">
+        <v>0</v>
+      </c>
+      <c r="I479" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J479" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1102128974</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>1211561315</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>HappyBGLD</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>【20%OFF 全ブランド跨ぎ割引】油水分バランスパッケージ / スキャルプシャンプー 500ml + ブラックトリートメント 500ml +マスクパックをプレゼント</t>
+        </is>
+      </c>
+      <c r="E480" t="inlineStr">
+        <is>
+          <t>KEMA</t>
+        </is>
+      </c>
+      <c r="F480" t="n">
+        <v>13890</v>
+      </c>
+      <c r="G480" t="n">
+        <v>0</v>
+      </c>
+      <c r="H480" t="b">
+        <v>0</v>
+      </c>
+      <c r="I480" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J480" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211561315</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>1211067492</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>HappyBGLD</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>【20%OFF 全ブランド跨ぎ割引】スキンボリック ゴールドカプセル 100ml 高濃度の保湿ハリシワ改善アンプル+マスクパックをプレゼント</t>
+        </is>
+      </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>SKINBOLIC</t>
+        </is>
+      </c>
+      <c r="F481" t="n">
+        <v>19100</v>
+      </c>
+      <c r="G481" t="n">
+        <v>0</v>
+      </c>
+      <c r="H481" t="b">
+        <v>0</v>
+      </c>
+      <c r="I481" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J481" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211067492</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>1210939334</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>HappyBGLD</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>【20%OFF 全ブランド跨ぎ割引】オルソミンC ルミジアンプル (15ml) 40% 高濃度の純粋ビタミンCを含有+マスクパックをプレゼント</t>
+        </is>
+      </c>
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>VEMONTES</t>
+        </is>
+      </c>
+      <c r="F482" t="n">
+        <v>5790</v>
+      </c>
+      <c r="G482" t="n">
+        <v>0</v>
+      </c>
+      <c r="H482" t="b">
+        <v>0</v>
+      </c>
+      <c r="I482" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J482" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210939334</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J476"/>
+  <autoFilter ref="A1:J482"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 13)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$482</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$489</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J482"/>
+  <dimension ref="A1:J489"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20082,8 +20082,295 @@
         </is>
       </c>
     </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>1168247824</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>manmulsang</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>チョンギダン ファヒョン バランサー 5ml×30個 韓方化粧水 高保湿 ハリ ツヤ 個包装 韓国コスメ サンプル</t>
+        </is>
+      </c>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>THE WHOO</t>
+        </is>
+      </c>
+      <c r="F483" t="n">
+        <v>2009</v>
+      </c>
+      <c r="G483" t="n">
+        <v>0</v>
+      </c>
+      <c r="H483" t="b">
+        <v>0</v>
+      </c>
+      <c r="I483" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J483" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168247824</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>1123203922</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>manmulsang</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>【大容量セット】[1+1]カラーフィット ヘアシャンプー 1000ml/トリートメント1000ml カラーケア用 韓国ヘアケア 毎日使える ダメージ補修 保湿 ツヤ髪ケア</t>
+        </is>
+      </c>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>LODEURLETTE</t>
+        </is>
+      </c>
+      <c r="F484" t="n">
+        <v>4694</v>
+      </c>
+      <c r="G484" t="n">
+        <v>1</v>
+      </c>
+      <c r="H484" t="b">
+        <v>0</v>
+      </c>
+      <c r="I484" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J484" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1123203922</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>1106987513</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>manmulsang</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>[1+1]タイムエナジーリセッティングトナー170mL / エマルジョン120mL 化粧水・乳液セット 保湿・ハリ・ツヤケア 韓国スキンケア</t>
+        </is>
+      </c>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>sum37</t>
+        </is>
+      </c>
+      <c r="F485" t="n">
+        <v>5901</v>
+      </c>
+      <c r="G485" t="n">
+        <v>0</v>
+      </c>
+      <c r="H485" t="b">
+        <v>0</v>
+      </c>
+      <c r="I485" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J485" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1106987513</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>1081525647</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>manmulsang</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>拱辰享フォーム クレンザー 2ml 120個 韓国コスメ 洗顔フォーム 個包装 サンプル パウチ 旅行用 スキンケア</t>
+        </is>
+      </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>THE WHOO</t>
+        </is>
+      </c>
+      <c r="F486" t="n">
+        <v>2161</v>
+      </c>
+      <c r="G486" t="n">
+        <v>4</v>
+      </c>
+      <c r="H486" t="b">
+        <v>0</v>
+      </c>
+      <c r="I486" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J486" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1081525647</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>1212873959</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>refill</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>フォリゲン シックニング スカルプトニック 120ml 2個 韓国頭皮ケア 髪のハリコシケア ボリューム感ケア</t>
+        </is>
+      </c>
+      <c r="E487" t="inlineStr">
+        <is>
+          <t>Dr.FORHAIR</t>
+        </is>
+      </c>
+      <c r="F487" t="n">
+        <v>4299</v>
+      </c>
+      <c r="G487" t="n">
+        <v>0</v>
+      </c>
+      <c r="H487" t="b">
+        <v>0</v>
+      </c>
+      <c r="I487" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J487" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212873959</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>1212719705</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>refill</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>グルタハイヤ セラム ボディローション フローレスブライト 300ml 韓国ボディケア 保湿ローション 明るいツヤ肌印象</t>
+        </is>
+      </c>
+      <c r="E488" t="inlineStr">
+        <is>
+          <t>ヴァセリン</t>
+        </is>
+      </c>
+      <c r="F488" t="n">
+        <v>1950</v>
+      </c>
+      <c r="G488" t="n">
+        <v>0</v>
+      </c>
+      <c r="H488" t="b">
+        <v>0</v>
+      </c>
+      <c r="I488" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J488" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212719705</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>1212719275</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>refill</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>グルタハイヤ セラム ボディローション プロエイジリストア 300ml 韓国ボディケア 保湿ローション しっとりハリツヤ肌印象</t>
+        </is>
+      </c>
+      <c r="E489" t="inlineStr">
+        <is>
+          <t>ヴァセリン</t>
+        </is>
+      </c>
+      <c r="F489" t="n">
+        <v>1950</v>
+      </c>
+      <c r="G489" t="n">
+        <v>0</v>
+      </c>
+      <c r="H489" t="b">
+        <v>0</v>
+      </c>
+      <c r="I489" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J489" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212719275</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J482"/>
+  <autoFilter ref="A1:J489"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 16)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$493</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$499</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J493"/>
+  <dimension ref="A1:J499"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20533,8 +20533,254 @@
         </is>
       </c>
     </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>1209836455</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>k-essential</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>VT PDRN美容液2ml 6個入り 4箱 セット 韓国 SNS人気 美容液 エッセンス スキンケア コスメ 保湿 潤い ハリ ツヤ 弾力 キメ ツヤ肌 トラブル肌 乾燥肌 敏感肌 デイリーケア</t>
+        </is>
+      </c>
+      <c r="E494" t="inlineStr">
+        <is>
+          <t>ダイソー</t>
+        </is>
+      </c>
+      <c r="F494" t="n">
+        <v>2990</v>
+      </c>
+      <c r="G494" t="n">
+        <v>0</v>
+      </c>
+      <c r="H494" t="b">
+        <v>0</v>
+      </c>
+      <c r="I494" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J494" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209836455</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>1197118760</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>k-essential</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>ボディローション 520ml 1+1セット ホワイトムスク 香り 大容量 保湿 ボディミルク ボディケア 乾燥肌 しっとり べたつかない ポンプ式 全身 潤い 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E495" t="inlineStr">
+        <is>
+          <t>ブーケガルニ</t>
+        </is>
+      </c>
+      <c r="F495" t="n">
+        <v>3990</v>
+      </c>
+      <c r="G495" t="n">
+        <v>0</v>
+      </c>
+      <c r="H495" t="b">
+        <v>0</v>
+      </c>
+      <c r="I495" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J495" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197118760</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>1209992767</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>k-essential</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>足を洗おう 385ml フットシャンプー 泡 足の臭い 対策 角質 ケア 足洗い ソープ 爽快 バブル フットウォッシャー スプレー 足裏 洗浄 すっきり 潤い 保湿 フットケア ニオイ</t>
+        </is>
+      </c>
+      <c r="E496" t="inlineStr">
+        <is>
+          <t>オン・ザ・ボディー</t>
+        </is>
+      </c>
+      <c r="F496" t="n">
+        <v>1340</v>
+      </c>
+      <c r="G496" t="n">
+        <v>0</v>
+      </c>
+      <c r="H496" t="b">
+        <v>0</v>
+      </c>
+      <c r="I496" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J496" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209992767</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>1214125215</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>k-pick72811</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>[トーン&amp;amp;スポット][正規品]トーン＆スポット リカバリークリーム 80ml（ボディ美白/色素沈着ケア/背中ニキビ/ツヤ肌/大容量）</t>
+        </is>
+      </c>
+      <c r="E497" t="inlineStr">
+        <is>
+          <t>Redence</t>
+        </is>
+      </c>
+      <c r="F497" t="n">
+        <v>6284</v>
+      </c>
+      <c r="G497" t="n">
+        <v>0</v>
+      </c>
+      <c r="H497" t="b">
+        <v>0</v>
+      </c>
+      <c r="I497" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J497" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1214125215</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>1209488237</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>k-pick72811</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>[正規品][1+1+1]アクネ クレンジングフォーム 20ml／ニキビ機能性／緑茶水鎮静／ニキビ1位</t>
+        </is>
+      </c>
+      <c r="E498" t="inlineStr">
+        <is>
+          <t>ブランネイチャー</t>
+        </is>
+      </c>
+      <c r="F498" t="n">
+        <v>2924</v>
+      </c>
+      <c r="G498" t="n">
+        <v>0</v>
+      </c>
+      <c r="H498" t="b">
+        <v>0</v>
+      </c>
+      <c r="I498" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J498" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209488237</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>1204254720</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>k-pick72811</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>[ウォーターミストプランピング][正規品] マダガスカル センテラ ヒアル-テカ プランピング アンプル 50ml／スキンブースティング／ヒアルプラム</t>
+        </is>
+      </c>
+      <c r="E499" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F499" t="n">
+        <v>5743</v>
+      </c>
+      <c r="G499" t="n">
+        <v>0</v>
+      </c>
+      <c r="H499" t="b">
+        <v>0</v>
+      </c>
+      <c r="I499" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J499" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204254720</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J493"/>
+  <autoFilter ref="A1:J499"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 17)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$499</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$501</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J499"/>
+  <dimension ref="A1:J501"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20779,8 +20779,90 @@
         </is>
       </c>
     </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>1190163642</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>happybear</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>PDRN ヒアルロン酸 モイストカプセルミスト 100ml / 30ml 選択1</t>
+        </is>
+      </c>
+      <c r="E500" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F500" t="n">
+        <v>1990</v>
+      </c>
+      <c r="G500" t="n">
+        <v>0</v>
+      </c>
+      <c r="H500" t="b">
+        <v>0</v>
+      </c>
+      <c r="I500" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J500" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190163642</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>1152733985</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>happybear</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>46cm 弱酸性 デオドラント ボディウォッシュ 600ML(SPARKLING CITRUS / REFRESHING HERBAL / CLEAN SOAP)</t>
+        </is>
+      </c>
+      <c r="E501" t="inlineStr">
+        <is>
+          <t>オン・ザ・ボディー</t>
+        </is>
+      </c>
+      <c r="F501" t="n">
+        <v>2270</v>
+      </c>
+      <c r="G501" t="n">
+        <v>0</v>
+      </c>
+      <c r="H501" t="b">
+        <v>0</v>
+      </c>
+      <c r="I501" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J501" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1152733985</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J499"/>
+  <autoFilter ref="A1:J501"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 13, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$530</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$533</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J530"/>
+  <dimension ref="A1:J533"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22050,8 +22050,131 @@
         </is>
       </c>
     </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>1190555877</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>Kbeauty_store</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>マスティナ マスティック シックス アワース アンプル 15ml</t>
+        </is>
+      </c>
+      <c r="E531" t="inlineStr">
+        <is>
+          <t>mastina</t>
+        </is>
+      </c>
+      <c r="F531" t="n">
+        <v>2140</v>
+      </c>
+      <c r="G531" t="n">
+        <v>0</v>
+      </c>
+      <c r="H531" t="b">
+        <v>0</v>
+      </c>
+      <c r="I531" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J531" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190555877</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>1201899429</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>Kbeauty_store</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>ドクダミ 70 スージング コラーゲン マスク 4枚</t>
+        </is>
+      </c>
+      <c r="E532" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F532" t="n">
+        <v>2750</v>
+      </c>
+      <c r="G532" t="n">
+        <v>1</v>
+      </c>
+      <c r="H532" t="b">
+        <v>0</v>
+      </c>
+      <c r="I532" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J532" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201899429</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>1204813717</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>Kbeauty_store</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>大容量トナー ツボクサ グリーンダーマ マイルド シカ ビッグトナー 500ml</t>
+        </is>
+      </c>
+      <c r="E533" t="inlineStr">
+        <is>
+          <t>ネイチャーリパブリック</t>
+        </is>
+      </c>
+      <c r="F533" t="n">
+        <v>3424</v>
+      </c>
+      <c r="G533" t="n">
+        <v>3</v>
+      </c>
+      <c r="H533" t="b">
+        <v>0</v>
+      </c>
+      <c r="I533" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J533" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204813717</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J530"/>
+  <autoFilter ref="A1:J533"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 17, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$540</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$542</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J540"/>
+  <dimension ref="A1:J542"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22460,8 +22460,90 @@
         </is>
       </c>
     </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>1208828941</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>doctorbio</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>【公式】NEW ブルーアガベスージングジェル 200g [ひんやり保湿 敏感肌対応 潤いケア</t>
+        </is>
+      </c>
+      <c r="E541" t="inlineStr">
+        <is>
+          <t>Dr.Bio</t>
+        </is>
+      </c>
+      <c r="F541" t="n">
+        <v>2180</v>
+      </c>
+      <c r="G541" t="n">
+        <v>2</v>
+      </c>
+      <c r="H541" t="b">
+        <v>0</v>
+      </c>
+      <c r="I541" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J541" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208828941</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>1174284175</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>doctorbio</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>【公式】グレープコラーゲン 毛穴タイトニングセラム&amp;amp;クリーム [葡萄 / コラーゲン / 美容液 / 毛穴レスケア/ ベタつかない使用感]</t>
+        </is>
+      </c>
+      <c r="E542" t="inlineStr">
+        <is>
+          <t>Dr.Bio</t>
+        </is>
+      </c>
+      <c r="F542" t="n">
+        <v>4760</v>
+      </c>
+      <c r="G542" t="n">
+        <v>7</v>
+      </c>
+      <c r="H542" t="b">
+        <v>0</v>
+      </c>
+      <c r="I542" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J542" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174284175</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J540"/>
+  <autoFilter ref="A1:J542"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 19, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$546</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$550</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J546"/>
+  <dimension ref="A1:J550"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22706,8 +22706,172 @@
         </is>
       </c>
     </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>1158950695</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>sizuccu</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>[1+1]エアリー フィット サンスティック 14g, 2個</t>
+        </is>
+      </c>
+      <c r="E547" t="inlineStr">
+        <is>
+          <t>KAHI</t>
+        </is>
+      </c>
+      <c r="F547" t="n">
+        <v>5400</v>
+      </c>
+      <c r="G547" t="n">
+        <v>0</v>
+      </c>
+      <c r="H547" t="b">
+        <v>0</v>
+      </c>
+      <c r="I547" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J547" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1158950695</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>1194502685</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>sizuccu</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>[NEW/透明ケア] スキン＆ラボ グルタチオントナー 200ml 1個</t>
+        </is>
+      </c>
+      <c r="E548" t="inlineStr">
+        <is>
+          <t>スキンアンドラブ</t>
+        </is>
+      </c>
+      <c r="F548" t="n">
+        <v>5100</v>
+      </c>
+      <c r="G548" t="n">
+        <v>0</v>
+      </c>
+      <c r="H548" t="b">
+        <v>0</v>
+      </c>
+      <c r="I548" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J548" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194502685</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>1187932783</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>sizuccu</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>[紫-PDRN毛穴弾力],今買うとお得な200枚チャンス PDRN 毛穴弾力 パッド 100枚+詰め替え 100枚</t>
+        </is>
+      </c>
+      <c r="E549" t="inlineStr">
+        <is>
+          <t>メディヒール</t>
+        </is>
+      </c>
+      <c r="F549" t="n">
+        <v>7210</v>
+      </c>
+      <c r="G549" t="n">
+        <v>0</v>
+      </c>
+      <c r="H549" t="b">
+        <v>0</v>
+      </c>
+      <c r="I549" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J549" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1187932783</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>1194387025</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>sizuccu</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>[簡単にサッと] ダブルセラム オールインワン マルチバーム 10g 1個/オールインワンスティック/ヴィーガンマルチバーム</t>
+        </is>
+      </c>
+      <c r="E550" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F550" t="n">
+        <v>4300</v>
+      </c>
+      <c r="G550" t="n">
+        <v>0</v>
+      </c>
+      <c r="H550" t="b">
+        <v>0</v>
+      </c>
+      <c r="I550" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J550" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194387025</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J546"/>
+  <autoFilter ref="A1:J550"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 22, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$553</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$557</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J553"/>
+  <dimension ref="A1:J557"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22993,8 +22993,172 @@
         </is>
       </c>
     </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>973486483</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>kstargoods_JP</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>[Pyunkang Yul] DEEP CLEANSING OIL</t>
+        </is>
+      </c>
+      <c r="E554" t="inlineStr">
+        <is>
+          <t>ブランドなし</t>
+        </is>
+      </c>
+      <c r="F554" t="n">
+        <v>2290</v>
+      </c>
+      <c r="G554" t="n">
+        <v>0</v>
+      </c>
+      <c r="H554" t="b">
+        <v>0</v>
+      </c>
+      <c r="I554" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J554" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=973486483</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>1083676754</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>kstargoods_JP</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>loccitane shea verbena liquid soap 300ml</t>
+        </is>
+      </c>
+      <c r="E555" t="inlineStr">
+        <is>
+          <t>ロクシタン</t>
+        </is>
+      </c>
+      <c r="F555" t="n">
+        <v>4999</v>
+      </c>
+      <c r="G555" t="n">
+        <v>0</v>
+      </c>
+      <c r="H555" t="b">
+        <v>0</v>
+      </c>
+      <c r="I555" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J555" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1083676754</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>969163642</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>kstargoods_JP</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>[Labelyoung] Shocking Vitamin Milk Whitening Cream</t>
+        </is>
+      </c>
+      <c r="E556" t="inlineStr">
+        <is>
+          <t>ラベルヤング</t>
+        </is>
+      </c>
+      <c r="F556" t="n">
+        <v>1899</v>
+      </c>
+      <c r="G556" t="n">
+        <v>4</v>
+      </c>
+      <c r="H556" t="b">
+        <v>0</v>
+      </c>
+      <c r="I556" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J556" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=969163642</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>821075839</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>kstargoods_JP</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>[THE SAEM] Urban Eco Harakeke Deep Moisture Toner</t>
+        </is>
+      </c>
+      <c r="E557" t="inlineStr">
+        <is>
+          <t>ブランドなし</t>
+        </is>
+      </c>
+      <c r="F557" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G557" t="n">
+        <v>0</v>
+      </c>
+      <c r="H557" t="b">
+        <v>0</v>
+      </c>
+      <c r="I557" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J557" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=821075839</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J553"/>
+  <autoFilter ref="A1:J557"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 25, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$559</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$560</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J559"/>
+  <dimension ref="A1:J560"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23239,8 +23239,49 @@
         </is>
       </c>
     </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>1053257413</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>daymellow_official</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>300ml+300ml/アクアロン ウォータリートナー+エマルジョン セット</t>
+        </is>
+      </c>
+      <c r="E560" t="inlineStr">
+        <is>
+          <t>デイメロウ</t>
+        </is>
+      </c>
+      <c r="F560" t="n">
+        <v>2880</v>
+      </c>
+      <c r="G560" t="n">
+        <v>5</v>
+      </c>
+      <c r="H560" t="b">
+        <v>0</v>
+      </c>
+      <c r="I560" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J560" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1053257413</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J559"/>
+  <autoFilter ref="A1:J560"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 26, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$560</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$561</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J560"/>
+  <dimension ref="A1:J561"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23280,8 +23280,49 @@
         </is>
       </c>
     </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>1168607816</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>pibumijp</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>センテルーション ナノシカ モイスチャークリーム 100ml 韓国コスメ /アトピー / かゆい肌/ 水分 / 潤い / 低刺激 乾燥肌 / 保湿クリーム</t>
+        </is>
+      </c>
+      <c r="E561" t="inlineStr">
+        <is>
+          <t>PIBUMI</t>
+        </is>
+      </c>
+      <c r="F561" t="n">
+        <v>2580</v>
+      </c>
+      <c r="G561" t="n">
+        <v>8</v>
+      </c>
+      <c r="H561" t="b">
+        <v>0</v>
+      </c>
+      <c r="I561" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J561" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168607816</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J560"/>
+  <autoFilter ref="A1:J561"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 28, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$563</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$565</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J563"/>
+  <dimension ref="A1:J565"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23403,8 +23403,90 @@
         </is>
       </c>
     </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>1213125468</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>niconicolife</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>日焼け止め SPF50+ PA++++ UVカット 紫外線対策 ソーラーDサンスクリーン Lion 顔 体用 強力UV 冬 乾燥対策 クリスマス プレゼント ギフト 40ml 100ml 選べる</t>
+        </is>
+      </c>
+      <c r="E564" t="inlineStr">
+        <is>
+          <t>Solar D</t>
+        </is>
+      </c>
+      <c r="F564" t="n">
+        <v>3060</v>
+      </c>
+      <c r="G564" t="n">
+        <v>1</v>
+      </c>
+      <c r="H564" t="b">
+        <v>0</v>
+      </c>
+      <c r="I564" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J564" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213125468</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>1209045783</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>m4-magic</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>プロバイオダーム コラーゲンリモデリング セラムパッド70枚 美容液 ハリ ツヤ 毛穴ケア －7－</t>
+        </is>
+      </c>
+      <c r="E565" t="inlineStr">
+        <is>
+          <t>バイオヒールボ</t>
+        </is>
+      </c>
+      <c r="F565" t="n">
+        <v>2340</v>
+      </c>
+      <c r="G565" t="n">
+        <v>0</v>
+      </c>
+      <c r="H565" t="b">
+        <v>0</v>
+      </c>
+      <c r="I565" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J565" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209045783</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J563"/>
+  <autoFilter ref="A1:J565"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 29, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$565</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$569</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J565"/>
+  <dimension ref="A1:J569"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23485,8 +23485,172 @@
         </is>
       </c>
     </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>1170355876</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>nextfield</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>ブレンディ スティック コーヒー カフェオレ(12gx100本入)【ブレンディ(Blendy)】</t>
+        </is>
+      </c>
+      <c r="E566" t="inlineStr">
+        <is>
+          <t>ブレンディ</t>
+        </is>
+      </c>
+      <c r="F566" t="n">
+        <v>3280</v>
+      </c>
+      <c r="G566" t="n">
+        <v>0</v>
+      </c>
+      <c r="H566" t="b">
+        <v>0</v>
+      </c>
+      <c r="I566" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J566" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1170355876</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>1214844125</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>HELLOJ</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>(パク・ボゴム脱毛アンプル)頭頂部脱毛アンプルポリジェンシックニング スカルプセラム50ml1個</t>
+        </is>
+      </c>
+      <c r="E567" t="inlineStr">
+        <is>
+          <t>Dr.FORHAIR</t>
+        </is>
+      </c>
+      <c r="F567" t="n">
+        <v>3299</v>
+      </c>
+      <c r="G567" t="n">
+        <v>0</v>
+      </c>
+      <c r="H567" t="b">
+        <v>0</v>
+      </c>
+      <c r="I567" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J567" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1214844125</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>1214302245</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>HELLOJ</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>ラブセント スクラブ ボディウォッシュ 500ml 8種から選択</t>
+        </is>
+      </c>
+      <c r="E568" t="inlineStr">
+        <is>
+          <t>ケラシス</t>
+        </is>
+      </c>
+      <c r="F568" t="n">
+        <v>1580</v>
+      </c>
+      <c r="G568" t="n">
+        <v>0</v>
+      </c>
+      <c r="H568" t="b">
+        <v>0</v>
+      </c>
+      <c r="I568" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J568" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1214302245</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>1208232494</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>HELLOJ</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>プリティスキン アンプルマスクパック 50P / シカ / コラーゲン / PDRN</t>
+        </is>
+      </c>
+      <c r="E569" t="inlineStr">
+        <is>
+          <t>プリティースキン</t>
+        </is>
+      </c>
+      <c r="F569" t="n">
+        <v>3750</v>
+      </c>
+      <c r="G569" t="n">
+        <v>0</v>
+      </c>
+      <c r="H569" t="b">
+        <v>0</v>
+      </c>
+      <c r="I569" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J569" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208232494</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J565"/>
+  <autoFilter ref="A1:J569"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 31, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$572</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$573</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J572"/>
+  <dimension ref="A1:J573"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23772,8 +23772,49 @@
         </is>
       </c>
     </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>1174515889</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>modehana</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>新芽のヨモギ 水分ヨモギヒアルクリーム 60ml/韓国 コスメ/皮脂/ 弾力/ 保湿/ 水分/テカリ/ 乾燥肌/顔肌/ 美容/ スキンケア</t>
+        </is>
+      </c>
+      <c r="E573" t="inlineStr">
+        <is>
+          <t>ハンユル</t>
+        </is>
+      </c>
+      <c r="F573" t="n">
+        <v>3494</v>
+      </c>
+      <c r="G573" t="n">
+        <v>1</v>
+      </c>
+      <c r="H573" t="b">
+        <v>0</v>
+      </c>
+      <c r="I573" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J573" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174515889</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J572"/>
+  <autoFilter ref="A1:J573"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 35, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$577</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$579</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J577"/>
+  <dimension ref="A1:J579"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -23977,8 +23977,90 @@
         </is>
       </c>
     </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>1211986132</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>JUNO_korea</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>【うるおい/ハリ肌】SKIN 100 4センテラ TECA アンプル 50ml</t>
+        </is>
+      </c>
+      <c r="E578" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F578" t="n">
+        <v>2990</v>
+      </c>
+      <c r="G578" t="n">
+        <v>0</v>
+      </c>
+      <c r="H578" t="b">
+        <v>0</v>
+      </c>
+      <c r="I578" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J578" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211986132</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>1203288896</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>JUNO_korea</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>T FITトランスルーセント セットサンパウダー 7g（UVケア/さらさら肌）</t>
+        </is>
+      </c>
+      <c r="E579" t="inlineStr">
+        <is>
+          <t>TFIT</t>
+        </is>
+      </c>
+      <c r="F579" t="n">
+        <v>2750</v>
+      </c>
+      <c r="G579" t="n">
+        <v>2</v>
+      </c>
+      <c r="H579" t="b">
+        <v>0</v>
+      </c>
+      <c r="I579" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J579" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203288896</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J577"/>
+  <autoFilter ref="A1:J579"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 38, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$580</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$585</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J580"/>
+  <dimension ref="A1:J585"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24100,8 +24100,213 @@
         </is>
       </c>
     </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>1206679102</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>RETURNITY</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>【公式】スキンヒーラーカプセルアンプルゲル 60ml</t>
+        </is>
+      </c>
+      <c r="E581" t="inlineStr">
+        <is>
+          <t>RETURNITY</t>
+        </is>
+      </c>
+      <c r="F581" t="n">
+        <v>999</v>
+      </c>
+      <c r="G581" t="n">
+        <v>2</v>
+      </c>
+      <c r="H581" t="b">
+        <v>0</v>
+      </c>
+      <c r="I581" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J581" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206679102</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>1206757350</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>RETURNITY</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>【公式】スキンヒーラーウォータートナー 300ml</t>
+        </is>
+      </c>
+      <c r="E582" t="inlineStr">
+        <is>
+          <t>RETURNITY</t>
+        </is>
+      </c>
+      <c r="F582" t="n">
+        <v>3200</v>
+      </c>
+      <c r="G582" t="n">
+        <v>4</v>
+      </c>
+      <c r="H582" t="b">
+        <v>0</v>
+      </c>
+      <c r="I582" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J582" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206757350</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>1195854561</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>mayjoy</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>マデカソルケア軟膏ニキビ擦り傷用のマデカソルクリームツボクサエキスネオマイシン配合韓国ソウル産</t>
+        </is>
+      </c>
+      <c r="E583" t="inlineStr">
+        <is>
+          <t>東国製薬</t>
+        </is>
+      </c>
+      <c r="F583" t="n">
+        <v>890</v>
+      </c>
+      <c r="G583" t="n">
+        <v>1</v>
+      </c>
+      <c r="H583" t="b">
+        <v>0</v>
+      </c>
+      <c r="I583" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J583" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195854561</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>1195851257</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>mayjoy</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>ドンア メラノサクリーム 30g Melanosa ハイドロキノン4%配合シミ・そばかす・黒ずみ・老人性色素斑用 / 韓国ソウル</t>
+        </is>
+      </c>
+      <c r="E584" t="inlineStr">
+        <is>
+          <t>東亜製薬</t>
+        </is>
+      </c>
+      <c r="F584" t="n">
+        <v>2690</v>
+      </c>
+      <c r="G584" t="n">
+        <v>4</v>
+      </c>
+      <c r="H584" t="b">
+        <v>0</v>
+      </c>
+      <c r="I584" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J584" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195851257</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>1168048606</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>mayjoy</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>Melatoning クリーム 大容量 50g 変色した肌そばかす肝斑メラニン色素沈着用 / 韓国ソウル発</t>
+        </is>
+      </c>
+      <c r="E585" t="inlineStr">
+        <is>
+          <t>東亜製薬</t>
+        </is>
+      </c>
+      <c r="F585" t="n">
+        <v>2390</v>
+      </c>
+      <c r="G585" t="n">
+        <v>9</v>
+      </c>
+      <c r="H585" t="b">
+        <v>0</v>
+      </c>
+      <c r="I585" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J585" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168048606</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J580"/>
+  <autoFilter ref="A1:J585"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 40, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$586</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$589</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J586"/>
+  <dimension ref="A1:J589"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24346,8 +24346,131 @@
         </is>
       </c>
     </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>1184489510</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>luckybravo</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>[2個セット] ミルキープレシャス EXリペア シャンプー ヘアトリートメント セット 詰替 ヘアケア 詰め替え [ギフトラッピング対応]</t>
+        </is>
+      </c>
+      <c r="E587" t="inlineStr">
+        <is>
+          <t>アンドハニー</t>
+        </is>
+      </c>
+      <c r="F587" t="n">
+        <v>2331</v>
+      </c>
+      <c r="G587" t="n">
+        <v>0</v>
+      </c>
+      <c r="H587" t="b">
+        <v>0</v>
+      </c>
+      <c r="I587" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J587" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1184489510</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>1068877755</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>luckybravo</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>[組合せ自由][2個セット] ディープリペア シャンプー ヘアトリートメント モイスト 本体 詰め替え用[4種類から選べる] アクアブロッサムハニーの香り[ギフトラッピング対応]</t>
+        </is>
+      </c>
+      <c r="E588" t="inlineStr">
+        <is>
+          <t>HONEYQUE</t>
+        </is>
+      </c>
+      <c r="F588" t="n">
+        <v>2580</v>
+      </c>
+      <c r="G588" t="n">
+        <v>0</v>
+      </c>
+      <c r="H588" t="b">
+        <v>0</v>
+      </c>
+      <c r="I588" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J588" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1068877755</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>1126331306</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>pront-express</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>plus eau (プリュスオー) メルティバーム 40g ホワイトフローラル&amp;amp;ペアーの香り ヘアバーム スタイリング剤</t>
+        </is>
+      </c>
+      <c r="E589" t="inlineStr">
+        <is>
+          <t>Plus more</t>
+        </is>
+      </c>
+      <c r="F589" t="n">
+        <v>2467</v>
+      </c>
+      <c r="G589" t="n">
+        <v>0</v>
+      </c>
+      <c r="H589" t="b">
+        <v>0</v>
+      </c>
+      <c r="I589" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J589" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1126331306</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J586"/>
+  <autoFilter ref="A1:J589"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 41, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$589</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$590</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J589"/>
+  <dimension ref="A1:J590"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24469,8 +24469,49 @@
         </is>
       </c>
     </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>1196396285</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>luxekosme</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>[組合せ自由][2個セット]スムース モイスト シャンプー トリートメント 詰め替え用 380ml $ヘアケア ツヤ髪 摩擦 $[ギフトラッピング対応]</t>
+        </is>
+      </c>
+      <c r="E590" t="inlineStr">
+        <is>
+          <t>メルト</t>
+        </is>
+      </c>
+      <c r="F590" t="n">
+        <v>2898</v>
+      </c>
+      <c r="G590" t="n">
+        <v>1</v>
+      </c>
+      <c r="H590" t="b">
+        <v>0</v>
+      </c>
+      <c r="I590" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J590" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196396285</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J589"/>
+  <autoFilter ref="A1:J590"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 43, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$593</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$594</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J593"/>
+  <dimension ref="A1:J594"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24633,8 +24633,49 @@
         </is>
       </c>
     </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>983100128</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>SICosmetics</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>ボディファンタジーボディスプレートワイライトミスト / 3個 / 236ml</t>
+        </is>
+      </c>
+      <c r="E594" t="inlineStr">
+        <is>
+          <t>ボディファンタジー</t>
+        </is>
+      </c>
+      <c r="F594" t="n">
+        <v>5301</v>
+      </c>
+      <c r="G594" t="n">
+        <v>1</v>
+      </c>
+      <c r="H594" t="b">
+        <v>0</v>
+      </c>
+      <c r="I594" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J594" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=983100128</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J593"/>
+  <autoFilter ref="A1:J594"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 44, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$594</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$602</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J594"/>
+  <dimension ref="A1:J602"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24674,8 +24674,336 @@
         </is>
       </c>
     </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>1211988367</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>kiseki-trend</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>ミルボン エルジューダ ポイントケアスティック 15ml アホ毛ケア 前髪キープ 浮き毛 おくれ毛 まとめ髪 ヘアスティック スタイリング</t>
+        </is>
+      </c>
+      <c r="E595" t="inlineStr">
+        <is>
+          <t>ミルボン</t>
+        </is>
+      </c>
+      <c r="F595" t="n">
+        <v>1087</v>
+      </c>
+      <c r="G595" t="n">
+        <v>0</v>
+      </c>
+      <c r="H595" t="b">
+        <v>0</v>
+      </c>
+      <c r="I595" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J595" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211988367</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>1196515028</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>kiseki-trend</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>ミルボン ジェミールフラン メルティバター 100g セット 洗い流さない トリートメント アウトバス 美容室 サロン</t>
+        </is>
+      </c>
+      <c r="E596" t="inlineStr">
+        <is>
+          <t>ミルボン</t>
+        </is>
+      </c>
+      <c r="F596" t="n">
+        <v>1720</v>
+      </c>
+      <c r="G596" t="n">
+        <v>0</v>
+      </c>
+      <c r="H596" t="b">
+        <v>0</v>
+      </c>
+      <c r="I596" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J596" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196515028</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>1186587839</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>kiseki-trend</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>Promille プロミルオイル ヘアオイル 150ml / 50ml ヘアケア 保湿 ツヤ まとまり スタイリングオイル 人気 ヘアケア オイル 日本製</t>
+        </is>
+      </c>
+      <c r="E597" t="inlineStr">
+        <is>
+          <t>ムコタ</t>
+        </is>
+      </c>
+      <c r="F597" t="n">
+        <v>1339</v>
+      </c>
+      <c r="G597" t="n">
+        <v>0</v>
+      </c>
+      <c r="H597" t="b">
+        <v>0</v>
+      </c>
+      <c r="I597" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J597" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1186587839</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>1192837627</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>orange-store</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>追跡あり A Q U A L A B E L エステ洗顔ジェル 130g 資生堂 毛穴汚れ 角質ケア うるおい洗顔 日本製</t>
+        </is>
+      </c>
+      <c r="E598" t="inlineStr">
+        <is>
+          <t>アクアレーベル</t>
+        </is>
+      </c>
+      <c r="F598" t="n">
+        <v>1360</v>
+      </c>
+      <c r="G598" t="n">
+        <v>3</v>
+      </c>
+      <c r="H598" t="b">
+        <v>0</v>
+      </c>
+      <c r="I598" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J598" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192837627</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>1190293015</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>orange-store</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>追跡あり M I N O N ブライトアップベース UV ナチュラルベージュ 25g 化粧下地 日焼け止め 敏感肌 乾燥肌</t>
+        </is>
+      </c>
+      <c r="E599" t="inlineStr">
+        <is>
+          <t>ミノンアミノモイスト</t>
+        </is>
+      </c>
+      <c r="F599" t="n">
+        <v>1418</v>
+      </c>
+      <c r="G599" t="n">
+        <v>1</v>
+      </c>
+      <c r="H599" t="b">
+        <v>0</v>
+      </c>
+      <c r="I599" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J599" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190293015</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>1181290025</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>orange-store</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>追跡あり スーパーモイスチャーUVライトアップエッセンス 70g 日焼け止め SPF50+ PA++++ ロート製薬</t>
+        </is>
+      </c>
+      <c r="E600" t="inlineStr">
+        <is>
+          <t>スキンアクア</t>
+        </is>
+      </c>
+      <c r="F600" t="n">
+        <v>662</v>
+      </c>
+      <c r="G600" t="n">
+        <v>0</v>
+      </c>
+      <c r="H600" t="b">
+        <v>0</v>
+      </c>
+      <c r="I600" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J600" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1181290025</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>1137388674</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>orange-store</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>2個セット アクアレーベル アクアローション 220ml しっとり 化粧水</t>
+        </is>
+      </c>
+      <c r="E601" t="inlineStr">
+        <is>
+          <t>資生堂</t>
+        </is>
+      </c>
+      <c r="F601" t="n">
+        <v>2750</v>
+      </c>
+      <c r="G601" t="n">
+        <v>0</v>
+      </c>
+      <c r="H601" t="b">
+        <v>0</v>
+      </c>
+      <c r="I601" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J601" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1137388674</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>1135820839</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>orange-store</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>追跡あり 並行輸入品 モイスチャークリーム ミニ 30ml フェイスクリーム 保湿 化粧下地</t>
+        </is>
+      </c>
+      <c r="E602" t="inlineStr">
+        <is>
+          <t>アンブリオリス</t>
+        </is>
+      </c>
+      <c r="F602" t="n">
+        <v>1570</v>
+      </c>
+      <c r="G602" t="n">
+        <v>1</v>
+      </c>
+      <c r="H602" t="b">
+        <v>0</v>
+      </c>
+      <c r="I602" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J602" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1135820839</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J594"/>
+  <autoFilter ref="A1:J602"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 46, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$604</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$607</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J604"/>
+  <dimension ref="A1:J607"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25084,8 +25084,131 @@
         </is>
       </c>
     </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>1062061074</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>zeromode</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>SHEZI 奢姿 日焼け止めクリーム 奢姿瑞嘉防晒霜 SPF30 化粧品 中国コスメ 中国変身メイク チャイボーク メイク TikTokで話題の商品</t>
+        </is>
+      </c>
+      <c r="E605" t="inlineStr">
+        <is>
+          <t>SHEZI</t>
+        </is>
+      </c>
+      <c r="F605" t="n">
+        <v>1480</v>
+      </c>
+      <c r="G605" t="n">
+        <v>4</v>
+      </c>
+      <c r="H605" t="b">
+        <v>0</v>
+      </c>
+      <c r="I605" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J605" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1062061074</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>1214231575</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>winwinlife1</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>ネコポス速達！フェイシャル トリートメント セラム 0.6ml*3枚 お試しセット サシェサンプル トラベルサイズ 美容液 スキンケア ツヤ ハリ モチ キレイロック 革新技術 濃縮成分</t>
+        </is>
+      </c>
+      <c r="E606" t="inlineStr">
+        <is>
+          <t>SK-Ⅱ</t>
+        </is>
+      </c>
+      <c r="F606" t="n">
+        <v>1070</v>
+      </c>
+      <c r="G606" t="n">
+        <v>1</v>
+      </c>
+      <c r="H606" t="b">
+        <v>0</v>
+      </c>
+      <c r="I606" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J606" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1214231575</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>1210832292</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>winwinlife1</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>ネコポス速達！エクストラオーディナリ一オイル モイストミルク（洗い流さないヘアトリートメント）7ml*4枚 お試しセット サシェサンプル トラベルサイズ 貯水セラミド配合 インナードライ髪ケア</t>
+        </is>
+      </c>
+      <c r="E607" t="inlineStr">
+        <is>
+          <t>LOREAL PARIS</t>
+        </is>
+      </c>
+      <c r="F607" t="n">
+        <v>990</v>
+      </c>
+      <c r="G607" t="n">
+        <v>0</v>
+      </c>
+      <c r="H607" t="b">
+        <v>0</v>
+      </c>
+      <c r="I607" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J607" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210832292</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J604"/>
+  <autoFilter ref="A1:J607"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 47, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$607</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$609</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J607"/>
+  <dimension ref="A1:J609"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25207,8 +25207,90 @@
         </is>
       </c>
     </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>1212568942</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>winwinlife2</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>ネコポス速達！UVイデア XL プロテクショントーンアップ ティント（日焼け止め乳液・化粧下地）3ml 外箱付き フランス製 ミニサイズ 特製サイズ サンプル ゆらぐ大人肌に光カバー</t>
+        </is>
+      </c>
+      <c r="E608" t="inlineStr">
+        <is>
+          <t>ラロッシュポゼ</t>
+        </is>
+      </c>
+      <c r="F608" t="n">
+        <v>741</v>
+      </c>
+      <c r="G608" t="n">
+        <v>1</v>
+      </c>
+      <c r="H608" t="b">
+        <v>0</v>
+      </c>
+      <c r="I608" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J608" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212568942</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>1180167989</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>winwinlife2</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>明色化粧品 ダーマブーストセラム（美容液）30ml 高濃度美容成分 高保湿 うるおい コラーゲンエキス ハリ 弾力 透明感 高保湿 水光肌 肌のすみずみまで浸透 乾燥・肌荒れ防ぐ 肌の欠点改善</t>
+        </is>
+      </c>
+      <c r="E609" t="inlineStr">
+        <is>
+          <t>MEDI DERMA</t>
+        </is>
+      </c>
+      <c r="F609" t="n">
+        <v>1930</v>
+      </c>
+      <c r="G609" t="n">
+        <v>2</v>
+      </c>
+      <c r="H609" t="b">
+        <v>0</v>
+      </c>
+      <c r="I609" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J609" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180167989</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J607"/>
+  <autoFilter ref="A1:J609"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 55, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$611</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$612</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J611"/>
+  <dimension ref="A1:J612"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25371,8 +25371,49 @@
         </is>
       </c>
     </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>1135520115</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>aopapa</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>【公式】青パパイヤ酵素 シートマスク オリジナル 7枚セット バイオノーマライザー フェイスパック パック フェイスマスク 保湿 潤い スキンケア 酵素 美容液 無添加 ツヤ肌 キメ 敏感肌</t>
+        </is>
+      </c>
+      <c r="E612" t="inlineStr">
+        <is>
+          <t>青パパイヤ酵素</t>
+        </is>
+      </c>
+      <c r="F612" t="n">
+        <v>2970</v>
+      </c>
+      <c r="G612" t="n">
+        <v>2</v>
+      </c>
+      <c r="H612" t="b">
+        <v>0</v>
+      </c>
+      <c r="I612" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J612" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1135520115</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J611"/>
+  <autoFilter ref="A1:J612"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 56, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$612</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$616</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J612"/>
+  <dimension ref="A1:J616"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25412,8 +25412,172 @@
         </is>
       </c>
     </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>1194323430</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>js</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>【選べる】オージュア　シャンプー1000ml各種 詰め替え　クエンチ　クエンチモイスト　イミュライズ　タイムサージ インメトリィ　リペアリティ　フィルメロウ　エクイアル　ディオーラム　モイストカーム</t>
+        </is>
+      </c>
+      <c r="E613" t="inlineStr">
+        <is>
+          <t>オージュア</t>
+        </is>
+      </c>
+      <c r="F613" t="n">
+        <v>9200</v>
+      </c>
+      <c r="G613" t="n">
+        <v>1</v>
+      </c>
+      <c r="H613" t="b">
+        <v>0</v>
+      </c>
+      <c r="I613" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J613" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194323430</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>1194323429</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>js</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>【選べる】オージュア　トリートメント1000g各種 詰め替え　クエンチ　クエンチモイスト　イミュライズ　タイムサージ インメトリィ　リペアリティ　フィルメロウ　エクイアル　ディオーラム　モイストカーム</t>
+        </is>
+      </c>
+      <c r="E614" t="inlineStr">
+        <is>
+          <t>オージュア</t>
+        </is>
+      </c>
+      <c r="F614" t="n">
+        <v>11500</v>
+      </c>
+      <c r="G614" t="n">
+        <v>0</v>
+      </c>
+      <c r="H614" t="b">
+        <v>0</v>
+      </c>
+      <c r="I614" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J614" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194323429</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>1195074904</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>js</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>【正規品】フィヨーレ　クオルシア　カラーシャンプー　紫　purple　1000ml　【サロン専売品】【ブリーチケア】【カラーケア】【ムラシャン】【最安値更新中】【正規品】【色落ちケア】</t>
+        </is>
+      </c>
+      <c r="E615" t="inlineStr">
+        <is>
+          <t>フィヨーレ</t>
+        </is>
+      </c>
+      <c r="F615" t="n">
+        <v>5250</v>
+      </c>
+      <c r="G615" t="n">
+        <v>3</v>
+      </c>
+      <c r="H615" t="b">
+        <v>0</v>
+      </c>
+      <c r="I615" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J615" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195074904</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>1180483040</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>mycos</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>化粧水 ザ・タイムR アクア</t>
+        </is>
+      </c>
+      <c r="E616" t="inlineStr">
+        <is>
+          <t>イプサ</t>
+        </is>
+      </c>
+      <c r="F616" t="n">
+        <v>3550</v>
+      </c>
+      <c r="G616" t="n">
+        <v>6</v>
+      </c>
+      <c r="H616" t="b">
+        <v>0</v>
+      </c>
+      <c r="I616" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J616" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180483040</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J612"/>
+  <autoFilter ref="A1:J616"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 58, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$623</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$624</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J623"/>
+  <dimension ref="A1:J624"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25863,8 +25863,49 @@
         </is>
       </c>
     </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>1122581093</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>skymik</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>薬用ミスト 150ml</t>
+        </is>
+      </c>
+      <c r="E624" t="inlineStr">
+        <is>
+          <t>オードムーゲ</t>
+        </is>
+      </c>
+      <c r="F624" t="n">
+        <v>1148</v>
+      </c>
+      <c r="G624" t="n">
+        <v>3</v>
+      </c>
+      <c r="H624" t="b">
+        <v>0</v>
+      </c>
+      <c r="I624" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J624" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1122581093</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J623"/>
+  <autoFilter ref="A1:J624"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 59, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$624</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$628</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J624"/>
+  <dimension ref="A1:J628"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -25904,8 +25904,172 @@
         </is>
       </c>
     </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>1097778656</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>aihada</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>[大容量]パフュームシャンプー+リンスセット(Sweet&amp;amp;Flowery)(Fresh&amp;amp;Lush)香り高い毛髪ツヤケア</t>
+        </is>
+      </c>
+      <c r="E625" t="inlineStr">
+        <is>
+          <t>ケラシス</t>
+        </is>
+      </c>
+      <c r="F625" t="n">
+        <v>3050</v>
+      </c>
+      <c r="G625" t="n">
+        <v>9</v>
+      </c>
+      <c r="H625" t="b">
+        <v>0</v>
+      </c>
+      <c r="I625" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J625" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1097778656</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>1197441390</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>17hours</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>(3種セット) スピーディ バブルマスク 3種セット 95ml (グルタチオン/PDRN/コラーゲン)</t>
+        </is>
+      </c>
+      <c r="E626" t="inlineStr">
+        <is>
+          <t>17hours</t>
+        </is>
+      </c>
+      <c r="F626" t="n">
+        <v>5840</v>
+      </c>
+      <c r="G626" t="n">
+        <v>0</v>
+      </c>
+      <c r="H626" t="b">
+        <v>0</v>
+      </c>
+      <c r="I626" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J626" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197441390</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>1138183957</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>17hours</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>スキンブースティング ヒアロン アンプル 30ml</t>
+        </is>
+      </c>
+      <c r="E627" t="inlineStr">
+        <is>
+          <t>17hours</t>
+        </is>
+      </c>
+      <c r="F627" t="n">
+        <v>1820</v>
+      </c>
+      <c r="G627" t="n">
+        <v>1</v>
+      </c>
+      <c r="H627" t="b">
+        <v>0</v>
+      </c>
+      <c r="I627" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J627" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1138183957</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>1137892528</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>17hours</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>メルティングエアバブルクレンザー 150ml</t>
+        </is>
+      </c>
+      <c r="E628" t="inlineStr">
+        <is>
+          <t>17hours</t>
+        </is>
+      </c>
+      <c r="F628" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G628" t="n">
+        <v>3</v>
+      </c>
+      <c r="H628" t="b">
+        <v>0</v>
+      </c>
+      <c r="I628" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J628" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1137892528</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J624"/>
+  <autoFilter ref="A1:J628"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 65, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$629</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$632</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J629"/>
+  <dimension ref="A1:J632"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26109,8 +26109,131 @@
         </is>
       </c>
     </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>1202794270</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>JLVENTURES</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>トラネキサム酸1%シートマスク, 30枚</t>
+        </is>
+      </c>
+      <c r="E630" t="inlineStr">
+        <is>
+          <t>Derma Factory</t>
+        </is>
+      </c>
+      <c r="F630" t="n">
+        <v>4980</v>
+      </c>
+      <c r="G630" t="n">
+        <v>5</v>
+      </c>
+      <c r="H630" t="b">
+        <v>0</v>
+      </c>
+      <c r="I630" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J630" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202794270</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>1206222392</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>JLVENTURES</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>【公式販売店】フレッシュウォーターUVクリーム 50g</t>
+        </is>
+      </c>
+      <c r="E631" t="inlineStr">
+        <is>
+          <t>Derma Factory</t>
+        </is>
+      </c>
+      <c r="F631" t="n">
+        <v>1200</v>
+      </c>
+      <c r="G631" t="n">
+        <v>0</v>
+      </c>
+      <c r="H631" t="b">
+        <v>0</v>
+      </c>
+      <c r="I631" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J631" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206222392</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>1199698795</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>JLVENTURES</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>【公式販売店】ペプチドフェイシャル &amp;amp; アイクリーム 20ml</t>
+        </is>
+      </c>
+      <c r="E632" t="inlineStr">
+        <is>
+          <t>Derma Factory</t>
+        </is>
+      </c>
+      <c r="F632" t="n">
+        <v>1350</v>
+      </c>
+      <c r="G632" t="n">
+        <v>1</v>
+      </c>
+      <c r="H632" t="b">
+        <v>0</v>
+      </c>
+      <c r="I632" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J632" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199698795</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J629"/>
+  <autoFilter ref="A1:J632"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 68, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$633</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$635</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J633"/>
+  <dimension ref="A1:J635"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26273,8 +26273,90 @@
         </is>
       </c>
     </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>1158769414</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>waterconnect</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>正規代理店 炭酸泡 トリートメント エイジングケア成分を炭酸泡で浸透 美髪 頭皮ケア 潤い 艶 ヘアケア 洗い流さない レヴィ モイストバブル トリートメント</t>
+        </is>
+      </c>
+      <c r="E634" t="inlineStr">
+        <is>
+          <t>LOUVREDO</t>
+        </is>
+      </c>
+      <c r="F634" t="n">
+        <v>4180</v>
+      </c>
+      <c r="G634" t="n">
+        <v>1</v>
+      </c>
+      <c r="H634" t="b">
+        <v>0</v>
+      </c>
+      <c r="I634" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J634" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1158769414</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>1171629860</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>waterconnect</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>【正規販売店】 レヴィミストローション ミスト スプレー 化粧水 120g 日本製 エイジングケア＆保湿 NMN ツバメの巣エキス ENM 配合 高濃度炭酸ミストが角質層まで届ける</t>
+        </is>
+      </c>
+      <c r="E635" t="inlineStr">
+        <is>
+          <t>LOUVREDO</t>
+        </is>
+      </c>
+      <c r="F635" t="n">
+        <v>2860</v>
+      </c>
+      <c r="G635" t="n">
+        <v>1</v>
+      </c>
+      <c r="H635" t="b">
+        <v>0</v>
+      </c>
+      <c r="I635" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J635" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171629860</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J633"/>
+  <autoFilter ref="A1:J635"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 73, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$635</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$636</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J635"/>
+  <dimension ref="A1:J636"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26355,8 +26355,49 @@
         </is>
       </c>
     </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>1156890626</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>onedamstore</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>【予約販売・LDK1位受賞】ヒートケア ヘアミルク ヘアオイル 各100ml シトラスの香り 熱でダメージ補修 洗い流さないトリートメント ベーススタイリング レディース メンズ</t>
+        </is>
+      </c>
+      <c r="E636" t="inlineStr">
+        <is>
+          <t>Onedam</t>
+        </is>
+      </c>
+      <c r="F636" t="n">
+        <v>2970</v>
+      </c>
+      <c r="G636" t="n">
+        <v>1</v>
+      </c>
+      <c r="H636" t="b">
+        <v>0</v>
+      </c>
+      <c r="I636" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J636" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1156890626</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J635"/>
+  <autoFilter ref="A1:J636"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 74, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$636</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$638</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J636"/>
+  <dimension ref="A1:J638"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26396,8 +26396,90 @@
         </is>
       </c>
     </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>1145897065</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>marketrhea</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>PDRN ピンクペプチドアンプル 50ml</t>
+        </is>
+      </c>
+      <c r="E637" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F637" t="n">
+        <v>1285</v>
+      </c>
+      <c r="G637" t="n">
+        <v>8</v>
+      </c>
+      <c r="H637" t="b">
+        <v>0</v>
+      </c>
+      <c r="I637" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J637" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1145897065</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>1213658245</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>marketrhea</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>バウンシー＆ファーム スリーピングマスク 60mL</t>
+        </is>
+      </c>
+      <c r="E638" t="inlineStr">
+        <is>
+          <t>ラネージュ</t>
+        </is>
+      </c>
+      <c r="F638" t="n">
+        <v>2480</v>
+      </c>
+      <c r="G638" t="n">
+        <v>0</v>
+      </c>
+      <c r="H638" t="b">
+        <v>0</v>
+      </c>
+      <c r="I638" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J638" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213658245</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J636"/>
+  <autoFilter ref="A1:J638"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 76, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$638</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$641</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J638"/>
+  <dimension ref="A1:J641"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26478,8 +26478,131 @@
         </is>
       </c>
     </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>1097518333</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>EPONA</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>【クリーム 1 + 1】 プレミアムクリーム4種 / インテンシブ馬油 / 紅参ゴールド / サーモン油 / スネイル トーンアップ クリーム</t>
+        </is>
+      </c>
+      <c r="E639" t="inlineStr">
+        <is>
+          <t>エポナ</t>
+        </is>
+      </c>
+      <c r="F639" t="n">
+        <v>9990</v>
+      </c>
+      <c r="G639" t="n">
+        <v>1</v>
+      </c>
+      <c r="H639" t="b">
+        <v>0</v>
+      </c>
+      <c r="I639" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J639" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1097518333</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>1110543246</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>EPONA</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>【公式】リブート エッセンシャルアンプル マスクシート 2種 (レチノール+スネイル/コラーゲン+ビタミン) 10枚</t>
+        </is>
+      </c>
+      <c r="E640" t="inlineStr">
+        <is>
+          <t>エポナ</t>
+        </is>
+      </c>
+      <c r="F640" t="n">
+        <v>1990</v>
+      </c>
+      <c r="G640" t="n">
+        <v>0</v>
+      </c>
+      <c r="H640" t="b">
+        <v>0</v>
+      </c>
+      <c r="I640" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J640" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1110543246</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>1183925811</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>mizon_village11</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>7 ヴィーガンペプチドブースターセラム ナイアシンアミドとヒアルロン酸配合の韓国製保湿美容液 150ml</t>
+        </is>
+      </c>
+      <c r="E641" t="inlineStr">
+        <is>
+          <t>ミズオン</t>
+        </is>
+      </c>
+      <c r="F641" t="n">
+        <v>4180</v>
+      </c>
+      <c r="G641" t="n">
+        <v>8</v>
+      </c>
+      <c r="H641" t="b">
+        <v>0</v>
+      </c>
+      <c r="I641" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J641" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183925811</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J638"/>
+  <autoFilter ref="A1:J641"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 77, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$641</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$646</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J641"/>
+  <dimension ref="A1:J646"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26601,8 +26601,213 @@
         </is>
       </c>
     </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>1015316207</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>beacos</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>アリミノ BSスタイリング フリーズキープスプレー 189g/280ml</t>
+        </is>
+      </c>
+      <c r="E642" t="inlineStr">
+        <is>
+          <t>アリミノ</t>
+        </is>
+      </c>
+      <c r="F642" t="n">
+        <v>1329</v>
+      </c>
+      <c r="G642" t="n">
+        <v>1</v>
+      </c>
+      <c r="H642" t="b">
+        <v>0</v>
+      </c>
+      <c r="I642" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J642" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1015316207</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>1183102894</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>beacos</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>ファイバープレックス ボンドシャンプー 250ml &amp;amp; トリートメント250g セット</t>
+        </is>
+      </c>
+      <c r="E643" t="inlineStr">
+        <is>
+          <t>シュワルツコフ</t>
+        </is>
+      </c>
+      <c r="F643" t="n">
+        <v>3920</v>
+      </c>
+      <c r="G643" t="n">
+        <v>3</v>
+      </c>
+      <c r="H643" t="b">
+        <v>0</v>
+      </c>
+      <c r="I643" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J643" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183102894</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>1183102300</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>beacos</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>ファイバープレックス ボンドミルク 100g　×3本セット</t>
+        </is>
+      </c>
+      <c r="E644" t="inlineStr">
+        <is>
+          <t>シュワルツコフ</t>
+        </is>
+      </c>
+      <c r="F644" t="n">
+        <v>4970</v>
+      </c>
+      <c r="G644" t="n">
+        <v>1</v>
+      </c>
+      <c r="H644" t="b">
+        <v>0</v>
+      </c>
+      <c r="I644" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J644" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183102300</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>1167443232</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>beacos</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>シェルパ コアプロテクトミルク 1000g</t>
+        </is>
+      </c>
+      <c r="E645" t="inlineStr">
+        <is>
+          <t>アリミノ</t>
+        </is>
+      </c>
+      <c r="F645" t="n">
+        <v>5426</v>
+      </c>
+      <c r="G645" t="n">
+        <v>5</v>
+      </c>
+      <c r="H645" t="b">
+        <v>0</v>
+      </c>
+      <c r="I645" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J645" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1167443232</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>1167442148</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>beacos</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>シェルパ コアプロテクトミルク 120g</t>
+        </is>
+      </c>
+      <c r="E646" t="inlineStr">
+        <is>
+          <t>アリミノ</t>
+        </is>
+      </c>
+      <c r="F646" t="n">
+        <v>2160</v>
+      </c>
+      <c r="G646" t="n">
+        <v>1</v>
+      </c>
+      <c r="H646" t="b">
+        <v>0</v>
+      </c>
+      <c r="I646" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J646" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1167442148</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J641"/>
+  <autoFilter ref="A1:J646"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 85, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$646</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$650</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J646"/>
+  <dimension ref="A1:J650"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26806,8 +26806,172 @@
         </is>
       </c>
     </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>1210140326</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>suiping</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>お得セット グローパック FUTURE 7回分＋ユーグレナ女神90粒　正規品　新パッケージ商品</t>
+        </is>
+      </c>
+      <c r="E647" t="inlineStr">
+        <is>
+          <t>エニシー</t>
+        </is>
+      </c>
+      <c r="F647" t="n">
+        <v>16500</v>
+      </c>
+      <c r="G647" t="n">
+        <v>0</v>
+      </c>
+      <c r="H647" t="b">
+        <v>0</v>
+      </c>
+      <c r="I647" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J647" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210140326</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>1210874656</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>suiping</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>ゾンビパック 90g （専用ハケ専用スプーン付） 正規品　ハリ・ツヤ肌へ導く話題のパック剤 ZOMBIE フェイスパック リフトアップ リフトパック 顔 引き締め</t>
+        </is>
+      </c>
+      <c r="E648" t="inlineStr">
+        <is>
+          <t>ルリビオ</t>
+        </is>
+      </c>
+      <c r="F648" t="n">
+        <v>6930</v>
+      </c>
+      <c r="G648" t="n">
+        <v>0</v>
+      </c>
+      <c r="H648" t="b">
+        <v>0</v>
+      </c>
+      <c r="I648" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J648" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210874656</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>1208250494</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>suiping</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>シェリースキン STCC ストロングサン 50g　LCクリーム コンビネーションクリーム　クリスタルライティングCC 美容液タイプ化粧下地　ヒトNK細胞 培養液 ヒト幹細胞 女優ライト</t>
+        </is>
+      </c>
+      <c r="E649" t="inlineStr">
+        <is>
+          <t>Re LABEAUTE</t>
+        </is>
+      </c>
+      <c r="F649" t="n">
+        <v>7320</v>
+      </c>
+      <c r="G649" t="n">
+        <v>0</v>
+      </c>
+      <c r="H649" t="b">
+        <v>0</v>
+      </c>
+      <c r="I649" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J649" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208250494</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>1180303482</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>MART-IN</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>旭研究所 ハイドロキノン 皮膚科 業務用 10g</t>
+        </is>
+      </c>
+      <c r="E650" t="inlineStr">
+        <is>
+          <t>旭研究所</t>
+        </is>
+      </c>
+      <c r="F650" t="n">
+        <v>1436</v>
+      </c>
+      <c r="G650" t="n">
+        <v>7</v>
+      </c>
+      <c r="H650" t="b">
+        <v>0</v>
+      </c>
+      <c r="I650" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J650" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180303482</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J646"/>
+  <autoFilter ref="A1:J650"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 86, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$650</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$651</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J650"/>
+  <dimension ref="A1:J651"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -26970,8 +26970,49 @@
         </is>
       </c>
     </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>1021098578</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>capecodcosme</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>V3プロテクションサンスクリーン 50日分 Cサンクリーム 2024年4月リニューアル</t>
+        </is>
+      </c>
+      <c r="E651" t="inlineStr">
+        <is>
+          <t>SPICARE</t>
+        </is>
+      </c>
+      <c r="F651" t="n">
+        <v>4400</v>
+      </c>
+      <c r="G651" t="n">
+        <v>1</v>
+      </c>
+      <c r="H651" t="b">
+        <v>0</v>
+      </c>
+      <c r="I651" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J651" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1021098578</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J650"/>
+  <autoFilter ref="A1:J651"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 94, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$656</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$658</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J656"/>
+  <dimension ref="A1:J658"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27216,8 +27216,90 @@
         </is>
       </c>
     </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>1159561347</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>beautifulmountain</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>NU SKIN エンハンサー</t>
+        </is>
+      </c>
+      <c r="E657" t="inlineStr">
+        <is>
+          <t>ニュースキン</t>
+        </is>
+      </c>
+      <c r="F657" t="n">
+        <v>2508</v>
+      </c>
+      <c r="G657" t="n">
+        <v>1</v>
+      </c>
+      <c r="H657" t="b">
+        <v>0</v>
+      </c>
+      <c r="I657" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J657" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1159561347</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>1007477093</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>richfield</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>ルベル ナチュラル ヘアソープウィズ シーウィードSW(10ml)ナチュラルヘアトリートメントウィズ ライスプロテインRP(10g) 各6袋 セット</t>
+        </is>
+      </c>
+      <c r="E658" t="inlineStr">
+        <is>
+          <t>Lebel</t>
+        </is>
+      </c>
+      <c r="F658" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G658" t="n">
+        <v>0</v>
+      </c>
+      <c r="H658" t="b">
+        <v>0</v>
+      </c>
+      <c r="I658" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J658" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1007477093</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J656"/>
+  <autoFilter ref="A1:J658"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 95, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$658</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$661</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J658"/>
+  <dimension ref="A1:J661"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27298,8 +27298,131 @@
         </is>
       </c>
     </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>1196054203</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>AIRI_SHOP</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>[韓国純正]期間限定コラーゲンベールクリーム50ml+コラーゲンベールアンプル50ml+プレゼント贈呈/弾力強化/イデベノン成分粉化装品/保湿弾力美容液/韓国コスメ/サロン化粧品/顔色光彩</t>
+        </is>
+      </c>
+      <c r="E659" t="inlineStr">
+        <is>
+          <t>MEDIPAIR</t>
+        </is>
+      </c>
+      <c r="F659" t="n">
+        <v>6420</v>
+      </c>
+      <c r="G659" t="n">
+        <v>0</v>
+      </c>
+      <c r="H659" t="b">
+        <v>0</v>
+      </c>
+      <c r="I659" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J659" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196054203</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>1162809369</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>AIRI_SHOP</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>【韓国正規品発送】ハイドロ バルサム パーソナルキット(ブースター 5ml x 2 + アンプル 5ml x 2 + クリーム 20ml)+ マスクパック追加贈呈,エステティック専用製品</t>
+        </is>
+      </c>
+      <c r="E660" t="inlineStr">
+        <is>
+          <t>シバサン</t>
+        </is>
+      </c>
+      <c r="F660" t="n">
+        <v>11200</v>
+      </c>
+      <c r="G660" t="n">
+        <v>1</v>
+      </c>
+      <c r="H660" t="b">
+        <v>0</v>
+      </c>
+      <c r="I660" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J660" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1162809369</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>1172888043</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>AIRI_SHOP</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>[韓国純正]ピルマスク10種30枚+プレゼント贈呈/1日1マスクパック/肌悩み別マスクパック</t>
+        </is>
+      </c>
+      <c r="E661" t="inlineStr">
+        <is>
+          <t>GRACE DAY</t>
+        </is>
+      </c>
+      <c r="F661" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G661" t="n">
+        <v>5</v>
+      </c>
+      <c r="H661" t="b">
+        <v>0</v>
+      </c>
+      <c r="I661" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J661" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172888043</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J658"/>
+  <autoFilter ref="A1:J661"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 98, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$661</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$664</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J661"/>
+  <dimension ref="A1:J664"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27421,8 +27421,131 @@
         </is>
       </c>
     </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>1194005545</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>corindo</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>エリクシール シュペリエル リフトモイストローション しっとりタイプｂａ つめかえ用 SHISEIDO 22721</t>
+        </is>
+      </c>
+      <c r="E662" t="inlineStr">
+        <is>
+          <t>資生堂</t>
+        </is>
+      </c>
+      <c r="F662" t="n">
+        <v>2970</v>
+      </c>
+      <c r="G662" t="n">
+        <v>0</v>
+      </c>
+      <c r="H662" t="b">
+        <v>0</v>
+      </c>
+      <c r="I662" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J662" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194005545</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>1144044630</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>corindo</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>エステ洗顔ジェル 130g SHISEIDO 21263</t>
+        </is>
+      </c>
+      <c r="E663" t="inlineStr">
+        <is>
+          <t>アクアレーベル</t>
+        </is>
+      </c>
+      <c r="F663" t="n">
+        <v>1358</v>
+      </c>
+      <c r="G663" t="n">
+        <v>5</v>
+      </c>
+      <c r="H663" t="b">
+        <v>0</v>
+      </c>
+      <c r="I663" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J663" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1144044630</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>1134992045</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>corindo</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>グラナス クレンジングミルク</t>
+        </is>
+      </c>
+      <c r="E664" t="inlineStr">
+        <is>
+          <t>リバイタル</t>
+        </is>
+      </c>
+      <c r="F664" t="n">
+        <v>4180</v>
+      </c>
+      <c r="G664" t="n">
+        <v>0</v>
+      </c>
+      <c r="H664" t="b">
+        <v>0</v>
+      </c>
+      <c r="I664" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J664" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1134992045</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J661"/>
+  <autoFilter ref="A1:J664"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 100, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$668</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$671</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J668"/>
+  <dimension ref="A1:J671"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27708,8 +27708,131 @@
         </is>
       </c>
     </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>1182175285</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>toakaiyou</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>【国内正規品】スキンパワー リニューエアリー クリーム 80g</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr">
+        <is>
+          <t>SK-Ⅱ</t>
+        </is>
+      </c>
+      <c r="F669" t="n">
+        <v>24057</v>
+      </c>
+      <c r="G669" t="n">
+        <v>3</v>
+      </c>
+      <c r="H669" t="b">
+        <v>0</v>
+      </c>
+      <c r="I669" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J669" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1182175285</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>1156566791</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>toakaiyou</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>アトリエメイド アンリミテッド メイクアップ フィックス ミスト 100mlメイクアップアーティスト ベースメイク ベース メイク ベース メイク</t>
+        </is>
+      </c>
+      <c r="E670" t="inlineStr">
+        <is>
+          <t>シュウウエムラ</t>
+        </is>
+      </c>
+      <c r="F670" t="n">
+        <v>4180</v>
+      </c>
+      <c r="G670" t="n">
+        <v>3</v>
+      </c>
+      <c r="H670" t="b">
+        <v>0</v>
+      </c>
+      <c r="I670" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J670" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1156566791</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>1213657170</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>cottonleaf</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>LIPOPEEL リポピールセラム 30ml 導入美容液 ピーリング 角質ケア 毛穴ケア ごわつき 敏感肌 グルタチオン ナイアシンアミド スキンケア サリチル酸</t>
+        </is>
+      </c>
+      <c r="E671" t="inlineStr">
+        <is>
+          <t>LIPOPEEL</t>
+        </is>
+      </c>
+      <c r="F671" t="n">
+        <v>3200</v>
+      </c>
+      <c r="G671" t="n">
+        <v>0</v>
+      </c>
+      <c r="H671" t="b">
+        <v>0</v>
+      </c>
+      <c r="I671" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J671" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213657170</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J668"/>
+  <autoFilter ref="A1:J671"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 104, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$671</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$679</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J671"/>
+  <dimension ref="A1:J679"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27831,8 +27831,336 @@
         </is>
       </c>
     </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>1210748902</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>japangateway</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>kéralis noir ケラリス ノワール ヒートシールヘアミスト スムース＆モイスト</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr">
+        <is>
+          <t>ISSHI</t>
+        </is>
+      </c>
+      <c r="F672" t="n">
+        <v>2310</v>
+      </c>
+      <c r="G672" t="n">
+        <v>0</v>
+      </c>
+      <c r="H672" t="b">
+        <v>0</v>
+      </c>
+      <c r="I672" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J672" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210748902</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>1194972100</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>japangateway</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>kéralis noir ケラリス ノワール ヘアパックセラム スムージングリペアモイスト</t>
+        </is>
+      </c>
+      <c r="E673" t="inlineStr">
+        <is>
+          <t>ISSHI</t>
+        </is>
+      </c>
+      <c r="F673" t="n">
+        <v>2585</v>
+      </c>
+      <c r="G673" t="n">
+        <v>0</v>
+      </c>
+      <c r="H673" t="b">
+        <v>0</v>
+      </c>
+      <c r="I673" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J673" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194972100</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>1191782200</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>japangateway</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>keralis noir ケラリス ノワール シャンプー＆ヘアトリートメン トSET スムージングリペアモイスト</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr">
+        <is>
+          <t>ISSHI</t>
+        </is>
+      </c>
+      <c r="F674" t="n">
+        <v>5940</v>
+      </c>
+      <c r="G674" t="n">
+        <v>5</v>
+      </c>
+      <c r="H674" t="b">
+        <v>0</v>
+      </c>
+      <c r="I674" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J674" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191782200</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>1176040839</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>japangateway</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>薬用デオドラントロールオン スイートホワイトブーケ</t>
+        </is>
+      </c>
+      <c r="E675" t="inlineStr">
+        <is>
+          <t>メルサボン</t>
+        </is>
+      </c>
+      <c r="F675" t="n">
+        <v>990</v>
+      </c>
+      <c r="G675" t="n">
+        <v>0</v>
+      </c>
+      <c r="H675" t="b">
+        <v>0</v>
+      </c>
+      <c r="I675" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J675" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1176040839</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>1175152720</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>japangateway</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>ザ ヘアミルク Dx ディープリペアモイスト パウチタイプ</t>
+        </is>
+      </c>
+      <c r="E676" t="inlineStr">
+        <is>
+          <t>ISSHI</t>
+        </is>
+      </c>
+      <c r="F676" t="n">
+        <v>2090</v>
+      </c>
+      <c r="G676" t="n">
+        <v>0</v>
+      </c>
+      <c r="H676" t="b">
+        <v>0</v>
+      </c>
+      <c r="I676" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J676" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1175152720</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>1172391078</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>aquanoa</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>【 公式 】スリーク by サラサロン メルティリペア シャンプー 詰替 メルティリペア トリートメント 詰替</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr">
+        <is>
+          <t>Sleek by Sarasalon</t>
+        </is>
+      </c>
+      <c r="F677" t="n">
+        <v>1650</v>
+      </c>
+      <c r="G677" t="n">
+        <v>5</v>
+      </c>
+      <c r="H677" t="b">
+        <v>0</v>
+      </c>
+      <c r="I677" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J677" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172391078</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>1172391077</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>aquanoa</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>【 公式 】スリーク by サラサロン ナイトケアセラム シャンプー ナイトケアセラム トリートメント セット</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr">
+        <is>
+          <t>Sleek by Sarasalon</t>
+        </is>
+      </c>
+      <c r="F678" t="n">
+        <v>3520</v>
+      </c>
+      <c r="G678" t="n">
+        <v>7</v>
+      </c>
+      <c r="H678" t="b">
+        <v>0</v>
+      </c>
+      <c r="I678" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J678" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172391077</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>1174516764</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>aquanoa</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>【 公式 】スリーク by サラサロン ナイトケアセラム シャンプー ナイトケアセラム トリートメント 3Way オイルミストセット</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr">
+        <is>
+          <t>Sleek by Sarasalon</t>
+        </is>
+      </c>
+      <c r="F679" t="n">
+        <v>5170</v>
+      </c>
+      <c r="G679" t="n">
+        <v>4</v>
+      </c>
+      <c r="H679" t="b">
+        <v>0</v>
+      </c>
+      <c r="I679" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J679" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174516764</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J671"/>
+  <autoFilter ref="A1:J679"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 110, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$679</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$680</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J679"/>
+  <dimension ref="A1:J680"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28159,8 +28159,49 @@
         </is>
       </c>
     </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>1194578982</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>houseofhur</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>【NEW】 【公式】 フィトブリュー抹茶アンプル 50ml / 美容液 / セラム / 保湿 / うるおい / 鎮静 / バリアケア / くすみケア /</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr">
+        <is>
+          <t>HOUSE OF Hur</t>
+        </is>
+      </c>
+      <c r="F680" t="n">
+        <v>1820</v>
+      </c>
+      <c r="G680" t="n">
+        <v>1</v>
+      </c>
+      <c r="H680" t="b">
+        <v>0</v>
+      </c>
+      <c r="I680" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J680" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194578982</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J679"/>
+  <autoFilter ref="A1:J680"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 112, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$681</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$683</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J681"/>
+  <dimension ref="A1:J683"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28241,8 +28241,90 @@
         </is>
       </c>
     </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>1161939902</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>quvee</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>シゾピリンセルラー メスクリーム 35ml メスクリーム鎮生 + シートマスクをプレゼント</t>
+        </is>
+      </c>
+      <c r="E682" t="inlineStr">
+        <is>
+          <t>シバサン</t>
+        </is>
+      </c>
+      <c r="F682" t="n">
+        <v>10700</v>
+      </c>
+      <c r="G682" t="n">
+        <v>2</v>
+      </c>
+      <c r="H682" t="b">
+        <v>0</v>
+      </c>
+      <c r="I682" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J682" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1161939902</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>1137321213</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>Ureun</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>【公式】ヴィーガン ツバキオイル セラム ミスト 100ml / ミスト化粧水 保湿</t>
+        </is>
+      </c>
+      <c r="E683" t="inlineStr">
+        <is>
+          <t>Ureun</t>
+        </is>
+      </c>
+      <c r="F683" t="n">
+        <v>2800</v>
+      </c>
+      <c r="G683" t="n">
+        <v>0</v>
+      </c>
+      <c r="H683" t="b">
+        <v>0</v>
+      </c>
+      <c r="I683" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J683" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1137321213</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J681"/>
+  <autoFilter ref="A1:J683"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 113, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$683</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$684</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J683"/>
+  <dimension ref="A1:J684"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28323,8 +28323,49 @@
         </is>
       </c>
     </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>1191318451</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>frommedi</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>ナノステップ コラーゲン メルティングマスク（16枚）/ ナイトパック / 韓国スキンケア</t>
+        </is>
+      </c>
+      <c r="E684" t="inlineStr">
+        <is>
+          <t>フロムメディ</t>
+        </is>
+      </c>
+      <c r="F684" t="n">
+        <v>11400</v>
+      </c>
+      <c r="G684" t="n">
+        <v>7</v>
+      </c>
+      <c r="H684" t="b">
+        <v>0</v>
+      </c>
+      <c r="I684" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J684" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191318451</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J683"/>
+  <autoFilter ref="A1:J684"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 115, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$684</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$688</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J684"/>
+  <dimension ref="A1:J688"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28364,8 +28364,172 @@
         </is>
       </c>
     </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>1199582203</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>Kiero</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>【角質・毛穴ケアを一度に】バランストナーパッド 60枚入り　AHA うるおいエッセンス 拭き取り化粧水 洗顔後の仕上げに デイリートナーパッド ツヤ肌 トーンアップ</t>
+        </is>
+      </c>
+      <c r="E685" t="inlineStr">
+        <is>
+          <t>Kiero</t>
+        </is>
+      </c>
+      <c r="F685" t="n">
+        <v>1800</v>
+      </c>
+      <c r="G685" t="n">
+        <v>7</v>
+      </c>
+      <c r="H685" t="b">
+        <v>0</v>
+      </c>
+      <c r="I685" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J685" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199582203</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>1199580421</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>Kiero</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>【酵素洗顔】リファイニング エンザイムクレンザー50g　酵素クレンジング 低刺激 角質ケア 保湿 なめらか泡 敏感肌 鎮静 パパイヤ酵素</t>
+        </is>
+      </c>
+      <c r="E686" t="inlineStr">
+        <is>
+          <t>Kiero</t>
+        </is>
+      </c>
+      <c r="F686" t="n">
+        <v>1700</v>
+      </c>
+      <c r="G686" t="n">
+        <v>1</v>
+      </c>
+      <c r="H686" t="b">
+        <v>0</v>
+      </c>
+      <c r="I686" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J686" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199580421</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>1199580084</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>Kiero</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>【さっぱりなのに高保湿】モイスチャライジング バリアクリーム50g メイク前でも負担なく使える べたつかない 肌バリア インナードライ 水分ロック 油分バランス</t>
+        </is>
+      </c>
+      <c r="E687" t="inlineStr">
+        <is>
+          <t>Kiero</t>
+        </is>
+      </c>
+      <c r="F687" t="n">
+        <v>1600</v>
+      </c>
+      <c r="G687" t="n">
+        <v>1</v>
+      </c>
+      <c r="H687" t="b">
+        <v>0</v>
+      </c>
+      <c r="I687" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J687" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199580084</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>1199579508</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>Kiero</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>【2個セットならさらにお得！】プライマーサンジェル50ml メイク密着 日焼け止め 毛穴カバー 化粧下地 白浮きなし ベースメイク 毛穴隠し 鎮静 UV 敏感肌</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr">
+        <is>
+          <t>Kiero</t>
+        </is>
+      </c>
+      <c r="F688" t="n">
+        <v>1700</v>
+      </c>
+      <c r="G688" t="n">
+        <v>0</v>
+      </c>
+      <c r="H688" t="b">
+        <v>0</v>
+      </c>
+      <c r="I688" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J688" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199579508</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J684"/>
+  <autoFilter ref="A1:J688"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 116, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$688</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$690</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J688"/>
+  <dimension ref="A1:J690"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28528,8 +28528,90 @@
         </is>
       </c>
     </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>1200988290</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>NAAP</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>グルタチオンダークスポットアンプル 30ml</t>
+        </is>
+      </c>
+      <c r="E689" t="inlineStr">
+        <is>
+          <t>NAAP</t>
+        </is>
+      </c>
+      <c r="F689" t="n">
+        <v>1650</v>
+      </c>
+      <c r="G689" t="n">
+        <v>0</v>
+      </c>
+      <c r="H689" t="b">
+        <v>0</v>
+      </c>
+      <c r="I689" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J689" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200988290</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>1174229881</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>cell29</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>【韓国コスメ】【公式正品】CELLASINCE PDRN アンプル 32ml / シワ改善 アンプル 美容液 ハリ 弾力 アンチエイジング</t>
+        </is>
+      </c>
+      <c r="E690" t="inlineStr">
+        <is>
+          <t>CELL29</t>
+        </is>
+      </c>
+      <c r="F690" t="n">
+        <v>7100</v>
+      </c>
+      <c r="G690" t="n">
+        <v>3</v>
+      </c>
+      <c r="H690" t="b">
+        <v>0</v>
+      </c>
+      <c r="I690" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J690" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174229881</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J688"/>
+  <autoFilter ref="A1:J690"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 117, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$690</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$691</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J690"/>
+  <dimension ref="A1:J691"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28610,8 +28610,49 @@
         </is>
       </c>
     </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>1163508511</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>KLALAB</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>リカバリー シカミスト 100ml フェイスアンド ボディミスト 即時水分補給 敏感肌用 赤みケア 大人ニキビ対策 エイジングケア イオンミネラル 低刺激処方</t>
+        </is>
+      </c>
+      <c r="E691" t="inlineStr">
+        <is>
+          <t>KLALAB</t>
+        </is>
+      </c>
+      <c r="F691" t="n">
+        <v>2600</v>
+      </c>
+      <c r="G691" t="n">
+        <v>7</v>
+      </c>
+      <c r="H691" t="b">
+        <v>0</v>
+      </c>
+      <c r="I691" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J691" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1163508511</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J690"/>
+  <autoFilter ref="A1:J691"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 120, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$691</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$694</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J691"/>
+  <dimension ref="A1:J694"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28651,8 +28651,131 @@
         </is>
       </c>
     </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>1151131775</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>taviecompany</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>【ゼオスキンヘルス】コンプレクションリニューアルパッド 30枚</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr">
+        <is>
+          <t>ZO SKIN</t>
+        </is>
+      </c>
+      <c r="F692" t="n">
+        <v>1880</v>
+      </c>
+      <c r="G692" t="n">
+        <v>0</v>
+      </c>
+      <c r="H692" t="b">
+        <v>0</v>
+      </c>
+      <c r="I692" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J692" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1151131775</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>1155683046</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>taviecompany</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>(ドゥゴナEGFクリーム+エルボリアンCC進呈）【ゼオスキンヘルス】バランサートナー 180ml 化粧水</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr">
+        <is>
+          <t>ZO SKIN</t>
+        </is>
+      </c>
+      <c r="F693" t="n">
+        <v>6280</v>
+      </c>
+      <c r="G693" t="n">
+        <v>0</v>
+      </c>
+      <c r="H693" t="b">
+        <v>0</v>
+      </c>
+      <c r="I693" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J693" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1155683046</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>1139821001</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>taviecompany</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>【POLA】ポーラ B.A グランラグゼIV マスク 27mL 2枚 + B.A グランラグゼ IV 美容液 0.6g×14包</t>
+        </is>
+      </c>
+      <c r="E694" t="inlineStr">
+        <is>
+          <t>ポーラ</t>
+        </is>
+      </c>
+      <c r="F694" t="n">
+        <v>5980</v>
+      </c>
+      <c r="G694" t="n">
+        <v>2</v>
+      </c>
+      <c r="H694" t="b">
+        <v>0</v>
+      </c>
+      <c r="I694" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J694" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1139821001</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J691"/>
+  <autoFilter ref="A1:J694"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 121, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$694</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$699</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J694"/>
+  <dimension ref="A1:J699"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -28774,8 +28774,213 @@
         </is>
       </c>
     </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>1113430417</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>k-beautic</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>ピュア＆ソフトフェミニンウォッシュ/弱酸性/低刺激/無香料/鎮静・保湿/vioソープかゆみ・匂いケア/クーリング感/170ml [デリケートゾーン ニオイケア ボディソープ ボディーソープ フェムテッ</t>
+        </is>
+      </c>
+      <c r="E695" t="inlineStr">
+        <is>
+          <t>アロマティカ</t>
+        </is>
+      </c>
+      <c r="F695" t="n">
+        <v>1699</v>
+      </c>
+      <c r="G695" t="n">
+        <v>4</v>
+      </c>
+      <c r="H695" t="b">
+        <v>0</v>
+      </c>
+      <c r="I695" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J695" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1113430417</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>1213226123</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>k-beautic</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>[正規販売店] 1+1 アドバンスドPDRNカーミングサンセラム, 50ml PDRNマデカッソシド配合 美容液UVセラム</t>
+        </is>
+      </c>
+      <c r="E696" t="inlineStr">
+        <is>
+          <t>Dr.Reju-All</t>
+        </is>
+      </c>
+      <c r="F696" t="n">
+        <v>6199</v>
+      </c>
+      <c r="G696" t="n">
+        <v>1</v>
+      </c>
+      <c r="H696" t="b">
+        <v>0</v>
+      </c>
+      <c r="I696" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J696" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213226123</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>1213226533</t>
+        </is>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>k-beautic</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>[正規販売店]アドバンスドPDLLA ファーミングクリーム 30ml / PDLLA 12,000ppm / CICAスピキュール / ハリ・うるおいケア/rejuall rijuall</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr">
+        <is>
+          <t>Dr.Reju-All</t>
+        </is>
+      </c>
+      <c r="F697" t="n">
+        <v>4699</v>
+      </c>
+      <c r="G697" t="n">
+        <v>0</v>
+      </c>
+      <c r="H697" t="b">
+        <v>0</v>
+      </c>
+      <c r="I697" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J697" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213226533</t>
+        </is>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>1213226060</t>
+        </is>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>k-beautic</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>[正規販売店] アドバンスドPDRNカーミングサンセラム, 50ml PDRNマデカッソシド配合 美容液UVセラム</t>
+        </is>
+      </c>
+      <c r="E698" t="inlineStr">
+        <is>
+          <t>Dr.Reju-All</t>
+        </is>
+      </c>
+      <c r="F698" t="n">
+        <v>3199</v>
+      </c>
+      <c r="G698" t="n">
+        <v>0</v>
+      </c>
+      <c r="H698" t="b">
+        <v>0</v>
+      </c>
+      <c r="I698" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J698" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213226060</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>1205771223</t>
+        </is>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>k-beautic</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>韓国薬局コスメの本気5点セットREJUALL レチノメラセラム30ml・PDRNクリーム20ml・セラミドバリアクリーム50ml・リップセラム10g・シートマスク 36g×4枚 Rijuall</t>
+        </is>
+      </c>
+      <c r="E699" t="inlineStr">
+        <is>
+          <t>Dr.Reju-All</t>
+        </is>
+      </c>
+      <c r="F699" t="n">
+        <v>12999</v>
+      </c>
+      <c r="G699" t="n">
+        <v>4</v>
+      </c>
+      <c r="H699" t="b">
+        <v>0</v>
+      </c>
+      <c r="I699" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J699" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205771223</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J694"/>
+  <autoFilter ref="A1:J699"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 23, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$714</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$715</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J714"/>
+  <dimension ref="A1:J715"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -29594,8 +29594,49 @@
         </is>
       </c>
     </row>
+    <row r="715">
+      <c r="A715" t="inlineStr">
+        <is>
+          <t>1195296807</t>
+        </is>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>k-mono</t>
+        </is>
+      </c>
+      <c r="C715" t="inlineStr">
+        <is>
+          <t>1025 独島トナー 200ml 500ml 韓国正規品 敏感肌 保湿 化粧水</t>
+        </is>
+      </c>
+      <c r="E715" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F715" t="n">
+        <v>2167</v>
+      </c>
+      <c r="G715" t="n">
+        <v>0</v>
+      </c>
+      <c r="H715" t="b">
+        <v>0</v>
+      </c>
+      <c r="I715" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J715" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1195296807</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J714"/>
+  <autoFilter ref="A1:J715"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 32, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$727</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$728</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J727"/>
+  <dimension ref="A1:J728"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30127,8 +30127,49 @@
         </is>
       </c>
     </row>
+    <row r="728">
+      <c r="A728" t="inlineStr">
+        <is>
+          <t>1167236355</t>
+        </is>
+      </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>global-k</t>
+        </is>
+      </c>
+      <c r="C728" t="inlineStr">
+        <is>
+          <t>メラトーニングクリーム 30g /色素沈着・保湿対策 /トーンアップ /フェイスクリーム</t>
+        </is>
+      </c>
+      <c r="E728" t="inlineStr">
+        <is>
+          <t>東亜製薬</t>
+        </is>
+      </c>
+      <c r="F728" t="n">
+        <v>3900</v>
+      </c>
+      <c r="G728" t="n">
+        <v>0</v>
+      </c>
+      <c r="H728" t="b">
+        <v>0</v>
+      </c>
+      <c r="I728" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J728" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1167236355</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J727"/>
+  <autoFilter ref="A1:J728"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 50, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$732</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$733</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J732"/>
+  <dimension ref="A1:J733"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30332,8 +30332,49 @@
         </is>
       </c>
     </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>1040248028</t>
+        </is>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>toyokoubeauty</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>ファ　ンケル FAN　CL BC 化粧液 30mL（製造日2024年10月）未開封：製造年月日より2年</t>
+        </is>
+      </c>
+      <c r="E733" t="inlineStr">
+        <is>
+          <t>ファンケル</t>
+        </is>
+      </c>
+      <c r="F733" t="n">
+        <v>2300</v>
+      </c>
+      <c r="G733" t="n">
+        <v>0</v>
+      </c>
+      <c r="H733" t="b">
+        <v>0</v>
+      </c>
+      <c r="I733" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J733" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1040248028</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J732"/>
+  <autoFilter ref="A1:J733"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 79, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$736</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$737</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J736"/>
+  <dimension ref="A1:J737"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30496,8 +30496,49 @@
         </is>
       </c>
     </row>
+    <row r="737">
+      <c r="A737" t="inlineStr">
+        <is>
+          <t>1211080915</t>
+        </is>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>tamz</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>シグネチャー ヘアエッセンス プルメリア フレグランス 100ml（ヴィーガン認証・弱酸性)</t>
+        </is>
+      </c>
+      <c r="E737" t="inlineStr">
+        <is>
+          <t>tamz</t>
+        </is>
+      </c>
+      <c r="F737" t="n">
+        <v>3150</v>
+      </c>
+      <c r="G737" t="n">
+        <v>1</v>
+      </c>
+      <c r="H737" t="b">
+        <v>0</v>
+      </c>
+      <c r="I737" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J737" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211080915</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J736"/>
+  <autoFilter ref="A1:J737"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 80, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$737</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$738</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J737"/>
+  <dimension ref="A1:J738"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30537,8 +30537,49 @@
         </is>
       </c>
     </row>
+    <row r="738">
+      <c r="A738" t="inlineStr">
+        <is>
+          <t>1163511279</t>
+        </is>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>vegannature</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr">
+        <is>
+          <t>弱酸性 ビーガン シャンプーバー シトラス 100g ヴィーガンシャンプー ノンシリコン 弱酸性 固形シャンプー 天然由来成分配合 地肌をすこやかに 敏感肌にも使い</t>
+        </is>
+      </c>
+      <c r="E738" t="inlineStr">
+        <is>
+          <t>VEGANNATURE</t>
+        </is>
+      </c>
+      <c r="F738" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G738" t="n">
+        <v>1</v>
+      </c>
+      <c r="H738" t="b">
+        <v>0</v>
+      </c>
+      <c r="I738" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J738" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1163511279</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J737"/>
+  <autoFilter ref="A1:J738"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 16, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$748</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$749</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J748"/>
+  <dimension ref="A1:J749"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -30988,8 +30988,49 @@
         </is>
       </c>
     </row>
+    <row r="749">
+      <c r="A749" t="inlineStr">
+        <is>
+          <t>1202542070</t>
+        </is>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>haeirin</t>
+        </is>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>ダーマファーム スージングリペアクリーム R4 保湿クリーム 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E749" t="inlineStr">
+        <is>
+          <t>DERMAFIRM</t>
+        </is>
+      </c>
+      <c r="F749" t="n">
+        <v>1900</v>
+      </c>
+      <c r="G749" t="n">
+        <v>0</v>
+      </c>
+      <c r="H749" t="b">
+        <v>0</v>
+      </c>
+      <c r="I749" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J749" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202542070</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J748"/>
+  <autoFilter ref="A1:J749"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 11, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$759</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$761</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J759"/>
+  <dimension ref="A1:J761"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -31439,8 +31439,90 @@
         </is>
       </c>
     </row>
+    <row r="760">
+      <c r="A760" t="inlineStr">
+        <is>
+          <t>1207412267</t>
+        </is>
+      </c>
+      <c r="B760" t="inlineStr">
+        <is>
+          <t>ashitarunrun</t>
+        </is>
+      </c>
+      <c r="C760" t="inlineStr">
+        <is>
+          <t>コウジ酸4%美容液　コウジ酸 アルブチン ビタミンC ジェル 美容液</t>
+        </is>
+      </c>
+      <c r="E760" t="inlineStr">
+        <is>
+          <t>あしたるんるん</t>
+        </is>
+      </c>
+      <c r="F760" t="n">
+        <v>2780</v>
+      </c>
+      <c r="G760" t="n">
+        <v>3</v>
+      </c>
+      <c r="H760" t="b">
+        <v>0</v>
+      </c>
+      <c r="I760" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J760" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207412267</t>
+        </is>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" t="inlineStr">
+        <is>
+          <t>1194181730</t>
+        </is>
+      </c>
+      <c r="B761" t="inlineStr">
+        <is>
+          <t>ashitarunrun</t>
+        </is>
+      </c>
+      <c r="C761" t="inlineStr">
+        <is>
+          <t>【公式ショップ】除毛クリーム 医薬部外品 子供 脱毛 ムダ毛 ムダ毛処理 除毛剤 SUBEKO 薬用除毛ミルク (スプレータイプ)</t>
+        </is>
+      </c>
+      <c r="E761" t="inlineStr">
+        <is>
+          <t>withmoon</t>
+        </is>
+      </c>
+      <c r="F761" t="n">
+        <v>2480</v>
+      </c>
+      <c r="G761" t="n">
+        <v>3</v>
+      </c>
+      <c r="H761" t="b">
+        <v>0</v>
+      </c>
+      <c r="I761" t="inlineStr">
+        <is>
+          <t>120000019</t>
+        </is>
+      </c>
+      <c r="J761" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194181730</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J759"/>
+  <autoFilter ref="A1:J761"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 20, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$774</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$775</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J774"/>
+  <dimension ref="A1:J775"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -32054,8 +32054,49 @@
         </is>
       </c>
     </row>
+    <row r="775">
+      <c r="A775" t="inlineStr">
+        <is>
+          <t>989719203</t>
+        </is>
+      </c>
+      <c r="B775" t="inlineStr">
+        <is>
+          <t>mcos</t>
+        </is>
+      </c>
+      <c r="C775" t="inlineStr">
+        <is>
+          <t>いろは VIO TREATMENT LOTION デリケートゾーン用保湿化粧水 保湿 ムダ毛ケア</t>
+        </is>
+      </c>
+      <c r="E775" t="inlineStr">
+        <is>
+          <t>iroha</t>
+        </is>
+      </c>
+      <c r="F775" t="n">
+        <v>1815</v>
+      </c>
+      <c r="G775" t="n">
+        <v>2</v>
+      </c>
+      <c r="H775" t="b">
+        <v>0</v>
+      </c>
+      <c r="I775" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J775" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=989719203</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J774"/>
+  <autoFilter ref="A1:J775"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 61, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$815</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$816</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J815"/>
+  <dimension ref="A1:J816"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -33735,8 +33735,49 @@
         </is>
       </c>
     </row>
+    <row r="816">
+      <c r="A816" t="inlineStr">
+        <is>
+          <t>1000094101</t>
+        </is>
+      </c>
+      <c r="B816" t="inlineStr">
+        <is>
+          <t>Hachi88</t>
+        </is>
+      </c>
+      <c r="C816" t="inlineStr">
+        <is>
+          <t>plus alpha 3 bee さらさらUVスティック 14g 日本製 SPF50+/PA++++ スティックタイプ 日焼け止め 無香料 ノンパラペン</t>
+        </is>
+      </c>
+      <c r="E816" t="inlineStr">
+        <is>
+          <t>plus alpha 3</t>
+        </is>
+      </c>
+      <c r="F816" t="n">
+        <v>1380</v>
+      </c>
+      <c r="G816" t="n">
+        <v>5</v>
+      </c>
+      <c r="H816" t="b">
+        <v>0</v>
+      </c>
+      <c r="I816" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J816" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1000094101</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J815"/>
+  <autoFilter ref="A1:J816"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 10)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$821</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$822</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J821"/>
+  <dimension ref="A1:J822"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -33981,8 +33981,49 @@
         </is>
       </c>
     </row>
+    <row r="822">
+      <c r="A822" t="inlineStr">
+        <is>
+          <t>1199380329</t>
+        </is>
+      </c>
+      <c r="B822" t="inlineStr">
+        <is>
+          <t>hahahalabo</t>
+        </is>
+      </c>
+      <c r="C822" t="inlineStr">
+        <is>
+          <t>【公式販売店】キラトス（KIRATOTH ）酵素炭配合 ホワイトニング歯磨き粉 口臭ケア W美白コート 日本製 (1本)</t>
+        </is>
+      </c>
+      <c r="E822" t="inlineStr">
+        <is>
+          <t>KIRATOTH</t>
+        </is>
+      </c>
+      <c r="F822" t="n">
+        <v>3400</v>
+      </c>
+      <c r="G822" t="n">
+        <v>9</v>
+      </c>
+      <c r="H822" t="b">
+        <v>0</v>
+      </c>
+      <c r="I822" t="inlineStr">
+        <is>
+          <t>120000019</t>
+        </is>
+      </c>
+      <c r="J822" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199380329</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J821"/>
+  <autoFilter ref="A1:J822"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 2 own-file progress (반복 20)
</commit_message>
<xml_diff>
--- a/output/discovery_result_2.xlsx
+++ b/output/discovery_result_2.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$822</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$823</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J822"/>
+  <dimension ref="A1:J823"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -34022,8 +34022,49 @@
         </is>
       </c>
     </row>
+    <row r="823">
+      <c r="A823" t="inlineStr">
+        <is>
+          <t>1212777156</t>
+        </is>
+      </c>
+      <c r="B823" t="inlineStr">
+        <is>
+          <t>SAVAWAYTEST</t>
+        </is>
+      </c>
+      <c r="C823" t="inlineStr">
+        <is>
+          <t>test【頭皮ケアセット】リファハートブラシフォースカルプ（マットオレ） + リファパドルプレミアム</t>
+        </is>
+      </c>
+      <c r="E823" t="inlineStr">
+        <is>
+          <t>リファ</t>
+        </is>
+      </c>
+      <c r="F823" t="n">
+        <v>100</v>
+      </c>
+      <c r="G823" t="n">
+        <v>0</v>
+      </c>
+      <c r="H823" t="b">
+        <v>0</v>
+      </c>
+      <c r="I823" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J823" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212777156</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J822"/>
+  <autoFilter ref="A1:J823"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>